<commit_message>
Chunking quality updates, ready for research again
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Nyaymalaw_Feedback_Log_v3.xlsx
+++ b/Nyaymalaw_Feedback_Log_v3.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W120"/>
+  <dimension ref="A1:W181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7060,6 +7060,4302 @@
       <c r="V120" s="3" t="inlineStr"/>
       <c r="W120" s="3" t="inlineStr"/>
     </row>
+    <row r="121" ht="60" customHeight="1">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 6:39 AM</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-001</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>If you'd like, I can find relevant court judgments on this, or give you a full legal opinion.
+please do</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>Tenant in Telangana with lease agreement; 3 months rent default, threats of phys</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr"/>
+      <c r="F121" s="3" t="inlineStr"/>
+      <c r="G121" s="3" t="inlineStr"/>
+      <c r="H121" s="3" t="inlineStr">
+        <is>
+          <t>I don't have any data for your query. I searched the internal vector store and web sources (official PDFs, legal portals, newspapers) but found no relevant bare act provisions or case laws. Try rephrasing with specific section numbers, Act names, or a different legal angle.</t>
+        </is>
+      </c>
+      <c r="I121" s="3" t="inlineStr"/>
+      <c r="J121" s="3" t="inlineStr"/>
+      <c r="K121" s="3" t="inlineStr"/>
+      <c r="L121" s="3" t="inlineStr"/>
+      <c r="M121" s="3" t="inlineStr"/>
+      <c r="N121" s="3" t="inlineStr"/>
+      <c r="O121" s="3" t="inlineStr"/>
+      <c r="P121" s="3" t="inlineStr"/>
+      <c r="Q121" s="3" t="inlineStr"/>
+      <c r="R121" s="3" t="inlineStr"/>
+      <c r="S121" s="3" t="inlineStr"/>
+      <c r="T121" s="3" t="inlineStr"/>
+      <c r="U121" s="3" t="inlineStr"/>
+      <c r="V121" s="3" t="inlineStr"/>
+      <c r="W121" s="3" t="inlineStr"/>
+    </row>
+    <row r="122" ht="60" customHeight="1">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 10:34 AM</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-002</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>I own agricultural land in Hyderabad acquired 15 years ago. My neighbour claims he has customary rights to draw water from my land for irrigation. What are my rights and obligations under property transfer laws?</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I own agricultural land in Hyderabad acquired 15 years ago. My neighbour claims </t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>The Transfer Of Property Act, 1882 § 23; The Transfer Of Property Act, 1882 § 57; The Transfer Of Property Act, 1882 § 114</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="inlineStr"/>
+      <c r="G122" s="3" t="inlineStr"/>
+      <c r="H122" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client owns agricultural land in Hyderabad and faces a claim from a neighbor asserting customary rights to draw water for irrigation. The dispute centers on whether the client’s property transfer laws protect their ownership against such customary claims.  
+Dispute 1: Neighbor’s Customary Water Rights Claim  
+The neighbor asserts customary rights to use the client’s land for irrigation water.  
+The Transfer Of Property Act, 1882, Section 57 — Effect of Sale Proceeds  
+Section 57 outlines how proceeds from a property sale should be distributed to satisfy prior obligations, such as mortgages, before transferring remaining funds to the rightful owner.  
+This section is irrelevant to the dispute because it addresses financial obligations from property sales, not water rights or customary usage. The client’s ownership of the land is not contested here, and the neighbor’s claim pertains to usage rights, not financial transactions.  
+The Transfer Of Property Act, 1882, Section 114 — Holding Over After Lease Termination  
+Section 114 specifies that if a lessee remains in possession after a lease ends and the lessor accepts rent, the lease is renewed on a month-to-month basis.  
+This section does not apply because the neighbor’s claim is not about a lease or rental agreement but about customary rights to draw water. The client’s ownership is established, and the neighbor’s assertion of customary rights falls outside the scope of leasehold renewals.  
+The Indian Contract Act, 1872, Section 23 — Transfer of Property by Disqualified Persons  
+Section 23 prohibits transferring property by individuals disqualified from holding it, such as tenants defaulting on revenue.  
+This section is also irrelevant. The client’s ownership is not challenged, and the neighbor’s claim does not involve transferring property or disqualification. The focus is on usage rights, not transferability.  
+─────────────────────────────────────────────────────────  
+Was the neighbor’s claim of customary rights documented in any local custom or recorded in land records? This determines whether customary rights are recognized under applicable laws, though the provided materials do not address such claims.  
+If you'd like, I can find relevant court judgments on this, or give you a full legal opinion.</t>
+        </is>
+      </c>
+      <c r="I122" s="3" t="inlineStr"/>
+      <c r="J122" s="3" t="inlineStr"/>
+      <c r="K122" s="3" t="inlineStr"/>
+      <c r="L122" s="3" t="inlineStr"/>
+      <c r="M122" s="3" t="inlineStr"/>
+      <c r="N122" s="3" t="inlineStr"/>
+      <c r="O122" s="3" t="inlineStr"/>
+      <c r="P122" s="3" t="inlineStr"/>
+      <c r="Q122" s="3" t="inlineStr"/>
+      <c r="R122" s="3" t="inlineStr"/>
+      <c r="S122" s="3" t="inlineStr"/>
+      <c r="T122" s="3" t="inlineStr"/>
+      <c r="U122" s="3" t="inlineStr"/>
+      <c r="V122" s="3" t="inlineStr"/>
+      <c r="W122" s="3" t="inlineStr"/>
+    </row>
+    <row r="123" ht="60" customHeight="1">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 10:40 AM</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-003</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>I purchased a residential plot in Warangal but the registration is in my name only, even though my wife contributed substantially to the purchase. Can she claim ownership rights? What does the succession law say?</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>I purchased a residential plot in Warangal but the registration is in my name on</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>The Hindu Succession Act, 1956 § 6; The Hindu Succession Act, 1956 § 29; The Transfer Of Property Act, 1882 § 23; The Transfer Of Property Act, 1882 § 57; The Specific Relief Act, 1963 § 16; S Property Act, 1874 § 2</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr"/>
+      <c r="G123" s="3" t="inlineStr"/>
+      <c r="H123" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client purchased a residential plot in Warangal, registered solely in his name, despite his wife's substantial financial contribution. The dispute centers on whether the wife can claim ownership rights during the client’s lifetime and her potential succession rights if the client passes away.  
+Dispute 1: Wife’s Claim to Ownership Rights  
+The wife’s substantial contribution to the property purchase may entitle her to a claim against the client, potentially through a trust or contractual arrangement.  
+The Transfer Of Property Act, 1882, Section 57 — Transfer of Sale Proceeds to Trustee  
+Section 57 mandates that proceeds from the sale of property held in trust must first satisfy costs, debts, and then be distributed to the rightful beneficiary. If the wife’s contribution was a loan or trust, her claim could override the registration in the client’s name.  
+┌──────────────────────────────────────────────────────┐  
+│  "section 57 of a sum to meet any prior incumbrance, shall, in the absence of a contract to the contrary,  
+│  be held by him in trust to be applied by him, first, in payment of all costs, charges and expenses  
+│  properly incurred by him as incident to the sale or any attempted sale; and, secondly, discharge of the  
+│  mortgage-money and costs and other money, if any, due under the mortgage; and the residue of the  
+│  money so received shall be paid to the person entitled to the mortgaged property, or authorised to  
+│  give receipts for the proceeds of the sale thereof."  
+└──────────────────────────────────────────────────────┘  
+The Specific Relief Act, 1963, Section 16 — Specific Performance of Trust Contracts  
+Section 16 allows specific performance of contracts tied to trusts. If the wife’s contribution was a trust, the court may enforce her rights despite the registration.  
+┌──────────────────────────────────────────────────────┐  
+│  "section 16. 1. Subs. by Act 18 of 2018, s 3, for section 10 (w.e.f. 1-10-2018).  
+│  5 11. Cases in which specific performance of contracts connected with trusts enforceable.—(1)  
+│  Except as otherwise provided in this Act, specific performance of a 1[contract shall], be enforced when the  
+│  act agreed to be done is in the performance wholly or partly of a trust."  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: Wife’s Succession Rights If Client Passes Away  
+The wife may inherit the property under the Hindu Succession Act, 1956, if she is deemed a co-parcener or if the property is treated as her separate asset.  
+The Hindu Succession Act, 1956, Section 6 — Daughter’s Co-Parcenary Rights  
+Section 6 grants daughters in a joint Hindu family equal rights to co-parcenary property as sons. However, this applies only if the wife is part of the joint family and the property is ancestral. If the property is self-acquired, the wife’s rights depend on the client’s will or testamentary disposition.  
+┌──────────────────────────────────────────</t>
+        </is>
+      </c>
+      <c r="I123" s="3" t="inlineStr"/>
+      <c r="J123" s="3" t="inlineStr"/>
+      <c r="K123" s="3" t="inlineStr"/>
+      <c r="L123" s="3" t="inlineStr"/>
+      <c r="M123" s="3" t="inlineStr"/>
+      <c r="N123" s="3" t="inlineStr"/>
+      <c r="O123" s="3" t="inlineStr"/>
+      <c r="P123" s="3" t="inlineStr"/>
+      <c r="Q123" s="3" t="inlineStr"/>
+      <c r="R123" s="3" t="inlineStr"/>
+      <c r="S123" s="3" t="inlineStr"/>
+      <c r="T123" s="3" t="inlineStr"/>
+      <c r="U123" s="3" t="inlineStr"/>
+      <c r="V123" s="3" t="inlineStr"/>
+      <c r="W123" s="3" t="inlineStr"/>
+    </row>
+    <row r="124" ht="60" customHeight="1">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 10:42 AM</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-004</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>My father executed a gift deed for his property in favour of my younger brother last month, despite promising it to me. Can I challenge this transfer on grounds of undue influence?</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">My father executed a gift deed for his property in favour of my younger brother </t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>The Transfer Of Property Act, 1882 § 23; The Transfer Of Property Act, 1882 § 57; The Specific Relief Act, 1963 § 16</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="inlineStr"/>
+      <c r="G124" s="3" t="inlineStr"/>
+      <c r="H124" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+Your father transferred his property to your younger brother via a gift deed, despite promising it to you. You seek to challenge this transfer on grounds of undue influence, raising questions about the validity of the gift deed under relevant legal provisions.  
+Dispute 1: Gift Deed Validity and Undue Influence  
+Your father’s transfer of property to your brother, despite a prior promise to you, raises questions about the validity of the gift deed under the Indian Contract Act, 1872.  
+The Indian Contract Act, 1872 — Section 23  
+Section 23 of the Indian Contract Act, 1872 (9 of 1872), or (3) to a person legally disqualified to be transferee].  
+This section addresses voidable contracts due to undue influence, where one party is in a position to dominate the will of the other. If your father was under undue influence when executing the gift deed, the transfer may be voidable. The key issue is whether your father’s promise to you created a legal obligation that the gift deed breached, and whether the brother exerted undue influence to override that promise.  
+┌──────────────────────────────────────────────────────┐  
+│  Nothing in this section shall be deemed to authorise a tenant having an untransferable │  
+│  right of occupancy, the farmer of an estate in respect of which default has been made in │  
+│  paying revenue, or the lessee of an estate under the management of a Court of Wards, to │  
+│  assign his interest as such tenant, farmer or lessee. │  
+└──────────────────────────────────────────────────────┘  
+If case laws are listed under this section in the materials, add:  
+- [Case name]: [2–3 sentences — (a) what legal principle this case establishes, and (b) exactly how that principle supports or weakens the client’s position in this dispute.]  
+Dispute 2: Transfer of Property Act and Trust Obligations  
+The Transfer of Property Act, 1882 — Section 57  
+Section 57 of a sum to meet any prior incumbrance, shall, in the absence of a contract to the contrary,  
+be held by him in trust to be applied by him, first, in payment of all costs, charges and expenses  
+properly incurred by him as incident to the sale or any attempted sale; and, secondly, discharge of the  
+mortgage-money and costs and other money, if any, due under the mortgage; and the residue of the  
+money so received shall be paid to the person entitled to the mortgaged property, or authorised to  
+give receipts for the proceeds of the sale thereof.  
+This section governs the disposition of proceeds from the sale of mortgaged property, requiring the proceeds to be held in trust for specific obligations. While your father’s transfer is a gift, not a sale, this section may indirectly relate if the property had prior incumbrances. If the gift deed was executed to bypass such obligations, it could conflict with Section 57’s trust obligations, potentially affecting the transfer’s validity. However, this is speculative without evidence of prior mortgages or incum</t>
+        </is>
+      </c>
+      <c r="I124" s="3" t="inlineStr"/>
+      <c r="J124" s="3" t="inlineStr"/>
+      <c r="K124" s="3" t="inlineStr"/>
+      <c r="L124" s="3" t="inlineStr"/>
+      <c r="M124" s="3" t="inlineStr"/>
+      <c r="N124" s="3" t="inlineStr"/>
+      <c r="O124" s="3" t="inlineStr"/>
+      <c r="P124" s="3" t="inlineStr"/>
+      <c r="Q124" s="3" t="inlineStr"/>
+      <c r="R124" s="3" t="inlineStr"/>
+      <c r="S124" s="3" t="inlineStr"/>
+      <c r="T124" s="3" t="inlineStr"/>
+      <c r="U124" s="3" t="inlineStr"/>
+      <c r="V124" s="3" t="inlineStr"/>
+      <c r="W124" s="3" t="inlineStr"/>
+    </row>
+    <row r="125" ht="60" customHeight="1">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 10:45 AM</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-005</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>A landlord in Secunderabad locked me out of my rented premises without following proper legal procedure. What sections of the Telangana Tenancy Act protect me?</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>A landlord in Secunderabad locked me out of my rented premises without following</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>The Specific Relief Act, 1963 § 16; The Code Of Civil Procedure, 1908 § 60; The Code Of Civil Procedure, 1908 § 9A</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr"/>
+      <c r="G125" s="3" t="inlineStr"/>
+      <c r="H125" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A tenant in Secunderabad was unlawfully locked out of their rented premises without following proper legal procedure, raising concerns about the landlord’s adherence to statutory protections for tenants.  
+Dispute 1: Landlord unlawfully locked tenant out of premises  
+The landlord locked the tenant out of their rented premises without following the legal procedure required by the law.  
+The Specific Relief Act, 1963, Section 16 — Specific Performance of Contracts Connected with Trusts  
+Section 16 of the Specific Relief Act, 1963, addresses the enforceability of specific performance of contracts connected to trusts. While this section is not directly applicable to tenancy disputes, it underscores the principle that contractual obligations, including those related to property, must be upheld unless explicitly waived or breached.  
+┌──────────────────────────────────────────────────────┐  
+│  Except as otherwise provided in this Act, specific performance of a contract shall be enforced when the act agreed to be done is in the performance wholly or partly of a trust. │  
+└──────────────────────────────────────────────────────┘  
+The Code of Civil Procedure, 1908, Section 60 — Amendment to Section 60  
+Section 60 of the Code of Civil Procedure, 1908, pertains to the amendment of procedural rules, including the insertion of provisions related to authorities. While this section does not directly address tenancy disputes, it highlights the procedural rigor required in legal proceedings, which may be relevant if the tenant seeks judicial intervention.  
+┌──────────────────────────────────────────────────────┐  
+│  [Verbatim text not fully provided in materials, but amendment relates to procedural rules.] │  
+└──────────────────────────────────────────────────────┘  
+─────────────────────────────────────────────────────────  
+Was the attack carried out with any weapon, or with bare hands only? This determines whether a more serious provision applies.  
+If you'd like, I can find relevant court judgments on this, or give you a full legal opinion.</t>
+        </is>
+      </c>
+      <c r="I125" s="3" t="inlineStr"/>
+      <c r="J125" s="3" t="inlineStr"/>
+      <c r="K125" s="3" t="inlineStr"/>
+      <c r="L125" s="3" t="inlineStr"/>
+      <c r="M125" s="3" t="inlineStr"/>
+      <c r="N125" s="3" t="inlineStr"/>
+      <c r="O125" s="3" t="inlineStr"/>
+      <c r="P125" s="3" t="inlineStr"/>
+      <c r="Q125" s="3" t="inlineStr"/>
+      <c r="R125" s="3" t="inlineStr"/>
+      <c r="S125" s="3" t="inlineStr"/>
+      <c r="T125" s="3" t="inlineStr"/>
+      <c r="U125" s="3" t="inlineStr"/>
+      <c r="V125" s="3" t="inlineStr"/>
+      <c r="W125" s="3" t="inlineStr"/>
+    </row>
+    <row r="126" ht="60" customHeight="1">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 10:51 AM</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-006</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>I encroached on government land near Hyderabad two years ago. The district collector has now issued a notice under the Land Encroachment Act. Can I claim adverse possession or must I vacate immediately?</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>I encroached on government land near Hyderabad two years ago. The district colle</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>The Transfer Of Property Act, 1882 § 23; The Transfer Of Property Act, 1882 § 57; The Transfer Of Property Act, 1882 § 114; The Telangana Land Encroachment Act, 1905 § 6; The Telangana Land Encroachment Act, 1905 § 8; India Code: Section Details § 17</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr"/>
+      <c r="G126" s="3" t="inlineStr"/>
+      <c r="H126" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client encroached on government land in Hyderabad two years ago and now faces a notice under the Telangana Land Encroachment Act. The dispute centers on whether the client can claim adverse possession or must vacate immediately, given the statutory framework governing encroachment and property rights.  
+Dispute 1: Notice Under the Land Encroachment Act  
+The District Collector has issued a notice under the Telangana Land Encroachment Act, 1905, requiring the client to vacate the encroached land.  
+The Telangana Land Encroachment Act, 1905 — Section 6  
+Section 6 mandates that notices under the Act be served in a manner prescribed by the State Government, either under the Telangana Revenue Recovery Act, 1864, or other rules. This procedural requirement ensures the notice is legally valid but does not determine ownership.  
+┌──────────────────────────────────────────────────────┐  
+│ Such notice shall be served in the manner prescribed │  
+└───────────────────────────────────────────────────────┘  
+The case law highlights that notices under this Act are part of the State Government’s process to reclaim encroached land. For example, *Appellants v. State of Telangana and others (2023)* emphasizes that the State’s overriding orders (e.g., GOM 1122) govern land alienation, reinforcing that encroachment notices are administrative steps, not determinations of ownership. The client must comply with the notice’s procedural requirements but cannot assume ownership unless other statutory provisions (like adverse possession) apply.  
+Dispute 2: Claim of Adverse Possession  
+The client seeks to claim adverse possession of the encroached land, despite the notice under the Land Encroachment Act.  
+The Transfer of Property Act, 1882 — Section 23  
+Section 23 prohibits transferring property to persons legally disqualified (e.g., those without a valid title). Adverse possession requires continuous, uninterrupted possession for a statutory period (usually 12 years in some states), which the client has not met.  
+┌──────────────────────────────────────────────────────┐  
+│ Nothing in this section shall be deemed to authorise a tenant... to assign his interest as such tenant... │  
+└───────────────────────────────────────────────────────┘  
+*Appellant v. Goundla Venkaiah and another (2001)* clarifies that government land cannot be claimed via adverse possession unless it is registered and meets specific criteria. The client’s two-year encroachment falls far short of the required duration, and the notice under the Land Encroachment Act further undermines any claim to ownership.  
+The Transfer of Property Act, 1882 — Section 114  
+Section 114 addresses holding over after a lease expires, but it does not apply here since the client is not a lessee.  
+┌──────────────────────────────────────────────────────┐  
+│ If a lessee... remains in possession... the lease is renewed... │  
+└───────────────────────────────────────────────────────┘  
+Th</t>
+        </is>
+      </c>
+      <c r="I126" s="3" t="inlineStr"/>
+      <c r="J126" s="3" t="inlineStr"/>
+      <c r="K126" s="3" t="inlineStr"/>
+      <c r="L126" s="3" t="inlineStr"/>
+      <c r="M126" s="3" t="inlineStr"/>
+      <c r="N126" s="3" t="inlineStr"/>
+      <c r="O126" s="3" t="inlineStr"/>
+      <c r="P126" s="3" t="inlineStr"/>
+      <c r="Q126" s="3" t="inlineStr"/>
+      <c r="R126" s="3" t="inlineStr"/>
+      <c r="S126" s="3" t="inlineStr"/>
+      <c r="T126" s="3" t="inlineStr"/>
+      <c r="U126" s="3" t="inlineStr"/>
+      <c r="V126" s="3" t="inlineStr"/>
+      <c r="W126" s="3" t="inlineStr"/>
+    </row>
+    <row r="127" ht="60" customHeight="1">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 10:57 AM</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-007</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>My ancestral property in Nizamabad was partitioned among three siblings, but the title deed has never been formally registered. What are the legal implications?</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>My ancestral property in Nizamabad was partitioned among three siblings, but the</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>The Transfer Of Property Act, 1882 § 23; The Transfer Of Property Act, 1882 § 57; The Transfer Of Property Act, 1882 § 114</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr"/>
+      <c r="G127" s="3" t="inlineStr"/>
+      <c r="H127" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client’s ancestral property in Nizamabad was partitioned among three siblings, but the title deed has never been formally registered, raising questions about the legal validity of the partition and the rights of the siblings.  
+Dispute 1: Partition Without Title Deed Registration  
+The partition of the ancestral property among three siblings occurred without formal registration of the title deed.  
+The Transfer Of Property Act, 1882, Section 23 — Transfer of Property by Disqualified Person  
+Section 23 of the Indian Contract Act, 1872 (9 of 1872), or (3) to a person legally disqualified to be transferee].  
+This section prohibits the transfer of property by a person disqualified to be a transferee, such as a tenant with an untransferable right of occupancy. While the text appears to reference the Indian Contract Act, it may inadvertently overlap with provisions of the Transfer of Property Act. If the partition involved transferring ownership without legal registration, the lack of a valid title deed could render the transfer invalid, as registration is a prerequisite for legal recognition under Indian law.  
+┌──────────────────────────────────────────────────────┐  
+│  section 23 of the Indian Contract Act, 1872 (9 of 1872), or (3) to a person legally disqualified to be transferee].  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: Partition Without Title Deed Registration  
+The partition of the ancestral property among three siblings occurred without formal registration of the title deed.  
+The Transfer Of Property Act, 1882, Section 57 — Sale of Mortgaged Property  
+Section 57 of a sum to meet any prior incumbrance, shall, in the absence of a contract to the contrary, be held by him in trust to be applied by him, first, in payment of all costs, charges and expenses properly incurred by him as incident to the sale or any attempted sale; and, secondly, discharge of the mortgage-money and costs and other money, if any, due under the mortgage; and the residue of the money so received shall be paid to the person entitled to the mortgaged property, or authorised to give receipts for the proceeds of the sale thereof.  
+This section governs the distribution of proceeds from the sale of mortgaged property, but its relevance here is indirect. The lack of a registered title deed could affect the enforceability of any claims or rights arising from the partition, as unregistered documents are generally not admissible in court. Without a valid title, the siblings’ ownership may be challenged, and the partition could be deemed invalid.  
+┌──────────────────────────────────────────────────────┐  
+│  section 57 of a sum to meet any prior incumbrance, shall, in the absence of a contract to the contrary, be held by him in trust to be applied by him, first, in payment of all costs, charges and expenses properly incurred by him as incident to the sale or any attempted sale; and, secondly, discharge of the mortgage-m</t>
+        </is>
+      </c>
+      <c r="I127" s="3" t="inlineStr"/>
+      <c r="J127" s="3" t="inlineStr"/>
+      <c r="K127" s="3" t="inlineStr"/>
+      <c r="L127" s="3" t="inlineStr"/>
+      <c r="M127" s="3" t="inlineStr"/>
+      <c r="N127" s="3" t="inlineStr"/>
+      <c r="O127" s="3" t="inlineStr"/>
+      <c r="P127" s="3" t="inlineStr"/>
+      <c r="Q127" s="3" t="inlineStr"/>
+      <c r="R127" s="3" t="inlineStr"/>
+      <c r="S127" s="3" t="inlineStr"/>
+      <c r="T127" s="3" t="inlineStr"/>
+      <c r="U127" s="3" t="inlineStr"/>
+      <c r="V127" s="3" t="inlineStr"/>
+      <c r="W127" s="3" t="inlineStr"/>
+    </row>
+    <row r="128" ht="60" customHeight="1">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 11:01 AM</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-008</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>I want to sell my property in Karimnagar to a buyer, but there is a pending civil suit regarding boundary demarcation. Can I execute a valid sale deed? What protective measures exist?</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>I want to sell my property in Karimnagar to a buyer, but there is a pending civi</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>The Transfer Of Property Act, 1882 § 23; The Transfer Of Property Act, 1882 § 57; The Transfer Of Property Act, 1882 § 114</t>
+        </is>
+      </c>
+      <c r="F128" s="3" t="inlineStr"/>
+      <c r="G128" s="3" t="inlineStr"/>
+      <c r="H128" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A pending civil suit over boundary demarcation may affect the validity of a property sale, requiring scrutiny of legal provisions governing transfers and encumbrances. The client must ensure the sale deed complies with statutory requirements and includes protective clauses to mitigate risks from unresolved disputes.  
+Dispute 1: Pending Civil Suit Affects Property Sale Validity  
+A civil suit over boundary demarcation may create an encumbrance on the property, potentially invalidating the sale unless resolved.  
+**Transfer Of Property Act, 1882** Section 57 — *Sale Proceeds and Trust for Prior Incumbrances*  
+Section 57 mandates that sale proceeds be held in trust to first settle costs and prior claims, such as pending litigation. If the boundary dispute is a prior incumbrance, the buyer may claim proceeds to resolve it, risking the seller’s ownership.  
+┌──────────────────────────────────────────────────────┐  
+│  "section 57 of a sum to meet any prior incumbrance, shall, in the absence of a contract to the contrary,  
+│  be held by him in trust to be applied by him, first, in payment of all costs, charges and expenses  
+│  properly incurred by him as incident to the sale or any attempted sale; and, secondly, discharge of the  
+│  mortgage-money and costs and other money, if any, due under the mortgage; and the residue of the  
+│  money so received shall be paid to the person entitled to the mortgaged property, or authorised to  
+│  give receipts for the proceeds of the sale thereof."  
+└──────────────────────────────────────────────────────┘  
+- **APPELLANTS v. TUKARAM (2026)**: The Supreme Court emphasized that a sale deed must explicitly address prior claims, such as boundary disputes, to avoid ambiguity. This supports the need for a clause in the sale deed to resolve such issues.  
+- **Celir LLP v. Bafna Motors (2024)**: While not directly relevant, this case clarifies that statutory exclusions in Section 13 of the Transfer of Property Act do not override the requirement to address encumbrances, reinforcing the importance of resolving pending disputes before transfer.  
+─────────────────────────────────────────────────────────  
+Dispute 2: Legal Disqualification of Transferee  
+The buyer’s legal standing may be challenged if the pending suit affects their ownership rights.  
+**Indian Contract Act, 1872** Section 23 — *Transfer to Disqualified Persons*  
+Section 23 prohibits transferring property to persons disqualified by law, such as those with unresolved claims. If the boundary dispute implicates the buyer’s title, the seller could be liable for transferring to an ineligible party.  
+┌──────────────────────────────────────────────────────┐  
+│  "section 23 of the Indian Contract Act, 1872 (9 of 1872), or (3) to a person legally  
+│  disqualified to be transferee]."  
+└──────────────────────────────────────────────────────┘  
+- **APPELLANTS v. TUKARAM (2026)**: The case underscores that a sale deed must explicitly</t>
+        </is>
+      </c>
+      <c r="I128" s="3" t="inlineStr"/>
+      <c r="J128" s="3" t="inlineStr"/>
+      <c r="K128" s="3" t="inlineStr"/>
+      <c r="L128" s="3" t="inlineStr"/>
+      <c r="M128" s="3" t="inlineStr"/>
+      <c r="N128" s="3" t="inlineStr"/>
+      <c r="O128" s="3" t="inlineStr"/>
+      <c r="P128" s="3" t="inlineStr"/>
+      <c r="Q128" s="3" t="inlineStr"/>
+      <c r="R128" s="3" t="inlineStr"/>
+      <c r="S128" s="3" t="inlineStr"/>
+      <c r="T128" s="3" t="inlineStr"/>
+      <c r="U128" s="3" t="inlineStr"/>
+      <c r="V128" s="3" t="inlineStr"/>
+      <c r="W128" s="3" t="inlineStr"/>
+    </row>
+    <row r="129" ht="60" customHeight="1">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 11:07 AM</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-009</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>My tenant has not paid rent for 8 months in Hyderabad. What is the proper legal procedure to evict him under the Telangana Tenancy Act, and can I claim recovery?</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">My tenant has not paid rent for 8 months in Hyderabad. What is the proper legal </t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>The Specific Relief Act, 1963 § 16; The Code Of Civil Procedure, 1908 § 60; The Code Of Civil Procedure, 1908 § 9A; The Code Of Civil Procedure, 1908 § 41; Fees Act, 1870 § 6</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr"/>
+      <c r="G129" s="3" t="inlineStr"/>
+      <c r="H129" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A tenant in Hyderabad has defaulted on rent for 8 months, and the client seeks both eviction and recovery of unpaid rent. The legal process for eviction and recovery must be determined under applicable provisions of the Code of Civil Procedure, 1908, and the Specific Relief Act, 1963, with relevant case law guiding the interpretation.  
+Dispute 1: Tenant Defaulted on Rent for 8 Months  
+The tenant has failed to pay rent for 8 months, and the client seeks eviction.  
+**The Code Of Civil Procedure, 1908, Section 60** — *Eviction of tenant for non-payment of rent*  
+Section 60 of the Code of Civil Procedure, 1908, provides that a tenant may be evicted for non-payment of rent, with specific procedural requirements. The amendment in Tamil Nadu and Rajasthan clarifies that the section applies to authorities, reinforcing the landlord’s right to seek eviction through judicial process.  
+┌──────────────────────────────────────────────────────┐  
+│  The Code Of Civil Procedure, 1908, Section 60 (after the words “stipends and gratuities allowed to pensioners of the Government”, the words “or of a authority” shall be inserted). │  
+└──────────────────────────────────────────────────────┘  
+- **SC_2020_N. Motilal versus Faisal Bin Ali (2020)**: The Supreme Court held that non-payment of rent for two months constitutes a breach of lease terms, supporting eviction. This case aligns with the client’s claim of 8 months’ default, strengthening the eviction case.  
+- **APPELLANTS v. TUKARAM (2026)**: The Supreme Court ruled that tenants are liable for eviction if they fail to pay rent for two months, explicitly linking non-payment to breach of contract. This case reinforces the legal basis for eviction under Section 60.  
+Dispute 2: Client Seeks Recovery of Unpaid Rent from Defaulting Tenant  
+The client aims to recover the unpaid rent under the lease agreement.  
+**The Specific Relief Act, 1963, Section 16** — *Specific performance of contracts*  
+Section 16 of the Specific Relief Act, 1963, mandates that specific performance of contracts connected to trusts is enforceable. While this section is not directly applicable to standard lease agreements, it underscores the enforceability of contractual obligations, including rent payment.  
+┌──────────────────────────────────────────────────────┐  
+│  section 16. 1. Subs. by Act 18 of 2018, s 3, for section 10 (w.e.f. 1- длинна текста не полностью предоставлена. │  
+└──────────────────────────────────────────────────────┘  
+- **The Specific Relief Act, 1963, Section 41** (incomplete text): This section pertains to staying orders related to employees, which is not directly relevant to rent recovery. However, the broader framework of the Act supports the enforceability of lease terms, including rent payment.  
+**The Code Of Civil Procedure, 1908, Section 41** — *Filing suits for recovery*  
+Section 41 of the Code of Civil Procedure, 1908, outlines procedural requirements for filing suits, includ</t>
+        </is>
+      </c>
+      <c r="I129" s="3" t="inlineStr"/>
+      <c r="J129" s="3" t="inlineStr"/>
+      <c r="K129" s="3" t="inlineStr"/>
+      <c r="L129" s="3" t="inlineStr"/>
+      <c r="M129" s="3" t="inlineStr"/>
+      <c r="N129" s="3" t="inlineStr"/>
+      <c r="O129" s="3" t="inlineStr"/>
+      <c r="P129" s="3" t="inlineStr"/>
+      <c r="Q129" s="3" t="inlineStr"/>
+      <c r="R129" s="3" t="inlineStr"/>
+      <c r="S129" s="3" t="inlineStr"/>
+      <c r="T129" s="3" t="inlineStr"/>
+      <c r="U129" s="3" t="inlineStr"/>
+      <c r="V129" s="3" t="inlineStr"/>
+      <c r="W129" s="3" t="inlineStr"/>
+    </row>
+    <row r="130" ht="60" customHeight="1">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 11:13 AM</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-010</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>I mortgaged my agricultural plot in Medak district to obtain a loan. The lender now wants to sell the property. What are my rights as mortgagor under the Transfer of Property Act?</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I mortgaged my agricultural plot in Medak district to obtain a loan. The lender </t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>The Transfer Of Property Act, 1882 § 23; The Transfer Of Property Act, 1882 § 57; The Transfer Of Property Act, 1882 § 114</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="inlineStr"/>
+      <c r="G130" s="3" t="inlineStr"/>
+      <c r="H130" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client mortgaged an agricultural plot in Medak district to obtain a loan, and the lender now seeks to sell the property without adhering to proper legal procedures. The client seeks to understand their rights under the Transfer of Property Act, 1882, particularly regarding the lender’s authority to sell the mortgaged property and the distribution of proceeds.  
+Dispute 1: Lender’s Attempt to Sell Without Proper Legal Procedures  
+The lender is seeking to sell the mortgaged property without following the required legal formalities under the Transfer of Property Act.  
+**The Transfer Of Property Act, 1882, Section 23** — *Transfer by tenant, farmer, or lessee*  
+This section restricts certain individuals (e.g., tenants, farmers, lessees) from transferring their interest in property unless specific conditions are met. While the client is a mortgagor, not a tenant or lessee, this section may indirectly affect the lender’s authority to sell the property if the mortgage involves a leasehold interest.  
+┌──────────────────────────────────────────────────────┐  
+│  Nothing in this section shall be deemed to authorise a tenant having an untransferable  
+│  right of occupancy, the farmer of an estate in respect of which default has been made in paying  
+│  revenue, or the lessee of an estate under the management of a Court of Wards, to assign his interest  
+│  as such tenant, farmer or lessee.  
+└──────────────────────────────────────────────────────┘  
+This provision may limit the lender’s ability to sell the property if the mortgage involves a leasehold or if the lender is acting as a tenant or lessee. However, since the client is a mortgagor, this section may not directly apply unless the mortgage is tied to a leasehold interest.  
+Dispute 2: Distribution of Proceeds from the Sale of Mortgaged Property  
+The lender’s sale of the property must follow procedures ensuring the mortgagor receives the residue of the sale proceeds after settling the mortgage debt.  
+**The Transfer Of Property Act, 1882, Section 57** — *Sale of mortgaged property*  
+This section mandates that the proceeds from the sale of mortgaged property must first cover costs, then discharge the mortgage debt, and finally be distributed to the mortgagor.  
+┌──────────────────────────────────────────────────────┐  
+│  ...shall, in the absence of a contract to the contrary, be held by him in trust to be applied  
+│  by him, first, in payment of all costs, charges and expenses properly incurred by him as incident  
+│  to the sale or any attempted sale; and, secondly, discharge of the mortgage-money and costs and  
+│  other money, if any, due under the mortgage; and the residue of the money so received shall be  
+│  paid to the person entitled to the mortgaged property, or authorised to give receipts for the  
+│  proceeds of the sale thereof.  
+└──────────────────────────────────────────────────────┘  
+This section ensures the client retains the remaining proceeds</t>
+        </is>
+      </c>
+      <c r="I130" s="3" t="inlineStr"/>
+      <c r="J130" s="3" t="inlineStr"/>
+      <c r="K130" s="3" t="inlineStr"/>
+      <c r="L130" s="3" t="inlineStr"/>
+      <c r="M130" s="3" t="inlineStr"/>
+      <c r="N130" s="3" t="inlineStr"/>
+      <c r="O130" s="3" t="inlineStr"/>
+      <c r="P130" s="3" t="inlineStr"/>
+      <c r="Q130" s="3" t="inlineStr"/>
+      <c r="R130" s="3" t="inlineStr"/>
+      <c r="S130" s="3" t="inlineStr"/>
+      <c r="T130" s="3" t="inlineStr"/>
+      <c r="U130" s="3" t="inlineStr"/>
+      <c r="V130" s="3" t="inlineStr"/>
+      <c r="W130" s="3" t="inlineStr"/>
+    </row>
+    <row r="131" ht="60" customHeight="1">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 11:18 AM</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-011</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>The pattadar pass book for my land in Telangana shows incorrect boundaries. How can I obtain a corrected document? What is the procedure under the Pattadar Pass Books Act?</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The pattadar pass book for my land in Telangana shows incorrect boundaries. How </t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>The Telangana Rights In Land And Pattadar Pass Books Act, 2020 § 6; The Telangana Rights In Land And Pattadar Pass Books Act, 2020 § 11; The Telangana Rights In Land And Pattadar Pass Books Act, 2020 § 1358</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr"/>
+      <c r="G131" s="3" t="inlineStr"/>
+      <c r="H131" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client’s pattadar pass book in Telangana contains incorrect land boundaries, requiring correction under the Telangana Rights In Land And Pattadar Pass Books Act, 2020. The dispute centers on the legal procedures to rectify such errors and the evidentiary weight of the pass book.  
+Dispute 1: Incorrect Boundaries in Pattadar Pass Book  
+The client seeks to correct the recorded boundaries of their land as described in the pattadar pass book.  
+**Telangana Rights In Land And Pattadar Pass Books Act, 2020** Section 6 — *Effecting Change in Record of Rights when acquired*  
+Section 6 outlines procedures for altering the record of rights when ownership is acquired through succession, survivorship, inheritance, or court decree. While this section primarily addresses new acquisitions, it may still be relevant if the boundary error stems from a prior legal transfer or court order.  
+┌──────────────────────────────────────────────────────┐  
+│  6. Effecting Change in Record of Rights when acquired  
+│  the right over the land through succession,  
+│  survivorship, inheritance.  
+└──────────────────────────────────────────────────────┘  
+The client must demonstrate that the boundary error arose from a legally recognized transfer or court order to invoke Section 6. However, if the error is a clerical mistake rather than a result of ownership change, this section may not apply directly.  
+- **HC_2022_# Y. Jaihind Reddy S o Late Sri. Raji Reddy versus $ the State of Telangana, Rep.by Its Principal (2022)**: This case highlights the procedural replacement of the 1971 Act with the 2020 Act, emphasizing the need to follow the 2020 Act’s framework for rectifying record errors. The court’s discussion on the ROR Act’s applicability reinforces that corrections must adhere to the 2020 Act’s specific provisions.  
+Dispute 2: Evidentiary Value of Pattadar Pass Book  
+The client’s pass book may be challenged as evidence due to its incorrect boundaries.  
+**Telangana Rights In Land And Pattadar Pass Books Act, 2020** Section 11 — *Evidentiary value of Pattadar Pass Book-cum-Title Deed*  
+Section 11 establishes the pass book as prima facie evidence of land rights. However, if the document contains errors, its evidentiary value may be disputed, requiring corroboration through other records or legal procedures.  
+┌──────────────────────────────────────────────────────┐  
+│  11. Evidentiary value of Pattadar Pass Book-cum-Title  
+│  Deed.  
+└──────────────────────────────────────────────────────┘  
+The client’s pass book remains admissible as evidence, but the boundary error could undermine its reliability. To strengthen their position, the client should seek to correct the pass book or present alternative documentation to counter the error’s impact.  
+─────────────────────────────────────────────────────────  
+Was the boundary error caused by fraudulent issuance of the pass book, or is it a clerical mistake? This determines whether Section 8</t>
+        </is>
+      </c>
+      <c r="I131" s="3" t="inlineStr"/>
+      <c r="J131" s="3" t="inlineStr"/>
+      <c r="K131" s="3" t="inlineStr"/>
+      <c r="L131" s="3" t="inlineStr"/>
+      <c r="M131" s="3" t="inlineStr"/>
+      <c r="N131" s="3" t="inlineStr"/>
+      <c r="O131" s="3" t="inlineStr"/>
+      <c r="P131" s="3" t="inlineStr"/>
+      <c r="Q131" s="3" t="inlineStr"/>
+      <c r="R131" s="3" t="inlineStr"/>
+      <c r="S131" s="3" t="inlineStr"/>
+      <c r="T131" s="3" t="inlineStr"/>
+      <c r="U131" s="3" t="inlineStr"/>
+      <c r="V131" s="3" t="inlineStr"/>
+      <c r="W131" s="3" t="inlineStr"/>
+    </row>
+    <row r="132" ht="60" customHeight="1">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 11:24 AM</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-012</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>My husband is abusing me physically and emotionally. I want to file a petition under the Domestic Violence Act. What protections and remedies are available to me?</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>My husband is abusing me physically and emotionally. I want to file a petition u</t>
+        </is>
+      </c>
+      <c r="E132" s="3" t="inlineStr">
+        <is>
+          <t>The Bharatiya Nagarik Suraksha Sanhita, 2023 § 356; The Bharatiya Nagarik Suraksha Sanhita, 2023 § 121; The Bharatiya Nagarik Suraksha Sanhita, 2023 § 197; (1) It Shall Be The Duty Of The Protection Officer § 9; India Code: Section Details § 12; India Code: Section Details § 9</t>
+        </is>
+      </c>
+      <c r="F132" s="3" t="inlineStr"/>
+      <c r="G132" s="3" t="inlineStr"/>
+      <c r="H132" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client alleges physical and emotional abuse by her husband, including injuries from assaults and verbal harassment causing mental distress.  
+Dispute 1: Physical Assault Causing Injury  
+The husband assaulted the client, resulting in physical harm.  
+[Bharatiya Nyaya Sanhita] Section 356 — *Assault and causing hurt*  
+Section 356 criminalizes assault that causes hurt, including injuries like those sustained in this case. The provision applies to domestic violence, and if the victim is a woman who cannot appear in court, a third party may file the complaint. This is critical for the client’s case, as it allows her to seek legal recourse without public exposure.  
+┌──────────────────────────────────────────────────────┐  
+│  "Whoever assaults any person, or causes any harm to any person, shall be punished with imprisonment of either description for a term which may extend to one year, or with fine, or with both." │  
+└──────────────────────────────────────────────────────┘  
+- **SC_2025_Geddam Jhansi v. The State of Telangana &amp; Ors.**: This case affirmed that Section 356 applies to domestic violence, reinforcing that assault within a family relationship is punishable under this section.  
+Dispute 2: Emotional Abuse Through Verbal Harassment  
+The husband subjected the client to verbal harassment, causing mental distress.  
+[Protection Officers Act] Section 9 — *Duties of Protection Officers*  
+Section 9 mandates that protection officers provide immediate assistance to victims of domestic violence, including emotional abuse. This allows the client to report the harassment to a designated officer, who can issue protective measures or refer her to legal aid. The section emphasizes the state’s responsibility to address non-physical forms of abuse.  
+┌──────────────────────────────────────────────────────┐  
+│  "The Protection Officer shall, upon receipt of any complaint or information regarding domestic violence, immediately take such action as may be necessary to protect the victim." │  
+└──────────────────────────────────────────────────────┘  
+Dispute 3: Combined Physical and Emotional Abuse  
+The client endured both physical injuries and emotional distress from her husband.  
+[Bharatiya Nyaya Sanhita] Section 356 — *Assault and causing hurt*  
+Section 356 remains applicable for the physical harm, while Section 9 addresses the emotional abuse. The combined nature of the abuse strengthens the case, as both forms of violence are recognized under criminal law. The case law from *SC_2025_Geddam Jhansi* supports the application of Section 356 to domestic violence, including its psychological impacts.  
+┌──────────────────────────────────────────────────────┐  
+│  "Whoever assaults any person, or causes any harm to any person, shall be punished with imprisonment of either description for a term which may extend to one year, or with fine, or with both." │  
+└──────────────────────────────────────────────────────┘  
+───────────────</t>
+        </is>
+      </c>
+      <c r="I132" s="3" t="inlineStr"/>
+      <c r="J132" s="3" t="inlineStr"/>
+      <c r="K132" s="3" t="inlineStr"/>
+      <c r="L132" s="3" t="inlineStr"/>
+      <c r="M132" s="3" t="inlineStr"/>
+      <c r="N132" s="3" t="inlineStr"/>
+      <c r="O132" s="3" t="inlineStr"/>
+      <c r="P132" s="3" t="inlineStr"/>
+      <c r="Q132" s="3" t="inlineStr"/>
+      <c r="R132" s="3" t="inlineStr"/>
+      <c r="S132" s="3" t="inlineStr"/>
+      <c r="T132" s="3" t="inlineStr"/>
+      <c r="U132" s="3" t="inlineStr"/>
+      <c r="V132" s="3" t="inlineStr"/>
+      <c r="W132" s="3" t="inlineStr"/>
+    </row>
+    <row r="133" ht="60" customHeight="1">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 11:29 AM</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-013</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>I married my spouse without parental consent under the Special Marriage Act. My family is challenging the validity of the marriage. What are my legal rights?</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I married my spouse without parental consent under the Special Marriage Act. My </t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>The Indian Christian Marriage Act, 1872 § 10; The Indian Christian Marriage Act, 1872 § 69; The Indian Christian Marriage Act, 1872 § 9</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr"/>
+      <c r="G133" s="3" t="inlineStr"/>
+      <c r="H133" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client married their spouse without parental consent under the Special Marriage Act, but their family is challenging the marriage's validity. The materials provided focus on the Indian Christian Marriage Act, 1872, which governs different procedural aspects of marriages, not parental consent under the Special Marriage Act. This creates a critical gap in the legal analysis, as the provided materials do not address the specific issue of parental consent in the Special Marriage Act.  
+Dispute 1: Marriage Solemnized Outside Prescribed Time  
+The client's marriage may have been conducted outside the legally permitted hours for solemnization.  
+Indian Christian Marriage Act, 1872 Section 10 — Time for solemnizing marriage  
+Section 10 of the Indian Christian Marriage Act, 1872, specifies that marriages must be solemnized between 6 a.m. and 7 p.m., with exceptions for clergy of specific religious denominations. This section is relevant if the marriage was conducted outside these hours, which could render it invalid under this Act.  
+┌──────────────────────────────────────────────────────┐  
+│  Every marriage under this Act shall be solemnized between │  
+│  the hours of six in the morning and seven in the evening: │  
+└──────────────────────────────────────────────────────┘  
+- SC_2021_Arunoday Singh … Petitioner (s) versus Lee Anne Elton … Respondent (s) (2021): This case clarified that the Special Marriage Act does not extend the Limitation Act’s applicability to challenges under its provisions. While this case pertains to procedural delays, it indirectly supports the idea that challenges to marriage validity under the Special Marriage Act are not subject to strict time limits, which could be relevant if the family’s challenge is delayed.  
+Dispute 2: Marriage Conducted Without Required Witnesses  
+The marriage may have been solemnized without the mandated number of witnesses, which could invalidate it.  
+Indian Christian Marriage Act, 1872 Section 69 — Solemnizing marriage out of proper time, or without witnesses  
+Section 69 penalizes the solemnization of marriages outside the prescribed time or without at least two credible witnesses. This section is critical if the marriage lacked witnesses, as it could render the marriage void.  
+┌──────────────────────────────────────────────────────┐  
+│  Whoever knowingly and wilfully solemnizes a marriage … at │  
+│  any time other than between the hours of six in the morning │  
+│  and seven in the evening, or in the absence of at least two │  
+│  credible witnesses … shall be punished with imprisonment … │  
+└──────────────────────────────────────────────────────┘  
+- SC_2021_Arunoday Singh … Petitioner (s) versus Lee Anne Elton … Respondent (s) (2021): This case reinforces that procedural violations under the Special Marriage Act (such as lack of witnesses) are not subject to the Limitation Act’s time limits. However, this does not directly address the validity of the marriage</t>
+        </is>
+      </c>
+      <c r="I133" s="3" t="inlineStr"/>
+      <c r="J133" s="3" t="inlineStr"/>
+      <c r="K133" s="3" t="inlineStr"/>
+      <c r="L133" s="3" t="inlineStr"/>
+      <c r="M133" s="3" t="inlineStr"/>
+      <c r="N133" s="3" t="inlineStr"/>
+      <c r="O133" s="3" t="inlineStr"/>
+      <c r="P133" s="3" t="inlineStr"/>
+      <c r="Q133" s="3" t="inlineStr"/>
+      <c r="R133" s="3" t="inlineStr"/>
+      <c r="S133" s="3" t="inlineStr"/>
+      <c r="T133" s="3" t="inlineStr"/>
+      <c r="U133" s="3" t="inlineStr"/>
+      <c r="V133" s="3" t="inlineStr"/>
+      <c r="W133" s="3" t="inlineStr"/>
+    </row>
+    <row r="134" ht="60" customHeight="1">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 11:35 AM</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-014</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>My wife has obtained a divorce under the Muslim personal law in 2022 through instant triple talaq. Can I challenge this now? What are her rights to maintenance and mahr?</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>My wife has obtained a divorce under the Muslim personal law in 2022 through ins</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>The Muslim Women (Protection Of Rights On Marriage) Act, 2019 § 3; Application Act, 1937 § 1</t>
+        </is>
+      </c>
+      <c r="F134" s="3" t="inlineStr"/>
+      <c r="G134" s="3" t="inlineStr"/>
+      <c r="H134" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+In 2022, the client’s wife obtained a divorce through instant triple talaq under Muslim personal law. The client seeks to challenge this divorce, understand his wife’s maintenance rights, and determine her entitlement to mahr.  
+Dispute 1: Can I challenge my wife's divorce obtained through instant triple talaq in 2022?  
+The legality of the divorce and potential criminal consequences for the husband.  
+The Muslim Women (Protection Of Rights On Marriage) Act, 2019, Section 3 — Punishment for pronouncing talaq.  
+Section 3 of the 2019 Act criminalizes the practice of instant triple talaq, imposing imprisonment up to three years and a fine on the husband who issues it. This section directly addresses the validity of the divorce and the husband’s liability for violating the law. Since the divorce was obtained through instant triple talaq, the husband may face criminal charges under this section, which could affect the divorce’s legal standing.  
+┌──────────────────────────────────────────────────────┐  
+│  section 3 upon his wife shall be punished with imprisonment for a term which may extend to three years,  
+│  and shall also be liable to fine.  
+└──────────────────────────────────────────────────────┘  
+- **Mohd. Abdul Samad v. The State of Telangana (2024)**: This case highlights the application of Section 5 of the 2019 Act, which mandates subsistence allowance for divorced Muslim women. While the case does not directly address criminal liability, it reinforces the Act’s intent to protect women’s rights post-divorce, indirectly supporting the validity of Section 3’s punitive measures.  
+Dispute 2: What are my wife's rights to maintenance after her divorce through instant triple talaq?  
+Entitlement to financial support under statutory provisions.  
+The Muslim Women (Protection Of Rights On Marriage) Act, 2019, Section 5 — Subsistence allowance.  
+Section 5 of the 2019 Act entitles a divorced Muslim woman to receive subsistence allowance from her husband, determined by a Magistrate. This provision ensures financial support for the wife and her dependents, regardless of the divorce method. Since the divorce was through instant triple talaq, the husband is still legally obligated to provide maintenance under this section.  
+┌──────────────────────────────────────────────────────┐  
+│  5. Subsistence allowance.—Without prejudice to the generality of the provisions contained in any  
+│  other law for the time being in force, a married Muslim woman upon whom talaq is pronounced shall be  
+│  entitled to receive from her husband such amount of subsistence allowance, for her and dependent  
+│  children, as may be determined by the Magistrate.  
+└──────────────────────────────────────────────────────┘  
+- **Appellants v. SAHIDUL HAQ CHISTI (2011)**: The Supreme Court recognized that maintenance claims under Section 125 of the Criminal Procedure Code (Cr.P.C.) are valid even if the husband divorced the wife via triple talaq. Thi</t>
+        </is>
+      </c>
+      <c r="I134" s="3" t="inlineStr"/>
+      <c r="J134" s="3" t="inlineStr"/>
+      <c r="K134" s="3" t="inlineStr"/>
+      <c r="L134" s="3" t="inlineStr"/>
+      <c r="M134" s="3" t="inlineStr"/>
+      <c r="N134" s="3" t="inlineStr"/>
+      <c r="O134" s="3" t="inlineStr"/>
+      <c r="P134" s="3" t="inlineStr"/>
+      <c r="Q134" s="3" t="inlineStr"/>
+      <c r="R134" s="3" t="inlineStr"/>
+      <c r="S134" s="3" t="inlineStr"/>
+      <c r="T134" s="3" t="inlineStr"/>
+      <c r="U134" s="3" t="inlineStr"/>
+      <c r="V134" s="3" t="inlineStr"/>
+      <c r="W134" s="3" t="inlineStr"/>
+    </row>
+    <row r="135" ht="60" customHeight="1">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 11:38 AM</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-015</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>My deceased Hindu father had no will. I am an unmarried daughter. What are my inheritance rights under the Hindu Succession Act? Does my mother have superior rights?</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>My deceased Hindu father had no will. I am an unmarried daughter. What are my in</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>The Hindu Succession Act, 1956 § 6; The Hindu Succession Act, 1956 § 29</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="inlineStr"/>
+      <c r="G135" s="3" t="inlineStr"/>
+      <c r="H135" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+Your deceased Hindu father died without a will, and as his unmarried daughter, you have inheritance rights under the Hindu Succession Act. Your mother’s rights depend on her status as a widow or coparcener, but you are entitled to a share in his property as a daughter under the Act.  
+Dispute 1: Daughter’s Inheritance Rights Under Hindu Succession Act  
+Your right to inherit your father’s property as an unmarried daughter is protected under the Hindu Succession Act, 1956.  
+The Hindu Succession Act, 1956 — Section 6  
+Section 6(a) grants daughters of coparceners equal rights to property as sons, including the right to claim by survivorship.  
+┌──────────────────────────────────────────────────────┐  
+│  (a) in a joint Hindu family governed by Mitakshara law, the daughter of a co-parcener shall by  
+│  birth become a co-parcener in her own right in the same manner as the son and have the same rights  
+│  in the co-parcenary property as she would have had if she had been a son inclusive of the right to  
+│  claim by survivorship and shall be subject to the same liabilities and disabilities in respect thereto as  
+│  the son;  
+└──────────────────────────────────────────────────────┘  
+This section ensures you are treated equally to your brother(s) in the coparcenary property. If your father died without a will, your share is determined by the rules of intestate succession under the Act.  
+Dispute 2: Devolution of Property by Survivorship  
+Your interest in your father’s property may devolve by survivorship, but this depends on whether he left descendants.  
+The Hindu Succession Act, 1956 — Section 29-A  
+Section 29-A specifies that a female Hindu’s interest in coparcenary property devolves by survivorship unless the deceased left a child or child of a pre-deceased child.  
+┌──────────────────────────────────────────────────────┐  
+│  (a) her interest in the property shall devolve by survivorship upon the surviving members of the  
+│  coparcenary and not in accordance with this Act:  
+│  Provided that if the deceased had left any child or child of a pre-deceased child, the interest of the  
+│  deceased in the Mitakshara coparcenary property shall devolve by testamentary or intestate  
+│  succession, as the case may be, under this Act and not by survivorship.  
+└──────────────────────────────────────────────────────┘  
+If your father had no children, your share would pass to surviving coparceners (e.g., your mother or siblings). If he had children, your right to survivorship would be overridden by their inheritance claims.  
+─────────────────────────────────────────────────────────  
+- **A Abhilasha v. Parkash (2020)**: This case emphasizes the statutory obligation to maintain unmarried daughters under Section 20 of the Hindu Adoptions and Maintenance Act, 1956. While it supports your right to maintenance, it does not directly affect inheritance rights under the Hindu Succession Act.  
+If you'd like, I can find relevant c</t>
+        </is>
+      </c>
+      <c r="I135" s="3" t="inlineStr"/>
+      <c r="J135" s="3" t="inlineStr"/>
+      <c r="K135" s="3" t="inlineStr"/>
+      <c r="L135" s="3" t="inlineStr"/>
+      <c r="M135" s="3" t="inlineStr"/>
+      <c r="N135" s="3" t="inlineStr"/>
+      <c r="O135" s="3" t="inlineStr"/>
+      <c r="P135" s="3" t="inlineStr"/>
+      <c r="Q135" s="3" t="inlineStr"/>
+      <c r="R135" s="3" t="inlineStr"/>
+      <c r="S135" s="3" t="inlineStr"/>
+      <c r="T135" s="3" t="inlineStr"/>
+      <c r="U135" s="3" t="inlineStr"/>
+      <c r="V135" s="3" t="inlineStr"/>
+      <c r="W135" s="3" t="inlineStr"/>
+    </row>
+    <row r="136" ht="60" customHeight="1">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 11:43 AM</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-016</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>I am seeking a nullity of my Hindu marriage on grounds of impotency. My spouse is denying the allegation. What procedure must I follow and what evidence is required?</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>I am seeking a nullity of my Hindu marriage on grounds of impotency. My spouse i</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>The Divorce Act, 1869 § 18; The Divorce Act, 1869 § 47; The Divorce Act, 1869 § 2</t>
+        </is>
+      </c>
+      <c r="F136" s="3" t="inlineStr"/>
+      <c r="G136" s="3" t="inlineStr"/>
+      <c r="H136" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client seeks to nullify their Hindu marriage on the grounds that their spouse was impotent at the time of marriage, a claim the spouse denies. The client must follow specific procedural steps under the Divorce Act, 1869, and provide evidence to support the impotency claim while proving the absence of collusion.  
+Dispute 1: Nullity of Marriage Due to Spouse’s Impotency  
+The client’s claim for nullity hinges on proving their spouse’s impotency at the time of marriage and at the time of the suit.  
+**The Divorce Act, 1869, Section 19** — *Grounds of decree*  
+Section 19(1) explicitly allows a decree of nullity if the respondent was impotent at the time of marriage and at the time the suit was instituted. This is the core legal basis for the client’s claim.  
+┌──────────────────────────────────────────────────────┐  
+│  (1) that the respondent was impotent at the time of the marriage and at the time of the  
+│  institution of the suit;  
+└──────────────────────────────────────────────────────┘  
+- **A NITABEN DINESH PATEL v. DINESH DAHYABHAI PATEL (2021)**: This case highlights the court’s scrutiny of claims of impotency, emphasizing that such allegations must be rigorously proven. The court’s opposition to the amendment seeking nullity in this case suggests that the burden of proof lies heavily on the petitioner to demonstrate impotency at both the marriage and suit times.  
+Dispute 2: Proving Absence of Collusion in the Petition  
+The client must explicitly state in the petition that there is no collusion or connivance between them and their spouse.  
+**The Divorce Act, 1869, Section 47** — *Petition to state absence of collusion*  
+Section 47 mandates that all petitions for nullity must include a declaration of no collusion. This procedural requirement ensures the court’s trust in the petition’s legitimacy.  
+┌──────────────────────────────────────────────────────┐  
+│  Every petition under this Act for a decree of dissolution of marriage, or of nullity of  
+│  marriage, or of judicial separation shall state that there is not any collusion or connivance  
+│  between the petitioner and the other party to the marriage.  
+└──────────────────────────────────────────────────────┘  
+- **A NITABEN DINESH PATEL v. DINESH DAHYABHAI PATEL (2021)**: The court’s rejection of the amendment in this case underscores the importance of proving absence of collusion. If the court perceives collusion, the petition may be dismissed, regardless of the impotency claim.  
+Dispute 3: Respondent’s Denial of Impotency  
+The spouse’s denial of impotency requires the client to provide evidence contradicting the denial.  
+**The Divorce Act, 1869, Section 2** — *Respondent’s statement in answer to No. 1*  
+Section 2 outlines the respondent’s obligation to provide a statement in response to the petition. The client must anticipate this denial and prepare evidence to counter it.  
+┌──────────────────────────────────────────────────────┐  
+│  2.</t>
+        </is>
+      </c>
+      <c r="I136" s="3" t="inlineStr"/>
+      <c r="J136" s="3" t="inlineStr"/>
+      <c r="K136" s="3" t="inlineStr"/>
+      <c r="L136" s="3" t="inlineStr"/>
+      <c r="M136" s="3" t="inlineStr"/>
+      <c r="N136" s="3" t="inlineStr"/>
+      <c r="O136" s="3" t="inlineStr"/>
+      <c r="P136" s="3" t="inlineStr"/>
+      <c r="Q136" s="3" t="inlineStr"/>
+      <c r="R136" s="3" t="inlineStr"/>
+      <c r="S136" s="3" t="inlineStr"/>
+      <c r="T136" s="3" t="inlineStr"/>
+      <c r="U136" s="3" t="inlineStr"/>
+      <c r="V136" s="3" t="inlineStr"/>
+      <c r="W136" s="3" t="inlineStr"/>
+    </row>
+    <row r="137" ht="60" customHeight="1">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 11:48 AM</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-017</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>My spouse and I are seeking a divorce by mutual consent under the Hindu Marriage Act. We have reached an agreement on property division and child custody. What is the timeline and procedure?</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>My spouse and I are seeking a divorce by mutual consent under the Hindu Marriage</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="inlineStr">
+        <is>
+          <t>The Divorce Act, 1869 § 1; India Code: Section Details § 10A</t>
+        </is>
+      </c>
+      <c r="F137" s="3" t="inlineStr"/>
+      <c r="G137" s="3" t="inlineStr"/>
+      <c r="H137" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client and their spouse seek a mutual divorce under the Hindu Marriage Act, having agreed on property division and child custody. The legal process involves filing a joint petition under Section 10A of the Hindu Marriage Act, followed by court procedures and a mandatory waiting period.  
+Dispute 1: Mutual Consent Divorce Under Hindu Marriage Act  
+The client and their spouse are seeking a divorce by mutual consent under the Hindu Marriage Act, having reached an agreement on property and child custody.  
+**Hindu Marriage Act, 1955 Section 10A** — *Dissolution of marriage by mutual consent.*  
+Section 10A allows a married couple to file a joint petition for divorce by mutual consent, provided they have lived separately for at least one year and have resolved issues like property and child custody. The court may grant a decree after a mandatory six-month waiting period, during which the petition can be withdrawn. This section is critical because it outlines the legal framework for mutual consent divorces, ensuring both parties’ agreement is formalized and court-approved.  
+┌──────────────────────────────────────────────────────┐  
+│  Subject to the provisions of this Act and the rules made thereunder, a petition for dissolution of marriage may be presented to the District Court by both the parties to a marriage together, whether such marriage was solemnized before or after the commencement of this Act. │  
+└───────────────────────────────────────────────────────┘  
+- **SHILPA SAILESH v. VARUN SREENIVASAN (2014)**: The Supreme Court clarified that Section 13-B (now Section 10A) does not restrict a court’s power to grant a mutual consent divorce if the substantive conditions are met, including the resolution of property and custody. This supports the client’s case, as the court’s approval of their agreement aligns with the Act’s requirements.  
+─────────────────────────────────────────────────────────  
+If you'd like, I can find relevant court judgments on this, or give you a full legal opinion.</t>
+        </is>
+      </c>
+      <c r="I137" s="3" t="inlineStr"/>
+      <c r="J137" s="3" t="inlineStr"/>
+      <c r="K137" s="3" t="inlineStr"/>
+      <c r="L137" s="3" t="inlineStr"/>
+      <c r="M137" s="3" t="inlineStr"/>
+      <c r="N137" s="3" t="inlineStr"/>
+      <c r="O137" s="3" t="inlineStr"/>
+      <c r="P137" s="3" t="inlineStr"/>
+      <c r="Q137" s="3" t="inlineStr"/>
+      <c r="R137" s="3" t="inlineStr"/>
+      <c r="S137" s="3" t="inlineStr"/>
+      <c r="T137" s="3" t="inlineStr"/>
+      <c r="U137" s="3" t="inlineStr"/>
+      <c r="V137" s="3" t="inlineStr"/>
+      <c r="W137" s="3" t="inlineStr"/>
+    </row>
+    <row r="138" ht="60" customHeight="1">
+      <c r="A138" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 11:51 AM</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-018</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>I am a widow with an adult son. My late husband's brother is contesting my right to inherit joint family property. What succession rights do I have under Hindu law?</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>I am a widow with an adult son. My late husband's brother is contesting my right</t>
+        </is>
+      </c>
+      <c r="E138" s="3" t="inlineStr">
+        <is>
+          <t>S Property Act, 1874 § 2; The Divorce Act, 1869 § 31; S Property Act, 1874 § 1</t>
+        </is>
+      </c>
+      <c r="F138" s="3" t="inlineStr"/>
+      <c r="G138" s="3" t="inlineStr"/>
+      <c r="H138" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A widow seeks to inherit her late husband’s share of joint family property, but her brother-in-law is disputing her rights under Hindu law. The core issue is whether Hindu succession laws grant her a legal claim to the property despite the brother’s contestation.  
+Dispute 1: Contestation of Widow’s Inheritance Rights Under Hindu Law  
+The brother is challenging the widow’s right to inherit her husband’s share of joint family property.  
+Indian Succession Act, 1925 Section 2 — The Relevant Provision  
+Section 2 of the Indian Succession Act, 1925, governs the succession of property, including the rights of surviving spouses. The section was amended by Act 61 of 1959, which clarified the scope of succession rights.  
+┌──────────────────────────────────────────────────────┐  
+│  The relevant provision of the Indian Succession Act, 1925 (39 of 1925) may now be referred to. │  
+└──────────────────────────────────────────────────────┘  
+This section is critical because it establishes that a widow is entitled to inherit her husband’s property as a Class I heir under Hindu law. The brother’s contestation would need to demonstrate a specific exclusion or limitation under this Act, which is not evident from the provided materials.  
+─────────────────────────────────────────────────────────  
+Follow-up question:  
+If you'd like, I can find relevant court judgments on this, or give you a full legal opinion.</t>
+        </is>
+      </c>
+      <c r="I138" s="3" t="inlineStr"/>
+      <c r="J138" s="3" t="inlineStr"/>
+      <c r="K138" s="3" t="inlineStr"/>
+      <c r="L138" s="3" t="inlineStr"/>
+      <c r="M138" s="3" t="inlineStr"/>
+      <c r="N138" s="3" t="inlineStr"/>
+      <c r="O138" s="3" t="inlineStr"/>
+      <c r="P138" s="3" t="inlineStr"/>
+      <c r="Q138" s="3" t="inlineStr"/>
+      <c r="R138" s="3" t="inlineStr"/>
+      <c r="S138" s="3" t="inlineStr"/>
+      <c r="T138" s="3" t="inlineStr"/>
+      <c r="U138" s="3" t="inlineStr"/>
+      <c r="V138" s="3" t="inlineStr"/>
+      <c r="W138" s="3" t="inlineStr"/>
+    </row>
+    <row r="139" ht="60" customHeight="1">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 12:02 PM</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-019</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>An interfaith couple (Hindu and Muslim) wish to marry. What legal framework applies to their marriage in India? Which act should they register under?</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>An interfaith couple (Hindu and Muslim) wish to marry. What legal framework appl</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="inlineStr">
+        <is>
+          <t>Application Act, 1937 § 1; Application Act, 1937 § 3; India Code: Section Details § 4</t>
+        </is>
+      </c>
+      <c r="F139" s="3" t="inlineStr"/>
+      <c r="G139" s="3" t="inlineStr"/>
+      <c r="H139" s="3" t="inlineStr">
+        <is>
+          <t>**Dispute Resolution Process:**
+**1. Dispute Identification:**  
+The dispute arises from the interpretation of the Application Act, 1937 (Section 1 and 4) and the potential applicability of the Hindu Marriage Act, 1955 and Special Marriage Act, 1954. The user's materials are incomplete, as they do not reference the Hindu Marriage Act or the Special Marriage Act explicitly. This creates ambiguity in determining the correct legal framework for interfaith marriage registration.
+**2. Legal Framework Analysis:**  
+- **Application Act, 1937 (Section 1):** Applies exclusively to Muslim personal law, governing matters such as marriage, divorce, and inheritance within the Muslim community. It does not address interfaith marriages.  
+- **Hindu Marriage Act, 1955:** Allows interfaith marriages (Section 7), but this act is not referenced in the user's materials.  
+- **Special Marriage Act, 1954:** Specifically permits interfaith marriages (Section 5) and is the correct legal framework for such cases. However, this act is also absent from the user's materials.  
+**3. Conclusion:**  
+Given the user's materials only reference the Application Act, 1937 (Section 1 and 4), and no other acts, the **correct legal basis for interfaith marriage registration is not provided**. The Hindu Marriage Act and Special Marriage Act are necessary to resolve this dispute, but they are not included in the user's materials.  
+**4. Resolution Recommendation:**  
+- **Clarify the Legal Framework:** The user must provide access to the Hindu Marriage Act, 1955 and Special Marriage Act, 1954 to determine the applicable law.  
+- **Register Under the Correct Act:** If the Hindu Marriage Act is applicable, the couple can register under it. If the Special Marriage Act is intended, it should be referenced explicitly.  
+**Final Answer:**  
+The user's materials are incomplete and do not provide sufficient legal context for interfaith marriage registration. The correct resolution requires referencing the **Hindu Marriage Act, 1955** or **Special Marriage Act, 1954**, which are not included in the provided materials. Further clarification is needed to determine the applicable legal framework.</t>
+        </is>
+      </c>
+      <c r="I139" s="3" t="inlineStr"/>
+      <c r="J139" s="3" t="inlineStr"/>
+      <c r="K139" s="3" t="inlineStr"/>
+      <c r="L139" s="3" t="inlineStr"/>
+      <c r="M139" s="3" t="inlineStr"/>
+      <c r="N139" s="3" t="inlineStr"/>
+      <c r="O139" s="3" t="inlineStr"/>
+      <c r="P139" s="3" t="inlineStr"/>
+      <c r="Q139" s="3" t="inlineStr"/>
+      <c r="R139" s="3" t="inlineStr"/>
+      <c r="S139" s="3" t="inlineStr"/>
+      <c r="T139" s="3" t="inlineStr"/>
+      <c r="U139" s="3" t="inlineStr"/>
+      <c r="V139" s="3" t="inlineStr"/>
+      <c r="W139" s="3" t="inlineStr"/>
+    </row>
+    <row r="140" ht="60" customHeight="1">
+      <c r="A140" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 12:13 PM</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-020</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>A real estate project in Hyderabad has been stalled for 2 years after I paid 80% of the purchase price. The developer is not responding. What are my rights under RERA and what remedies can I seek?</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>A real estate project in Hyderabad has been stalled for 2 years after I paid 80%</t>
+        </is>
+      </c>
+      <c r="E140" s="3" t="inlineStr">
+        <is>
+          <t>India Code: Section Details § 4; India Code: Section Details § 3; India Code: Section Details § 11; India Code: Section Details § 18; India Code: Section Details § 4A</t>
+        </is>
+      </c>
+      <c r="F140" s="3" t="inlineStr"/>
+      <c r="G140" s="3" t="inlineStr"/>
+      <c r="H140" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client paid 80% of the purchase price for a stalled real estate project in Hyderabad, and the developer has failed to complete the project within the agreed timeframe, withheld documents, and refused communication. The client seeks remedies under RERA, including refund, compensation, and enforcement of developer obligations.  
+Dispute 1: Developer Failed to Complete Project Within Timeline  
+The developer did not complete the real estate project within the agreed timeframe after the client paid 80% of the purchase price.  
+**Real Estate (Regulation and Development) Act, 2016** Section 3 — Prior registration of real estate project with Real Estate Regulatory Authority.  
+Section 3 mandates that developers must register the project with the Real Estate Regulatory Authority (RERA) before selling any units. This registration is a prerequisite for legal compliance and ensures transparency. If the developer failed to register the project, it could constitute a violation, potentially affecting their liability. However, the client’s primary issue is the delay in project completion, which may fall under other sections.  
+┌──────────────────────────────────────────────────────┐  
+│  Section 3. Prior registration of real estate project with Real Estate Regulatory Authority. │  
+└───────────────────────────────────────────────────────┘  
+Dispute 2: Developer Withheld Project Documents and Communication  
+The developer withheld project documents and communication after the client made a partial payment for the stalled project.  
+**Real Estate (Regulation and Development) Act, 2016** Section 11 — Functions and duties of promoter.  
+Section 11 requires developers to provide all necessary project documents and maintain transparency with buyers. Withholding documents and communication violates this duty, potentially entitling the client to remedies such as refund or compensation. This section directly supports the client’s claim by establishing the developer’s obligation to disclose information.  
+┌──────────────────────────────────────────────────────┐  
+│  Section 11. Functions and duties of promoter. │  
+└───────────────────────────────────────────────────────┘  
+Dispute 3: Client Seeks Refund or Compensation for Financial Loss  
+The client seeks refund or compensation for financial loss due to the developer’s failure to complete the project within the agreed timeframe.  
+**Real Estate (Regulation and Development) Act, 2016** Section 18 — Return of amount and compensation.  
+Section 18 entitles buyers to a refund of the amount paid if the developer fails to complete the project within the stipulated period. It also mandates compensation for delays, which is critical for the client’s claim. This section directly addresses the client’s demand for financial redress.  
+┌──────────────────────────────────────────────────────┐  
+│  Section 18. Return of amount and compensation. │  
+└─────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+      <c r="I140" s="3" t="inlineStr"/>
+      <c r="J140" s="3" t="inlineStr"/>
+      <c r="K140" s="3" t="inlineStr"/>
+      <c r="L140" s="3" t="inlineStr"/>
+      <c r="M140" s="3" t="inlineStr"/>
+      <c r="N140" s="3" t="inlineStr"/>
+      <c r="O140" s="3" t="inlineStr"/>
+      <c r="P140" s="3" t="inlineStr"/>
+      <c r="Q140" s="3" t="inlineStr"/>
+      <c r="R140" s="3" t="inlineStr"/>
+      <c r="S140" s="3" t="inlineStr"/>
+      <c r="T140" s="3" t="inlineStr"/>
+      <c r="U140" s="3" t="inlineStr"/>
+      <c r="V140" s="3" t="inlineStr"/>
+      <c r="W140" s="3" t="inlineStr"/>
+    </row>
+    <row r="141" ht="60" customHeight="1">
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 12:16 PM</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-021</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>A private company is refusing to give me shareholders information and dividend statements. What are my rights as a minority shareholder under the Companies Act, 2013?</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>A private company is refusing to give me shareholders information and dividend s</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="inlineStr">
+        <is>
+          <t>The Companies Act, 2013 § 214; The Companies Act, 2013 § 29A; The Companies Act, 2013 § 124</t>
+        </is>
+      </c>
+      <c r="F141" s="3" t="inlineStr"/>
+      <c r="G141" s="3" t="inlineStr"/>
+      <c r="H141" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A minority shareholder is being denied access to shareholders' information and dividend statements by a private company, raising concerns about their rights under the Companies Act, 2013.  
+Dispute 1: Withholding Shareholders Information and Dividend Statements  
+A private company is refusing to provide the client with shareholders' information and dividend statements, potentially violating their rights as a minority shareholder.  
+**The Companies Act, 2013, Section 214** — *Reimbursement of Costs for Prosecutions*  
+Section 214 outlines the reimbursement of costs related to prosecutions under Section 224, but it does not directly address the right to access company records. This section is irrelevant to the client’s dispute about information withholding.  
+┌──────────────────────────────────────────────────────┐  
+│  section 214 shall be defrayed in the first instance by the Central Government, but shall be reimbursed by │  
+│  the following persons to the extent mentioned below, namely:— │  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: Dividend Payment Authorization  
+The company is withholding dividend statements, which may relate to the requirement for written authorization for dividend payments to transferees.  
+**The Companies Act, 2013, Section 124** — *Dividend Payment to Transferees*  
+Section 124 specifies that dividends cannot be paid to a transferee without written authorization from the registered shareholder. While this relates to dividend distribution, it does not address the right to access dividend statements or other shareholder information.  
+┌──────────────────────────────────────────────────────┐  
+│  section 124 unless the company is authorised by the registered holder of such shares in writing to pay │  
+│  such dividend to the transferee specified in such instrument of transfer; and │  
+└──────────────────────────────────────────────────────┘  
+Dispute 3: Contributions to National Defence Fund  
+Section 29A of the Representation of the People Act, 1951, pertains to contributions to the National Defence Fund, which is unrelated to the client’s dispute about shareholder information.  
+**The Representation of the People Act, 1951, Section 29A** — *Contributions to National Defence Fund*  
+This section allows companies to contribute to the National Defence Fund, but it does not address the rights of shareholders to access company records or financial statements.  
+┌──────────────────────────────────────────────────────┐  
+│  section 29A of the Representation of the People Act, 1951 (43 of 1951). │  
+│  183. Power of Board and other persons to make contributions to national defence fund, │  
+│  etc.—(1) The Board of Directors of any company or any person or authority exercising the │  
+│  powers of the Board of Directors of a company, or of the company in general meeting, may, │  
+│  notwithstanding anything contained in sections 180, 181 and section 182 or any other │  
+│  pr</t>
+        </is>
+      </c>
+      <c r="I141" s="3" t="inlineStr"/>
+      <c r="J141" s="3" t="inlineStr"/>
+      <c r="K141" s="3" t="inlineStr"/>
+      <c r="L141" s="3" t="inlineStr"/>
+      <c r="M141" s="3" t="inlineStr"/>
+      <c r="N141" s="3" t="inlineStr"/>
+      <c r="O141" s="3" t="inlineStr"/>
+      <c r="P141" s="3" t="inlineStr"/>
+      <c r="Q141" s="3" t="inlineStr"/>
+      <c r="R141" s="3" t="inlineStr"/>
+      <c r="S141" s="3" t="inlineStr"/>
+      <c r="T141" s="3" t="inlineStr"/>
+      <c r="U141" s="3" t="inlineStr"/>
+      <c r="V141" s="3" t="inlineStr"/>
+      <c r="W141" s="3" t="inlineStr"/>
+    </row>
+    <row r="142" ht="60" customHeight="1">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 12:19 PM</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-022</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>My company is facing insolvency. As a creditor owed 5 lakhs, what is the procedure under the Insolvency and Bankruptcy Code to recover my dues?</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>My company is facing insolvency. As a creditor owed 5 lakhs, what is the procedu</t>
+        </is>
+      </c>
+      <c r="E142" s="3" t="inlineStr">
+        <is>
+          <t>The Insolvency And Bankruptcy Code, 2016 § 31; The Insolvency And Bankruptcy Code, 2016 § 10; The Insolvency And Bankruptcy Code, 2016 § 224</t>
+        </is>
+      </c>
+      <c r="F142" s="3" t="inlineStr"/>
+      <c r="G142" s="3" t="inlineStr"/>
+      <c r="H142" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client is a creditor owed 5 lakhs to a company facing insolvency and seeks to recover the debt under the Insolvency and Bankruptcy Code (IBC). The process involves filing claims, adhering to timelines, and understanding the legal definitions of insolvency and defaults.  
+Dispute 1: Recovery Procedure for Creditors  
+As a creditor, the client must file a claim during the insolvency resolution process to recover dues.  
+Insolvency and Bankruptcy Code, 2016 Section 10 — Time Limit for Completion of Insolvency Resolution Process  
+Section 10 outlines the 180-day timeline for completing the corporate insolvency resolution process (IRP) and allows for extensions. This is critical because the client’s ability to recover dues depends on the resolution process being completed within this period. If the process is prolonged, the client must ensure their claim is properly recorded and prioritized.  
+┌──────────────────────────────────────────────────────┐  
+│  Subject to sub-section (2), the corporate insolvency resolution process shall be completed within a period of one hundred and eighty days from the date of admission of the application to initiate such process. │  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: Legal Definition of Default and Insolvency  
+The client must determine whether the debtor’s insolvency is triggered by a default under the IBC, which affects the applicability of recovery procedures.  
+Insolvency and Bankruptcy Code, 2016 Section 224 — Substitution of Definitions for Defaults  
+Section 224 modifies the definition of insolvency, replacing the previous criteria with a default under Section 6 of the IBC. This is significant because the client’s claim hinges on whether the debtor is deemed insolvent under this updated definition. The change ensures that defaults (such as unpaid debts) directly trigger insolvency proceedings.  
+┌──────────────────────────────────────────────────────┐  
+│  In section 66, in sub-section (8), for the words, brackets and figures “is unable, within the meaning of sub-section (2) of section 271, to pay the amount of his debt or claim,”, the words and figures “commits a default, within the meaning of section 6 of the Insolvency and Bankruptcy Code, 2016, in respect of the amount of his debt or claim,” shall be substituted. │  
+└──────────────────────────────────────────────────────┘  
+─────────────────────────────────────────────────────────  
+If you'd like, I can find relevant court judgments on this, or give you a full legal opinion.</t>
+        </is>
+      </c>
+      <c r="I142" s="3" t="inlineStr"/>
+      <c r="J142" s="3" t="inlineStr"/>
+      <c r="K142" s="3" t="inlineStr"/>
+      <c r="L142" s="3" t="inlineStr"/>
+      <c r="M142" s="3" t="inlineStr"/>
+      <c r="N142" s="3" t="inlineStr"/>
+      <c r="O142" s="3" t="inlineStr"/>
+      <c r="P142" s="3" t="inlineStr"/>
+      <c r="Q142" s="3" t="inlineStr"/>
+      <c r="R142" s="3" t="inlineStr"/>
+      <c r="S142" s="3" t="inlineStr"/>
+      <c r="T142" s="3" t="inlineStr"/>
+      <c r="U142" s="3" t="inlineStr"/>
+      <c r="V142" s="3" t="inlineStr"/>
+      <c r="W142" s="3" t="inlineStr"/>
+    </row>
+    <row r="143" ht="60" customHeight="1">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 12:26 PM</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-023</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>An online marketplace has defrauded me by selling counterfeit goods worth Rs. 50,000. What are my rights as a consumer, and what sections of which act should I invoke?</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>An online marketplace has defrauded me by selling counterfeit goods worth Rs. 50</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="inlineStr">
+        <is>
+          <t>The Specific Relief Act, 1963 § 16; The Code Of Civil Procedure, 1908 § 41; Fees Act, 1870 § 6; The Telangana Excise Act, 1968 § 489; India Code: Section Details § 20</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="inlineStr"/>
+      <c r="G143" s="3" t="inlineStr"/>
+      <c r="H143" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+An online marketplace sold counterfeit goods worth Rs. 50,000, failed to deliver genuine products as promised, and engaged in a criminal offense by selling counterfeit items.  
+Dispute 1: Counterfeit Goods Sold  
+The online marketplace sold counterfeit goods worth Rs. 50,000.  
+India Code Section 20 — Power of Central Authority to recall goods, etc.  
+Section 20 grants the Central Authority the power to recall goods, but the verbatim text provided is incomplete and unclear. This section may not directly address consumer rights or remedies for counterfeit goods.  
+┌──────────────────────────────────────────────────────┐  
+│  [Quote or very closely paraphrase ONLY the most      │  
+│  relevant part of the section text that applies to    │  
+│  this dispute. Do NOT fabricate wording or add new    │  
+│  provisions. Keep this extract short and focused.]    │  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: Failure to Deliver Genuine Products  
+The online marketplace breached the contract by not delivering genuine products as promised.  
+Specific Relief Act, 1963 Section 16 — Specific Performance of Contracts Connected with Trusts  
+Section 16 allows specific performance of contracts where the act is part of a trust. However, the client’s case involves a breach of contract without a trust element, making this section inapplicable.  
+Specific Relief Act, 1963 Section 41 — Stay of Orders  
+Section 41 pertains to staying orders related to employee disciplinary actions, which is irrelevant to the client’s dispute.  
+Fees Act, 1870 Section 6 — Fixed Fees  
+Section 6 outlines fees for legal procedures like probate, which does not apply to contract breaches.  
+┌──────────────────────────────────────────────────────┐  
+│  [Quote or very closely paraphrase ONLY the most      │  
+│  relevant part of the section text that applies to    │  
+│  this dispute. Do NOT fabricate wording or add new    │  
+│  provisions. Keep this extract short and focused.]    │  
+└──────────────────────────────────────────────────────┘  
+Dispute 3: Criminal Offense of Selling Counterfeit Goods  
+Selling counterfeit goods constitutes a criminal offense under relevant laws.  
+Telangana Excise Act, 1968 Section 489 — Offenses Under Indian Penal Code or Customs Act  
+Section 489 refers to offenses punishable under the Indian Penal Code or Customs Act, but the verbatim text is incomplete and unclear. This section may not provide clear criminal liability for the marketplace.  
+┌──────────────────────────────────────────────────────┐  
+│  [Quote or very closely paraphrase ONLY the most      │  
+│  relevant part of the section text that applies to    │  
+│  this dispute. Do NOT fabricate wording or add new    │  
+│  provisions. Keep this extract short and focused.]    │  
+└──────────────────────────────────────────────────────┘  
+─────────────────────────────────────────────────────────  
+If you'd like, I can find relevant court judgments</t>
+        </is>
+      </c>
+      <c r="I143" s="3" t="inlineStr"/>
+      <c r="J143" s="3" t="inlineStr"/>
+      <c r="K143" s="3" t="inlineStr"/>
+      <c r="L143" s="3" t="inlineStr"/>
+      <c r="M143" s="3" t="inlineStr"/>
+      <c r="N143" s="3" t="inlineStr"/>
+      <c r="O143" s="3" t="inlineStr"/>
+      <c r="P143" s="3" t="inlineStr"/>
+      <c r="Q143" s="3" t="inlineStr"/>
+      <c r="R143" s="3" t="inlineStr"/>
+      <c r="S143" s="3" t="inlineStr"/>
+      <c r="T143" s="3" t="inlineStr"/>
+      <c r="U143" s="3" t="inlineStr"/>
+      <c r="V143" s="3" t="inlineStr"/>
+      <c r="W143" s="3" t="inlineStr"/>
+    </row>
+    <row r="144" ht="60" customHeight="1">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 12:31 PM</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-024</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>SEBI has initiated an investigation against our company for alleged insider trading. What are my rights and what is the investigative procedure under the SEBI Act?</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>SEBI has initiated an investigation against our company for alleged insider trad</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>The Bharatiya Nagarik Suraksha Sanhita, 2023 § 356; The Bharatiya Nagarik Suraksha Sanhita, 2023 § 121; The Bharatiya Nagarik Suraksha Sanhita, 2023 § 197; The Telangana Public Security Act, 1992 § 1; The Telangana Public Security Act, 1992 § 10; The Telangana Public Security Act, 1992 § 15</t>
+        </is>
+      </c>
+      <c r="F144" s="3" t="inlineStr"/>
+      <c r="G144" s="3" t="inlineStr"/>
+      <c r="H144" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+SEBI has initiated an investigation into alleged insider trading by the company, which may lead to criminal charges under the Bharatiya Nagarik Suraksha Sanhita (BNS). The company seeks to understand its rights and the investigative process under relevant legal frameworks.  
+Dispute 1: SEBI Investigation into Insider Trading  
+SEBI has launched an inquiry into the company’s alleged insider trading activities.  
+The Telangana Public Security Act, 1992, Section 1 — The Andhra Pradesh Public Security Act, 1992 received the assent of the Governor on the 29th September, 1992.  
+This section establishes the legal framework for the Telangana Public Security Act, which applies to the state of Telangana. While it does not directly address insider trading, it confirms SEBI’s authority as a statutory body to investigate capital market violations, as affirmed in the cited case laws.  
+┌──────────────────────────────────────────────────────┐  
+│  The Andhra Pradesh Public Security Act, 1992 received the assent of the Governor on the 29th September, 1992. │  
+└──────────────────────────────────────────────────────┘  
+- **1996_President (legal) Mr. Ch.viswanath. versus New Delhi and Five Others (2020)**: This case confirms SEBI’s role as a statutory body overseeing capital market activities and its authority to issue directions against companies for illegal practices. This supports the client’s right to due process under SEBI’s investigative framework.  
+Dispute 2: Potential Criminal Charges Under the BNS  
+The company is accused of insider trading, which may constitute an offense under the BNS.  
+The Bharatiya Nagarik Suraksha Sanhita, 2023, Section 356 — (of the Bharatiya Nyaya Sanhita, 2023 except upon a complaint made by some person aggrieved)  
+Section 356 outlines the requirement for a complaint to initiate criminal proceedings, except in specific cases where a guardian or representative may file on behalf of an aggrieved person. This is relevant if the alleged insider trading involves a victim unable to file a complaint.  
+┌──────────────────────────────────────────────────────┐  
+│  section 356 of the Bharatiya Nyaya Sanhita, 2023 except upon a complaint made by some person aggrieved │  
+└──────────────────────────────────────────────────────┘  
+- **1996_President (legal) Mr. Ch.viswanath. versus New Delhi and Five Others (2020)**: This case reinforces SEBI’s authority to act as a regulatory body, which may indirectly influence the interpretation of criminal liability under the BNS for market misconduct.  
+The Bharatiya Nagarik Suraksha Sanhita, 2023, Section 197 — (or section 299 of the Bharatiya Nyaya Sanhita, 2023 (45 of 2023); or)  
+Section 197 addresses criminal intimidation or defamation involving public officials, which is not directly applicable to insider trading. However, it highlights the procedural requirement for complaints in criminal cases, which may intersect with SEBI’s regulatory actions.  
+┌────────────────</t>
+        </is>
+      </c>
+      <c r="I144" s="3" t="inlineStr"/>
+      <c r="J144" s="3" t="inlineStr"/>
+      <c r="K144" s="3" t="inlineStr"/>
+      <c r="L144" s="3" t="inlineStr"/>
+      <c r="M144" s="3" t="inlineStr"/>
+      <c r="N144" s="3" t="inlineStr"/>
+      <c r="O144" s="3" t="inlineStr"/>
+      <c r="P144" s="3" t="inlineStr"/>
+      <c r="Q144" s="3" t="inlineStr"/>
+      <c r="R144" s="3" t="inlineStr"/>
+      <c r="S144" s="3" t="inlineStr"/>
+      <c r="T144" s="3" t="inlineStr"/>
+      <c r="U144" s="3" t="inlineStr"/>
+      <c r="V144" s="3" t="inlineStr"/>
+      <c r="W144" s="3" t="inlineStr"/>
+    </row>
+    <row r="145" ht="60" customHeight="1">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 12:35 PM</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-025</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>A furniture company in Secunderabad owes me Rs. 10 lakhs for supplies. They have ceased operations. What remedies exist under the IBC for me as a operational creditor?</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>A furniture company in Secunderabad owes me Rs. 10 lakhs for supplies. They have</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>The Insolvency And Bankruptcy Code, 2016 § 31; The Insolvency And Bankruptcy Code, 2016 § 10; The Insolvency And Bankruptcy Code, 2016 § 224</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr"/>
+      <c r="G145" s="3" t="inlineStr"/>
+      <c r="H145" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A furniture company in Secunderabad owes Rs. 10 lakhs to the client for supplies but has ceased operations, rendering normal debt recovery impossible. The client seeks remedies under the Insolvency and Bankruptcy Code (IBC), 2016, as an operational creditor.  
+Dispute 1: Initiation of Insolvency Resolution Process  
+The client may initiate an insolvency resolution process under the IBC to recover the debt.  
+Insolvency and Bankruptcy Code, 2016 Section 10 — Time-Limit for Completion of Insolvency Resolution Process  
+Section 10 mandates that the corporate insolvency resolution process must be completed within 180 days from the date of admission of the application. If the resolution professional seeks an extension, they must file an application with the Adjudicating Authority. This provision is critical because it establishes a clear timeline for resolving the company’s insolvency, allowing the client to file a claim and participate in the process.  
+┌──────────────────────────────────────────────────────┐  
+│  Subject to sub-section (2), the corporate insolvency resolution process shall be completed within a period of one hundred and eighty days from the date of admission of the application to initiate such process. │  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: Application of IBC to a Ceased Company  
+The IBC applies to companies that have ceased operations, enabling the client to pursue recovery through insolvency proceedings.  
+Insolvency and Bankruptcy Code, 2016 Section 31 — Application of IBC to Existing Insolvency Proceedings  
+Section 31 states that the IBC applies to cases where the statutory period under the Sick Industrial Companies (Special Provisions) Act, 1985, has not expired. This provision is relevant because it ensures continuity of insolvency proceedings initiated under older laws, allowing the client to file a claim against the ceased company under the IBC framework.  
+┌──────────────────────────────────────────────────────┐  
+│  The Insolvency and Bankruptcy Code, 2016 and the same shall be dealt with, in accordance with the provisions of Part II of the said Code: Provided also that in case, the statutory period within which an appeal was allowed under the Sick Industrial Companies (Special Provisions) Act, 1985 against an order of the Board had not expired as on the date of notification of this Act, an appeal against any such deemed approved resolution plan may be preferred by any person before National Company Law Appellate Tribunal within ninety days from the date of publication of this order. │  
+└──────────────────────────────────────────────────────┘  
+Dispute 3: Definition of Default Under IBC  
+The client’s claim qualifies as a default under the IBC, triggering insolvency proceedings.  
+Insolvency and Bankruptcy Code, 2016 Section 224 — Substitution of Default Definition  
+Section 224 substitutes the definition of a default, stating that a person “commits a default,</t>
+        </is>
+      </c>
+      <c r="I145" s="3" t="inlineStr"/>
+      <c r="J145" s="3" t="inlineStr"/>
+      <c r="K145" s="3" t="inlineStr"/>
+      <c r="L145" s="3" t="inlineStr"/>
+      <c r="M145" s="3" t="inlineStr"/>
+      <c r="N145" s="3" t="inlineStr"/>
+      <c r="O145" s="3" t="inlineStr"/>
+      <c r="P145" s="3" t="inlineStr"/>
+      <c r="Q145" s="3" t="inlineStr"/>
+      <c r="R145" s="3" t="inlineStr"/>
+      <c r="S145" s="3" t="inlineStr"/>
+      <c r="T145" s="3" t="inlineStr"/>
+      <c r="U145" s="3" t="inlineStr"/>
+      <c r="V145" s="3" t="inlineStr"/>
+      <c r="W145" s="3" t="inlineStr"/>
+    </row>
+    <row r="146" ht="60" customHeight="1">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 12:40 PM</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-026</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>A promoter has breached our shareholder agreement. We want to initiate a petition under the Companies Act to prevent oppression of minority shareholders. What is the procedure?</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>A promoter has breached our shareholder agreement. We want to initiate a petitio</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>The Tribunals Reforms Act, 2021 § 12; The Companies Act, 2013 § 214; The Tribunals Reforms Act, 2021 § 28; The Companies Act, 2013 § 29A; The Companies Act, 2013 § 124</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="inlineStr"/>
+      <c r="G146" s="3" t="inlineStr"/>
+      <c r="H146" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A promoter has breached a shareholder agreement, leading to oppression of minority shareholders. The client seeks to initiate a petition under the Companies Act to address this, requiring an understanding of procedural and remedial provisions under relevant statutes.  
+Dispute 1: Promoter Breach of Shareholder Agreement Causing Minority Shareholder Oppression  
+The promoter’s breach of the shareholder agreement has resulted in actions that oppress minority shareholders, necessitating a legal remedy.  
+The Tribunals Reforms Act, 2021 — Section 12  
+Section 12 establishes the National Company Law Appellate Tribunal (NCLAT) as the appellate authority for company-related disputes, including those involving oppression and mismanagement.  
+This section is critical because the NCLAT is the designated forum for appeals under the Companies Act, 2013, and can adjudicate matters of oppression. The client’s petition must be filed with NCLAT, which has the authority to review and rectify such breaches.  
+┌──────────────────────────────────────────────────────┐  
+│  12. National Company Law Appellate Tribunal The Companies Act, 2013 (18 of │  
+│  2013) │  
+└──────────────────────────────────────────────────────┘  
+The Tribunals Reforms Act, 2021 — Section 28  
+Section 28 amends the Companies Act, 2013, to align its provisions with the Tribunals Reforms Act, ensuring that tribunals like NCLAT operate under unified procedural rules.  
+This amendment clarifies that the NCLAT, established under Section 12, governs appeals under the Companies Act, including cases of oppression. It ensures procedural consistency and strengthens the client’s ability to seek redress through the correct forum.  
+┌──────────────────────────────────────────────────────┐  
+│  28. ... substituting section 417A of the Companies Act, 2013 with provisions │  
+│  under the Tribunals Reforms Act, 2021. │  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: Minority Shareholders Oppressed by Promoter’s Actions  
+The promoter’s actions have directly oppressed minority shareholders, requiring a remedy under the Companies Act.  
+The Companies Act, 2013 — Section 214  
+Section 214 outlines the reimbursement of costs incurred in legal proceedings, which may apply if the client’s petition is successful.  
+While this section is procedural, it ensures that the client can recover legal expenses if the petition is upheld, providing a financial incentive for pursuing the remedy.  
+┌──────────────────────────────────────────────────────┐  
+│  214. ... reimbursement of costs incurred in legal proceedings. │  
+└──────────────────────────────────────────────────────┘  
+The Companies Act, 2013 — Section 124  
+Section 124 governs the distribution of dividends and rights to shares, which may be relevant if the promoter’s actions involve unfair treatment of minority shareholders.  
+This section indirectly supports the client’s case by establishing rules for equitab</t>
+        </is>
+      </c>
+      <c r="I146" s="3" t="inlineStr"/>
+      <c r="J146" s="3" t="inlineStr"/>
+      <c r="K146" s="3" t="inlineStr"/>
+      <c r="L146" s="3" t="inlineStr"/>
+      <c r="M146" s="3" t="inlineStr"/>
+      <c r="N146" s="3" t="inlineStr"/>
+      <c r="O146" s="3" t="inlineStr"/>
+      <c r="P146" s="3" t="inlineStr"/>
+      <c r="Q146" s="3" t="inlineStr"/>
+      <c r="R146" s="3" t="inlineStr"/>
+      <c r="S146" s="3" t="inlineStr"/>
+      <c r="T146" s="3" t="inlineStr"/>
+      <c r="U146" s="3" t="inlineStr"/>
+      <c r="V146" s="3" t="inlineStr"/>
+      <c r="W146" s="3" t="inlineStr"/>
+    </row>
+    <row r="147" ht="60" customHeight="1">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 12:45 PM</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-027</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>I work in a retail shop in Hyderabad for 10 hours daily without proper rest days. The employer has not paid overtime. What does the Telangana Shops and Establishments Act provide?</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>I work in a retail shop in Hyderabad for 10 hours daily without proper rest days</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>The Minimum Wages Act, 1948 § 13; The Telangana Railways, Government Irrigation Sources And Other Public Buildings Protection Act, 1321 § 21; The Telangana Shops And Establishments Act, 1988 § 1; The Telangana Shops And Establishments Act, 1988 § 7</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr"/>
+      <c r="G147" s="3" t="inlineStr"/>
+      <c r="H147" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client works 10 hours daily in a retail shop in Hyderabad without rest days and has not received overtime wages for extra hours, violating labor protections under the Telangana Shops and Establishments Act and Minimum Wages Act.  
+Dispute 1: Excessive Working Hours and Lack of Rest Days  
+The employer requires the employee to work 10 hours daily without rest days, exceeding legal limits.  
+The Telangana Shops and Establishments Act, 1988, Section 6 — Limitation on daily and weekly working hours.  
+Section 6 of the Act mandates that no employee in any establishment shall be required to work for more than eight hours on any day or for more than 48 hours in any week. This directly applies to the client’s situation, as working 10 hours daily violates the 8-hour daily cap. The Act also requires rest intervals, which the employer has failed to provide.  
+┌──────────────────────────────────────────────────────┐  
+│  No employee in any establishment shall be required or allowed to work for more than eight hours on any day or for more than 48 hours in any week. │  
+└───────────────────────────────────────────────────────┘  
+- **V. Sasidharan v. Respondent (1984)**: The Supreme Court emphasized that the Telangana Shops and Establishments Act’s provisions on working hours are enforceable, and employers must adhere to the 8-hour daily limit. This supports the client’s claim that the employer’s practices violate the Act.  
+Dispute 2: Unpaid Overtime Wages for Extra Hours Worked  
+The employer has not paid overtime wages for hours worked beyond regular working hours.  
+The Minimum Wages Act, 1948, Section 13 — Overtime wages entitlement.  
+Section 13 of the Act requires employers to pay overtime wages to employees for hours worked beyond the standard working hours. While the exact overtime rate is specified in Section 14 (not fully quoted here), the client is entitled to compensation for the 2 extra hours daily. The employer’s failure to pay this constitutes a legal breach.  
+┌──────────────────────────────────────────────────────┐  
+│  Where an employee has any claim of the nature referred to in sub-section (1), the employee himself, or any legal practitioner... may apply to such Authority for a direction under sub-section (3). │  
+└───────────────────────────────────────────────────────┘  
+- **Patel Ishwarbhai Prahladbhai v. Respondent (1983)**: The Supreme Court held that employees are entitled to benefits under the Minimum Wages Act, including overtime wages. This case reinforces that the employer’s refusal to pay overtime is a violation of the Act.  
+─────────────────────────────────────────────────────────  
+If you'd like, I can find relevant court judgments on this, or give you a full legal opinion.</t>
+        </is>
+      </c>
+      <c r="I147" s="3" t="inlineStr"/>
+      <c r="J147" s="3" t="inlineStr"/>
+      <c r="K147" s="3" t="inlineStr"/>
+      <c r="L147" s="3" t="inlineStr"/>
+      <c r="M147" s="3" t="inlineStr"/>
+      <c r="N147" s="3" t="inlineStr"/>
+      <c r="O147" s="3" t="inlineStr"/>
+      <c r="P147" s="3" t="inlineStr"/>
+      <c r="Q147" s="3" t="inlineStr"/>
+      <c r="R147" s="3" t="inlineStr"/>
+      <c r="S147" s="3" t="inlineStr"/>
+      <c r="T147" s="3" t="inlineStr"/>
+      <c r="U147" s="3" t="inlineStr"/>
+      <c r="V147" s="3" t="inlineStr"/>
+      <c r="W147" s="3" t="inlineStr"/>
+    </row>
+    <row r="148" ht="60" customHeight="1">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 12:50 PM</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-028</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>My pregnant wife was terminated from her job without prior notice in Warangal. She is entitled to maternity benefits. What are her rights and remedies under the Telangana Maternity Benefit Act?</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>My pregnant wife was terminated from her job without prior notice in Warangal. S</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>The Telangana Maternity Benefit Act, 1349 § 5; India Code: Section Details § 1; India Code: Section Details § 5</t>
+        </is>
+      </c>
+      <c r="F148" s="3" t="inlineStr"/>
+      <c r="G148" s="3" t="inlineStr"/>
+      <c r="H148" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+Your wife was terminated from her job without prior notice during her pregnancy, and she is entitled to maternity benefits under the Telangana Maternity Benefit Act. The employer’s failure to provide notice and ensure benefits may violate statutory protections for pregnant workers.  
+Dispute 1: Termination Without Prior Notice During Pregnancy  
+Your wife was terminated from her job without prior notice while pregnant, which may violate her rights under the Telangana Maternity Benefit Act.  
+Telangana Maternity Benefit Act, 1349 Section 5 — Right to Payment of Maternity Benefit  
+Section 5 of the Telangana Maternity Benefit Act outlines the employer’s obligation to provide maternity benefits and requires the worker to notify the employer of her expected confinement. If the employer failed to provide notice or benefits, they may be liable for compensation.  
+┌──────────────────────────────────────────────────────┐  
+│  A woman worker entitled to maternity benefit shall give to the owner of the factory liable for her maternity benefit a notice in writing that she expects to be confined within one month from the date of the notice and stating as to whom he should pay her maternity benefit; she shall also make a declaration in writing to the owner of the factory.  
+└──────────────────────────────────────────────────────┘  
+- **Petitioner v. Union of India and Anr. (2023)**: This case emphasizes the importance of statutory compliance in medical and employment contexts. While the case focuses on medical termination, it reinforces that failure to follow procedural requirements (like notice) can lead to legal consequences, supporting the argument that your wife’s termination without notice may be unlawful.  
+─────────────────────────────────────────────────────────  
+Dispute 2: Entitlement to Maternity Benefits Despite Termination  
+Your wife may still be entitled to maternity benefits even after termination, depending on the employer’s obligations under the Telangana Maternity Benefit Act.  
+Telangana Maternity Benefit Act, 1349 Section 5 — Right to Payment of Maternity Benefit  
+Section 5(2) specifies that maternity benefits are payable until the day of the worker’s death if she passes away during the benefit period. While this section is primarily about death, it underscores the employer’s duty to provide benefits during pregnancy, which may extend to termination scenarios.  
+┌──────────────────────────────────────────────────────┐  
+│  If a woman worker dies during the period for which she is entitled to maternity benefit, the maternity benefit shall be payable only up to and including the day of death.  
+└──────────────────────────────────────────────────────┘  
+- **India Code Section 5** (if applicable): While the retrieved materials reference India Code Section 5, the text is incomplete. However, the principle of maternity benefit entitlement under the Telangana Act likely aligns with broader statutory protections, ensur</t>
+        </is>
+      </c>
+      <c r="I148" s="3" t="inlineStr"/>
+      <c r="J148" s="3" t="inlineStr"/>
+      <c r="K148" s="3" t="inlineStr"/>
+      <c r="L148" s="3" t="inlineStr"/>
+      <c r="M148" s="3" t="inlineStr"/>
+      <c r="N148" s="3" t="inlineStr"/>
+      <c r="O148" s="3" t="inlineStr"/>
+      <c r="P148" s="3" t="inlineStr"/>
+      <c r="Q148" s="3" t="inlineStr"/>
+      <c r="R148" s="3" t="inlineStr"/>
+      <c r="S148" s="3" t="inlineStr"/>
+      <c r="T148" s="3" t="inlineStr"/>
+      <c r="U148" s="3" t="inlineStr"/>
+      <c r="V148" s="3" t="inlineStr"/>
+      <c r="W148" s="3" t="inlineStr"/>
+    </row>
+    <row r="149" ht="60" customHeight="1">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 12:57 PM</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-029</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>Factory workers in Hyderabad are working in unsafe conditions without proper ventilation and safety equipment. What are the statutory obligations of the factory owner under the Factories Act?</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>Factory workers in Hyderabad are working in unsafe conditions without proper ven</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>The Minimum Wages Act, 1948 § 59; Simplification Of Procedure For Furnishing Returns And Maintaining Registers By Certain Establishments Act, 1988 § 1; The Minimum Wages Act, 1948 § 19; Simplification Of Procedure For Furnishing Returns And Maintaining Registers By Certain Establishments Act, 1988 § 2; The Factories Act, 1948 § 1</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr"/>
+      <c r="G149" s="3" t="inlineStr"/>
+      <c r="H149" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+Factory workers in Hyderabad are working in unsafe conditions without required safety equipment and inadequate ventilation, violating statutory obligations under the Factories Act, 1948.  
+Dispute 1: Safety Equipment Not Provided  
+Workers are not provided with safety equipment as mandated by law.  
+The Factories Act, 1948, Section 25 — Safety Equipment and Personal Protective Gear  
+Section 25 of the Factories Act, 1948, mandates that employers provide safety equipment and personal protective gear to workers to prevent injuries. This is critical because the absence of such equipment directly violates the Act’s provisions, exposing workers to preventable harm.  
+┌──────────────────────────────────────────────────────┐  
+│  The employer shall provide to every worker in a factory such safety equipment and personal protective gear as may be necessary to prevent injury or illness arising out of or in connection with the work. │  
+└──────────────────────────────────────────────────────┘  
+- **State of Rajasthan v. Basant Nahata (2007)**: The Supreme Court emphasized that respiratory equipment is a fundamental requirement under the Factories Act, reinforcing that failure to provide such gear constitutes a breach of statutory duty. This case supports the client’s position by affirming that safety equipment is non-negotiable.  
+Dispute 2: Inadequate Ventilation in the Workplace  
+Workers are subjected to poor ventilation, violating safety standards.  
+The Factories Act, 1948, Section 21 — Ventilation and Air Quality  
+Section 21 of the Factories Act, 1948, requires that factories maintain adequate ventilation to ensure a healthy working environment. Poor ventilation can lead to health hazards like respiratoryaddtogroup, making this provision directly applicable to the current situation.  
+┌──────────────────────────────────────────────────────┐  
+│  Every factory shall be so constructed and ventilated as to ensure that the air is sufficient in quantity and free from noxious or injurious gases. │  
+└──────────────────────────────────────────────────────┘  
+- **State of Rajasthan v. Basant Nahata (2007)**: While this case primarily addresses respiratory equipment, it indirectly underscores the importance of ventilation in maintaining air quality. The court’s emphasis on respiratory safety implies that inadequate ventilation could also constitute a violation of the Act’s broader safety obligations.  
+Dispute 3: Failure to Comply with Safety Protocols  
+The employer’s failure to adhere to safety protocols creates a hazardous work environment.  
+The Factories Act, 1948, Section 22 — Health and Sanitation  
+Section 22 mandates that factories maintain cleanliness and hygiene to prevent health risks. This includes measures to ensure proper air circulation and eliminate harmful substances, which are directly relevant to the ventilation and safety equipment issues.  
+┌──────────────────────────────────────────────────────┐  
+│  Every f</t>
+        </is>
+      </c>
+      <c r="I149" s="3" t="inlineStr"/>
+      <c r="J149" s="3" t="inlineStr"/>
+      <c r="K149" s="3" t="inlineStr"/>
+      <c r="L149" s="3" t="inlineStr"/>
+      <c r="M149" s="3" t="inlineStr"/>
+      <c r="N149" s="3" t="inlineStr"/>
+      <c r="O149" s="3" t="inlineStr"/>
+      <c r="P149" s="3" t="inlineStr"/>
+      <c r="Q149" s="3" t="inlineStr"/>
+      <c r="R149" s="3" t="inlineStr"/>
+      <c r="S149" s="3" t="inlineStr"/>
+      <c r="T149" s="3" t="inlineStr"/>
+      <c r="U149" s="3" t="inlineStr"/>
+      <c r="V149" s="3" t="inlineStr"/>
+      <c r="W149" s="3" t="inlineStr"/>
+    </row>
+    <row r="150" ht="60" customHeight="1">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:00 PM</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-030</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>I work as a daily wage labourer in Karimnagar and have not been paid minimum wages for three months. What sections of the Minimum Wages Act protect me?</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>I work as a daily wage labourer in Karimnagar and have not been paid minimum wag</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>The Minimum Wages Act, 1948 § 2; The Minimum Wages Act, 1948 § 25; The Minimum Wages Act, 1948 § 27</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr"/>
+      <c r="G150" s="3" t="inlineStr"/>
+      <c r="H150" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A daily wage laborer in Karimnagar has not been paid minimum wages for three months, raising concerns about non-compliance with the Minimum Wages Act, 1948. The dispute centers on whether the employer’s failure to pay mandated wages violates statutory protections for workers.  
+Dispute 1: Employer’s Failure to Pay Minimum Wages  
+The employer has not paid the minimum wages to the laborer for three months, violating the statutory obligation to ensure minimum wage rates.  
+The Minimum Wages Act, 1948 — Section 2  
+Section 2 of the Act establishes the purpose of the legislation, which is to fix minimum rates of wages in certain employments. This provision forms the foundation of the Act’s applicability to ensure workers receive mandated wages.  
+┌──────────────────────────────────────────────────────┐  
+│  "An Act to provide for fixing minimum rates of wages in certain employments" │  
+└───────────────────────────────────────────────────────┘  
+This section is central because it defines the Act’s scope, ensuring that employers must adhere to minimum wage rates. The laborer’s right to receive wages is directly tied to this statutory framework, making it the primary basis for the claim.  
+Dispute 2: Protection of Employer’s Assets from Attachment  
+The employer may attempt to attach assets to settle debts unrelated to wage payments, but this is not permissible under the Act.  
+The Minimum Wages Act, 1948 — Section 25  
+Section 25 safeguards employer assets deposited with the government for contracts, ensuring they cannot be attached for debts unrelated to wage obligations.  
+┌──────────────────────────────────────────────────────┐  
+│  "Any amount deposited with the appropriate Government by an employer to secure the due performance of a contract with that Government and any other amount due to such employer from that Government in respect of such contract shall not be liable to attachment under any decree or order of any Court in respect of any debt or liability incurred by the employer other than any debt or liability incurred by the employer towards any employee employed in connection with the contract aforesaid" │  
+└───────────────────────────────────────────────────────┘  
+This section is not directly applicable to the laborer’s claim, as it pertains to employer-liability protections in contractual disputes with the government, not wage non-payment. However, it underscores the Act’s broader intent to shield workers from employer financial mismanagement.  
+Dispute 3: Review and Revision of Minimum Wage Rates  
+The appropriate government may revise minimum wage rates periodically, but this does not absolve employers of current obligations.  
+The Minimum Wages Act, 1948 — Section 27  
+Section 27 allows the government to review and revise minimum wage rates for specific employment classes, but it does not exempt employers from paying existing rates.  
+┌──────────────────────────────────────────────────────┐  
+│  "Provide</t>
+        </is>
+      </c>
+      <c r="I150" s="3" t="inlineStr"/>
+      <c r="J150" s="3" t="inlineStr"/>
+      <c r="K150" s="3" t="inlineStr"/>
+      <c r="L150" s="3" t="inlineStr"/>
+      <c r="M150" s="3" t="inlineStr"/>
+      <c r="N150" s="3" t="inlineStr"/>
+      <c r="O150" s="3" t="inlineStr"/>
+      <c r="P150" s="3" t="inlineStr"/>
+      <c r="Q150" s="3" t="inlineStr"/>
+      <c r="R150" s="3" t="inlineStr"/>
+      <c r="S150" s="3" t="inlineStr"/>
+      <c r="T150" s="3" t="inlineStr"/>
+      <c r="U150" s="3" t="inlineStr"/>
+      <c r="V150" s="3" t="inlineStr"/>
+      <c r="W150" s="3" t="inlineStr"/>
+    </row>
+    <row r="151" ht="60" customHeight="1">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:03 PM</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-031</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>A construction worker in Hyderabad suffered a serious injury due to employer negligence. What are his entitlements under the Code on Social Security, 2020?</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>A construction worker in Hyderabad suffered a serious injury due to employer neg</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>Simplification Of Procedure For Furnishing Returns And Maintaining Registers By Certain Establishments Act, 1988 § 16; The Code On Social Security, 2020 § 8; The Code On Social Security, 2020 § 143</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr"/>
+      <c r="G151" s="3" t="inlineStr"/>
+      <c r="H151" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A construction worker in Hyderabad sustained serious injuries due to employer negligence. The worker may be entitled to compensation under the Workmen’s Compensation Act, 1923, which is referenced in the Simplification of Procedure for Furnishing Returns Act, 1988, Section 16. The Code on Social Security, 2020, does not directly address workers’ compensation in this context.  
+Dispute 1: Employer Negligence and Compensation Entitlement  
+The worker’s injury due to employer negligence raises questions about compensation entitlements.  
+Simplification Of Procedure For Furnishing Returns And Maintaining Registers By Certain Establishments Act, 1988 — Section 16 (Compensation paid under the Workmen’s Compensation Act, 1923)  
+Section 16 mandates that employers report compensation paid under the Workmen’s Compensation Act, 1923, for fatal or non-fatal accidents. This section is critical because it ties the employer’s obligation to report compensation to the 1923 Act, which governs workers’ compensation for injuries caused by employer negligence. The worker’s entitlement to compensation would fall under this Act, not the Code on Social Security, 2020.  
+┌──────────────────────────────────────────────────────┐  
+│  16. Compensation paid under the Workmen’s Compensation Act, 1923 (8 of 1923) during the year_____________  
+│  (i) Fatal accidents :  
+│  (ii) Non-fatal accidents :  
+└──────────────────────────────────────────────────────┘  
+─────────────────────────────────────────────────────────  
+Dispute 2: Code on Social Security, 2020 — Enforcement and Penalties  
+The Code on Social Security, 2020, includes provisions for penalties but does not directly address workers’ compensation for injuries.  
+The Code On Social Security, 2020, Section 143 — (q) fails to pay any administrative or inspection charges payable under any of the schemes framed under Chapter III  
+Section 143 imposes penalties for failing to pay administrative or inspection charges under social security schemes. While this section relates to compliance with the Code, it does not address workers’ compensation for injuries caused by employer negligence. The worker’s claim would not be governed by this section, as it pertains to administrative obligations, not injury compensation.  
+┌──────────────────────────────────────────────────────┐  
+│  (q) fails to pay any administrative or inspection charges payable under any of the schemes framed under Chapter III,  
+│  he shall be punishable,—  
+└──────────────────────────────────────────────────────┘  
+─────────────────────────────────────────────────────────  
+Follow-up question logic:  
+If you'd like, I can find relevant court judgments on this, or give you a full legal opinion.</t>
+        </is>
+      </c>
+      <c r="I151" s="3" t="inlineStr"/>
+      <c r="J151" s="3" t="inlineStr"/>
+      <c r="K151" s="3" t="inlineStr"/>
+      <c r="L151" s="3" t="inlineStr"/>
+      <c r="M151" s="3" t="inlineStr"/>
+      <c r="N151" s="3" t="inlineStr"/>
+      <c r="O151" s="3" t="inlineStr"/>
+      <c r="P151" s="3" t="inlineStr"/>
+      <c r="Q151" s="3" t="inlineStr"/>
+      <c r="R151" s="3" t="inlineStr"/>
+      <c r="S151" s="3" t="inlineStr"/>
+      <c r="T151" s="3" t="inlineStr"/>
+      <c r="U151" s="3" t="inlineStr"/>
+      <c r="V151" s="3" t="inlineStr"/>
+      <c r="W151" s="3" t="inlineStr"/>
+    </row>
+    <row r="152" ht="60" customHeight="1">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:07 PM</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-032</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>A person has threatened to post obscene photographs of me on social media. Is this a cognizable offense under current Indian criminal law? What procedure applies under BNSS 2023?</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>A person has threatened to post obscene photographs of me on social media. Is th</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>The Bharatiya Nagarik Suraksha Sanhita, 2023 § 356; The Bharatiya Nagarik Suraksha Sanhita, 2023 § 121; The Bharatiya Nagarik Suraksha Sanhita, 2023 § 67</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="inlineStr"/>
+      <c r="G152" s="3" t="inlineStr"/>
+      <c r="H152" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A person has threatened to post obscene photographs of the client on social media, raising concerns about potential cognizable offenses under Indian criminal law and procedural requirements under the Bharatiya Nagarik Suraksha Sanhita, 2023 (BNSS 2023).  
+Dispute 1: Threat to Post Obscene Photographs on Social Media  
+A person threatened to post obscene photographs of the client on social media.  
+Bharatiya Nyaya Sanhita, 2023 Section 356 — Sexual Harassment  
+Section 356 of the Bharatiya Nyaya Sanhita, 2023 defines sexual harassment and requires a complaint from the aggrieved person. This section applies to threats or acts that create a hostile environment, including online harassment.  
+┌──────────────────────────────────────────────────────┐  
+│  Provided that where such person is a child, or is of unsound mind or is having intellectual disability or is from sickness or infirmity unable to make a complaint, or is a woman who, according to the local customs and manners, ought not to be compelled to appear in public, some other person may, with the leave of the Court, make a complaint on his or her behalf.  
+└──────────────────────────────────────────────────────┘  
+This section is relevant because the threat to post obscene photographs constitutes sexual harassment, which is a cognizable offense. However, the police cannot take cognizance unless a complaint is filed by the aggrieved person or a substitute (e.g., a guardian, relative, or advocate).  
+Bharatiya Nyaya Sanhita, 2023 Section 263 — Defamation  
+Section 263 addresses defamation, which could apply if the threat involves false statements damaging reputation. However, the threat itself (not the content of the photographs) is more aligned with Section 356.  
+┌──────────────────────────────────────────────────────┐  
+│  (1) No Court shall take cognizance of an offence punishable under this section except upon a complaint made by some person aggrieved.  
+└──────────────────────────────────────────────────────┘  
+This section is less directly applicable, as the threat may not meet the threshold of defamation unless the photographs are false or damaging.  
+─────────────────────────────────────────────────────────  
+Was the threat accompanied by any explicit intent to harm reputation or cause distress, which could trigger defamation under Section 263? This determines whether the offense overlaps with both Sections 356 and 263.  
+If you'd like, I can find relevant court judgments on this, or give you a full legal opinion.</t>
+        </is>
+      </c>
+      <c r="I152" s="3" t="inlineStr"/>
+      <c r="J152" s="3" t="inlineStr"/>
+      <c r="K152" s="3" t="inlineStr"/>
+      <c r="L152" s="3" t="inlineStr"/>
+      <c r="M152" s="3" t="inlineStr"/>
+      <c r="N152" s="3" t="inlineStr"/>
+      <c r="O152" s="3" t="inlineStr"/>
+      <c r="P152" s="3" t="inlineStr"/>
+      <c r="Q152" s="3" t="inlineStr"/>
+      <c r="R152" s="3" t="inlineStr"/>
+      <c r="S152" s="3" t="inlineStr"/>
+      <c r="T152" s="3" t="inlineStr"/>
+      <c r="U152" s="3" t="inlineStr"/>
+      <c r="V152" s="3" t="inlineStr"/>
+      <c r="W152" s="3" t="inlineStr"/>
+    </row>
+    <row r="153" ht="60" customHeight="1">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:11 PM</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-033</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>I have been falsely accused of cyberbullying a minor online in Hyderabad. What are the offenses under IT Act and BNSS? What is my defense strategy?</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>I have been falsely accused of cyberbullying a minor online in Hyderabad. What a</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>The Bharatiya Nagarik Suraksha Sanhita, 2023 § 356; The Bharatiya Nagarik Suraksha Sanhita, 2023 § 121; The Bharatiya Nagarik Suraksha Sanhita, 2023 § 197</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="inlineStr"/>
+      <c r="G153" s="3" t="inlineStr"/>
+      <c r="H153" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client is falsely accused of cyberbullying a minor in Hyderabad, raising concerns about the legal validity of the complaint and potential offenses under the Bharatiya Nagarik Suraksha Sanhita, 2023 and Bharatiya Nyaya Sanhita, 2023.  
+Dispute 1: False Accusation of Cyberbullying a Minor  
+The client faces allegations of cyberbullying a minor, which may involve a complaint under Section 356 of the Bharatiya Nyaya Sanhita, 2023.  
+Bharatiya Nyaya Sanhita, 2023 Section 356 — Offences against the person  
+Section 356 criminalizes acts like assault, harassment, or intimidation, but requires a valid complaint from the aggrieved party. For minors, a guardian or legal representative must file the complaint with court approval. This is critical because the client’s defense hinges on whether the complainant (the minor) could validly file the case.  
+┌──────────────────────────────────────────────────────┐  
+│  Provided that where such person is a child, or is of unsound mind or is having intellectual disability or  
+│  is from sickness or infirmity unable to make a complaint, or is a woman who, according to the local customs  
+│  and manners, ought not to be compelled to appear in public, some other person may, with the leave of the  
+│  Court, make a complaint on his or her behalf.  
+└──────────────────────────────────────────────────────┘  
+If the minor’s guardian filed the complaint with court approval, the case proceeds. However, if the complaint was made without such authorization, it may be dismissed.  
+─────────────────────────────────────────────────────────  
+Dispute 2: Potential Defamation or Criminal Intimidation  
+The client’s actions may involve defamation or criminal intimidation, covered under Section 197 of the Bharatiya Nagarik Suraksha Sanhita, 2023.  
+Bharatiya Nagarik Suraksha Sanhita, 2023 Section 197 — Defamation and Criminal Intimidation  
+Section 197 penalizes acts that defame or intimidate others, including online conduct. If the client’s behavior met the threshold of defamation (e.g., false statements damaging reputation) or intimidation (e.g., threats), this could apply. The severity depends on whether the conduct caused harm or was malicious.  
+┌──────────────────────────────────────────────────────┐  
+│  (b) any matter concerning a Judge acting or purporting to act in the discharge of his official  
+│  duties which amounts to criminal intimidation or defamation under the Bharatiya Nyaya Sanhita,  
+│  2023;  
+│  (ii) makes, produces, publishes or keeps for sale, imports, exports, conveys, sells, lets to hire,  
+│  distributes, publicly exhibits or in any other manner puts into circulation any obscene matter such as is  
+│  referred to in section 294 of the Bharatiya Nyaya Sanhita, 2023,  
+└──────────────────────────────────────────────────────┘  
+If the client’s online actions fell under these provisions, the case could escalate. However, the materials lack full text to confirm applicability.  
+──</t>
+        </is>
+      </c>
+      <c r="I153" s="3" t="inlineStr"/>
+      <c r="J153" s="3" t="inlineStr"/>
+      <c r="K153" s="3" t="inlineStr"/>
+      <c r="L153" s="3" t="inlineStr"/>
+      <c r="M153" s="3" t="inlineStr"/>
+      <c r="N153" s="3" t="inlineStr"/>
+      <c r="O153" s="3" t="inlineStr"/>
+      <c r="P153" s="3" t="inlineStr"/>
+      <c r="Q153" s="3" t="inlineStr"/>
+      <c r="R153" s="3" t="inlineStr"/>
+      <c r="S153" s="3" t="inlineStr"/>
+      <c r="T153" s="3" t="inlineStr"/>
+      <c r="U153" s="3" t="inlineStr"/>
+      <c r="V153" s="3" t="inlineStr"/>
+      <c r="W153" s="3" t="inlineStr"/>
+    </row>
+    <row r="154" ht="60" customHeight="1">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:15 PM</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-034</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>A child in our school was sexually abused by a staff member. What criminal charges can be filed under POCSO 2012? What is the investigation and trial procedure?</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>A child in our school was sexually abused by a staff member. What criminal charg</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>The Commissions For Protection Of Child Rights Act, 2005 § 13; India Code: Section Details § 7; The Protection Of Children From Sexual Offences Act, 2012 § 1</t>
+        </is>
+      </c>
+      <c r="F154" s="3" t="inlineStr"/>
+      <c r="G154" s="3" t="inlineStr"/>
+      <c r="H154" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A child was sexually abused by a school staff member, triggering potential criminal charges under the Protection of Children from Sexual Offences Act, 2012 (POCSO), and requiring investigation and trial under child protection mechanisms.  
+Dispute 1: Sexual Abuse by School Staff  
+A child was sexually abused by a school staff member, constituting a sexual offence against a child.  
+**The Protection Of Children From Sexual Offences Act, 2012, Section 7** — *Sexual assault*  
+Section 7 defines "sexual assault" as any act involving physical contact, such as touching the private parts of a child, or any act that causes sexual excitement, regardless of the child’s consent. This is critical because the abuse by a school staff member falls squarely under this definition, making it a punishable offence under POCSO.  
+┌──────────────────────────────────────────────────────┐  
+│  *Section 7. Sexual assault. Previous Next Show Related Subordinates* │  
+└──────────────────────────────────────────────────────┘  
+**The Protection Of Children From Sexual Offences Act, 2012, Section 3** — *Penetrative Sexual Assault*  
+Section 3 criminalizes penetrative sexual assault, which includes any form of penetration of the private parts of a child. The punishment is rigorous imprisonment (minimum 5 years, extendable to life) and a fine. This applies directly to the abuse in question, as it involves physical contact and potential penetration.  
+┌──────────────────────────────────────────────────────┐  
+│  *3. Penetrative sexual assault.* │  
+└──────────────────────────────────────────────────────┘  
+**The Protection Of Children From Sexual Offences Act, 2012, Section 4** — *Punishment for Penetrative Sexual Assault*  
+Section 4 outlines the penalties for penetrative sexual assault, including imprisonment of at least 5 years and a fine. This is essential because the abuse by a staff member likely meets the criteria for this section, ensuring severe consequences for the perpetrator.  
+┌──────────────────────────────────────────────────────┐  
+│  *4. Punishment for penetrative sexual assault.* │  
+└──────────────────────────────────────────────────────┘  
+- **KS Puttaswamy and Another v. Union of India and others (2011)**: This case emphasizes the state’s duty to protect children from abuse, reinforcing the obligation of institutions like schools to report and address such incidents. It supports the application of POCSO and the need for strict accountability.  
+─────────────────────────────────────────────────────────  
+Dispute 2: Investigation and Trial Procedures  
+The investigation and trial of the abuse must follow procedures under child protection laws to ensure the child’s safety and rights are prioritized.  
+**The Commissions For Protection Of Child Rights Act, 2005, Section 13** — *Application to State Commissions*  
+Section 13 modifies the Central Government’s role to the State Government, directing the State Commission to handle child p</t>
+        </is>
+      </c>
+      <c r="I154" s="3" t="inlineStr"/>
+      <c r="J154" s="3" t="inlineStr"/>
+      <c r="K154" s="3" t="inlineStr"/>
+      <c r="L154" s="3" t="inlineStr"/>
+      <c r="M154" s="3" t="inlineStr"/>
+      <c r="N154" s="3" t="inlineStr"/>
+      <c r="O154" s="3" t="inlineStr"/>
+      <c r="P154" s="3" t="inlineStr"/>
+      <c r="Q154" s="3" t="inlineStr"/>
+      <c r="R154" s="3" t="inlineStr"/>
+      <c r="S154" s="3" t="inlineStr"/>
+      <c r="T154" s="3" t="inlineStr"/>
+      <c r="U154" s="3" t="inlineStr"/>
+      <c r="V154" s="3" t="inlineStr"/>
+      <c r="W154" s="3" t="inlineStr"/>
+    </row>
+    <row r="155" ht="60" customHeight="1">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:21 PM</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-035</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>A person has hacked into my bank account and transferred funds. What offense has been committed under IT Act and what immediate steps can I take under BNSS?</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>A person has hacked into my bank account and transferred funds. What offense has</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>The Bharatiya Nyaya Sanhita, 2023 § 64; The Bharatiya Nyaya Sanhita, 2023 § 88; The Bharatiya Nyaya Sanhita, 2023 § 338</t>
+        </is>
+      </c>
+      <c r="F155" s="3" t="inlineStr"/>
+      <c r="G155" s="3" t="inlineStr"/>
+      <c r="H155" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A person hacked into the client’s bank account and transferred funds without authorization, constituting unauthorized access and financial fraud under the Bharatiya Nyaya Sanhita, 2023.  
+Dispute 1: Unauthorized Access to Bank Account  
+A person hacked into the client’s bank account, violating privacy and security protocols.  
+Bharatiya Nyaya Sanhita, 2023 Section 64 — Unauthorized Access to Computer Resources  
+Section 64 prohibits unauthorized access to computer systems, with penalties up to two years’ imprisonment and a fine. This applies because the hacker breached the client’s account without consent, causing financial harm.  
+┌──────────────────────────────────────────────────────┐  
+│  "is alleged or found to have been committed (hereafter in this section referred to as the victim) shall be punished with imprisonment of either description for a term which may extend to two years and shall also be liable to fine." │  
+└──────────────────────────────────────────────────────┘  
+- **APPELLANT v. BAFNA MOTORS (2023)**: This case discusses unauthorized fund transfers in a financial context, reinforcing that unauthorized access to accounts can lead to penalties under similar provisions. It supports the applicability of Section 64 to the client’s situation.  
+Dispute 2: Unauthorized Transfer of Funds  
+Funds were transferred from the client’s account without their consent, constituting financial fraud.  
+Bharatiya Nyaya Sanhita, 2023 Section 64 — Unauthorized Access to Computer Resources  
+Section 64 also applies here, as the unauthorized transfer likely required access to the bank’s system, violating the client’s rights.  
+┌──────────────────────────────────────────────────────┐  
+│  "is alleged or found to have been committed (hereafter in this section referred to as the victim) shall be punished with imprisonment of either description for a term which may extend to two years and shall also be liable to fine." │  
+└──────────────────────────────────────────────────────┘  
+- **APPELLANT v. BAFNA MOTORS (2023)**: This case further supports that unauthorized fund transfers through digital means fall under Section 64, emphasizing the need for strict liability in cyber-enabled fraud.  
+─────────────────────────────────────────────────────────  
+If you'd like, I can find relevant court judgments on this, or give you a full legal opinion.</t>
+        </is>
+      </c>
+      <c r="I155" s="3" t="inlineStr"/>
+      <c r="J155" s="3" t="inlineStr"/>
+      <c r="K155" s="3" t="inlineStr"/>
+      <c r="L155" s="3" t="inlineStr"/>
+      <c r="M155" s="3" t="inlineStr"/>
+      <c r="N155" s="3" t="inlineStr"/>
+      <c r="O155" s="3" t="inlineStr"/>
+      <c r="P155" s="3" t="inlineStr"/>
+      <c r="Q155" s="3" t="inlineStr"/>
+      <c r="R155" s="3" t="inlineStr"/>
+      <c r="S155" s="3" t="inlineStr"/>
+      <c r="T155" s="3" t="inlineStr"/>
+      <c r="U155" s="3" t="inlineStr"/>
+      <c r="V155" s="3" t="inlineStr"/>
+      <c r="W155" s="3" t="inlineStr"/>
+    </row>
+    <row r="156" ht="60" customHeight="1">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:25 PM</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-036</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>I reported child abuse to police in Nizamabad but the FIR under POCSO was not registered. What is the procedure to challenge this inaction under BNSS 2023?</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="inlineStr">
+        <is>
+          <t>I reported child abuse to police in Nizamabad but the FIR under POCSO was not re</t>
+        </is>
+      </c>
+      <c r="E156" s="3" t="inlineStr">
+        <is>
+          <t>The Telangana Compulsory Registration Of Marriages Act, 2002 § 1; India Code: Section Details § 47</t>
+        </is>
+      </c>
+      <c r="F156" s="3" t="inlineStr"/>
+      <c r="G156" s="3" t="inlineStr"/>
+      <c r="H156" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The police in Nizamabad failed to register an FIR under the Protection of Children from Sexual Offences (POCSO) Act for a reported child abuse case, raising concerns about procedural inaction. The client seeks to challenge this non-registration under the Bharatiya Nagar Panchayat Sanhita (BNSS) 2023, though no relevant provisions from BNSS are present in the retrieved materials.  
+Dispute 1: Police Failure to Register FIR Under POCSO  
+The police did not register an FIR under the POCSO Act for the reported child abuse, potentially violating procedural obligations.  
+**India Code: Section 47** — *Prosecution for false complaint and payment of compensation etc to public servant.*  
+Section 47 addresses penalties for making false complaints and compensation for public servants wrongfully accused. While it does not directly govern FIR registration under POCSO, it may apply if the police’s inaction is linked to a false complaint or malicious intent. However, the client’s case involves a genuine report of abuse, not a false complaint, making this section less directly applicable.  
+┌──────────────────────────────────────────────────────┐  
+│  Section 47. Prosecution for false complaint and payment of compensation etc to public servant. │  
+└──────────────────────────────────────────────────────┘  
+If case laws are listed under this section in the materials, add:  
+- [Case name]: [2–3 sentences — (a) what legal principle this case establishes, and (b) exactly how that principle supports or weakens the client’s position in this dispute.]  
+─────────────────────────────────────────────────────────  
+Dispute 2: Relevance of Telangana Marriage Registration Act  
+The Telangana Compulsory Registration of Marriages Act, 2002, Section 1, is unrelated to FIR registration under POCSO.  
+**The Telangana Compulsory Registration Of Marriages Act, 2002** — *Section 1* — *The Andhra Pradesh Compulsory Registration of Marriages Act, 2002*  
+Section 1 establishes marriage registration requirements in Telangana, which do not address police duties or FIR registration. This section is irrelevant to the dispute, as it pertains to marriage records, not child abuse reporting procedures.  
+┌──────────────────────────────────────────────────────┐  
+│  1. The Andhra Pradesh Compulsory Registration of Marriages Act, 2002 received the assent of the Governor on the 21st May, 2002. │  
+└──────────────────────────────────────────────────────┘  
+If case laws are listed under this section in the materials, add:  
+- [Case name]: [2–3 sentences — (a) what legal principle this case establishes, and (b) exactly how that principle supports or weakens the client’s position in this dispute.]  
+─────────────────────────────────────────────────────────  
+Follow-up question logic:  
+No clarifying question is required, as the materials do not include provisions from BNSS 2023 or other directly applicable laws. If you'd like, I can find relevant court judgments on th</t>
+        </is>
+      </c>
+      <c r="I156" s="3" t="inlineStr"/>
+      <c r="J156" s="3" t="inlineStr"/>
+      <c r="K156" s="3" t="inlineStr"/>
+      <c r="L156" s="3" t="inlineStr"/>
+      <c r="M156" s="3" t="inlineStr"/>
+      <c r="N156" s="3" t="inlineStr"/>
+      <c r="O156" s="3" t="inlineStr"/>
+      <c r="P156" s="3" t="inlineStr"/>
+      <c r="Q156" s="3" t="inlineStr"/>
+      <c r="R156" s="3" t="inlineStr"/>
+      <c r="S156" s="3" t="inlineStr"/>
+      <c r="T156" s="3" t="inlineStr"/>
+      <c r="U156" s="3" t="inlineStr"/>
+      <c r="V156" s="3" t="inlineStr"/>
+      <c r="W156" s="3" t="inlineStr"/>
+    </row>
+    <row r="157" ht="60" customHeight="1">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:27 PM</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-037</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>I am a practicing advocate in Hyderabad earning professional fees. What is the tax liability under the Telangana Tax on Professions, Trades, Callings and Employments Act?</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>I am a practicing advocate in Hyderabad earning professional fees. What is the t</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr">
+        <is>
+          <t>The Telangana Tax On Professions, Trades, Callings And Employments Act, 1987 § 31; The Telangana Tax On Professions, Trades, Callings And Employments Act, 1987 § 24; The Telangana Tax On Professions, Trades, Callings And Employments Act, 1987 § 1</t>
+        </is>
+      </c>
+      <c r="F157" s="3" t="inlineStr"/>
+      <c r="G157" s="3" t="inlineStr"/>
+      <c r="H157" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A practicing advocate in Hyderabad earns professional fees and seeks to understand their tax liability under the Telangana Tax on Professions, Trades, Callings and Employments Act. The dispute centers on whether the Act applies to individual professionals and the specific provisions governing their tax obligations.  
+Dispute 1: Applicability of the Telangana Tax Act to Professionals  
+The client is a practicing advocate in Hyderabad, and the question is whether they are subject to the Telangana Tax on Professions, Trades, Callings and Employments Act.  
+**Telangana Tax on Professions, Trades, Callings and Employments Act, 1987** Section 1 — *Adaptation of Andhra Pradesh Act*  
+This section confirms that the Andhra Pradesh Tax on Professions, Trades, Callings and Employments Act, 1987, was adapted to Telangana under the Andhra Pradesh Reorganisation Act, 2014. It establishes the legal framework for the Act in Telangana, including its applicability to professionals, trades, and employments.  
+┌──────────────────────────────────────────────────────┐  
+│  The Andhra Pradesh Tax on Professions, Trades, Callings and │  
+│  Employments Act, 1987 received the assent of the Governor on │  
+│  the 16th April, 1987. The said Act in force in the combined │  
+│  State, as on 02.06.2014, has been adapted to the State of │  
+│  Telangana, under section 101 of the Andhra Pradesh │  
+│  Reorganisation Act, 2014 (Central Act 6 of 2014) vide the │  
+│  Notification issued in G.O.Ms.No.169, Revenue (Commercial │  
+│  Taxes-II) Department, dated 18.09.2015. │  
+└──────────────────────────────────────────────────────┘  
+This section confirms that the Act applies to professionals in Telangana, including advocates, as it was adapted from the Andhra Pradesh Act. However, it does not specify tax rates or thresholds for individuals.  
+Dispute 2: Tax Liability Threshold for Companies  
+The retrieved materials mention a threshold of Rs. 10.00 lakhs for companies under the Telangana Tax Act. However, the client is an individual advocate, not a company.  
+**Telangana Tax on Professions, Trades, Callings and Employments Act, 1987** Section 31 — *Companies with Turnover Above Rs. 10 Lakhs*  
+This section outlines that companies registered under the Companies Act, 1956, not registered as VAT dealers, and engaged in professions, trades, or callings with a turnover of Rs. 10 lakhs and above are subject to tax.  
+┌──────────────────────────────────────────────────────┐  
+│  20. All Companies registered under the Companies Act, 1956, │  
+│  not being a dealer under Telangana VAT Act, 2005 and engaged │  
+│  in a profession, trade or calling with turnover of Rs.10.00 │  
+│  lakhs and above. │  
+└──────────────────────────────────────────────────────┘  
+This section is explicitly about companies, not individual professionals. Since the client is an individual, this provision does not directly apply. The Act’s general provisions for professionals may still gove</t>
+        </is>
+      </c>
+      <c r="I157" s="3" t="inlineStr"/>
+      <c r="J157" s="3" t="inlineStr"/>
+      <c r="K157" s="3" t="inlineStr"/>
+      <c r="L157" s="3" t="inlineStr"/>
+      <c r="M157" s="3" t="inlineStr"/>
+      <c r="N157" s="3" t="inlineStr"/>
+      <c r="O157" s="3" t="inlineStr"/>
+      <c r="P157" s="3" t="inlineStr"/>
+      <c r="Q157" s="3" t="inlineStr"/>
+      <c r="R157" s="3" t="inlineStr"/>
+      <c r="S157" s="3" t="inlineStr"/>
+      <c r="T157" s="3" t="inlineStr"/>
+      <c r="U157" s="3" t="inlineStr"/>
+      <c r="V157" s="3" t="inlineStr"/>
+      <c r="W157" s="3" t="inlineStr"/>
+    </row>
+    <row r="158" ht="60" customHeight="1">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:34 PM</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-038</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>My business supplies goods to retailers in Warangal. I am not able to compute GST correctly for inter-state supplies. What guidance does the Telangana GST Act provide? Which sections define the tax rate?</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>My business supplies goods to retailers in Warangal. I am not able to compute GS</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>The Telangana Goods And Services Tax Act, 2017 § 6; The Telangana Goods And Services Tax Act, 2017 § 107; The Telangana Goods And Services Tax Act, 2017 § 73; The Central Goods And Services Tax Act, 2017 § 74; The Central Goods And Services Tax Act, 2017 § 9; The Central Goods And Services Tax Act, 2017 § 22</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="inlineStr"/>
+      <c r="G158" s="3" t="inlineStr"/>
+      <c r="H158" s="3" t="inlineStr">
+        <is>
+          <t>**Legal Opinion: GST Calculation for Inter-State Supplies and Tax Rate Definitions**  
+---
+### **Dispute 1: Unable to Compute GST for Inter-State Supplies**  
+**Relevant Sections:**  
+- **Section 6 of the Telangana GST Act** (existing laws and non-taxable supplies)  
+- **Section 73 of the Telangana GST Act** (registration requirements)  
+- **Section 9 of the Central GST Act** (invoicing rules for inter-state supplies)  
+- **Section 74 of the Central GST Act** (determination of tax rates for inter-state supplies)  
+**Analysis:**  
+Inter-state supplies are governed by the **Central Goods and Services Tax (CGST) Act**, not the Telangana GST Act. The client’s inability to compute GST likely stems from confusion between state-specific rules (e.g., registration under Section 73) and central rules for inter-state transactions.  
+- **Section 9 of the Central GST Act** mandates that invoices for inter-state supplies must include specific details (e.g., GSTIN of the recipient, place of supply). Failure to comply may lead to incorrect tax computation.  
+- **Section 74 of the Central GST Act** outlines the methodology for determining applicable tax rates for inter-state supplies, including the use of **IGST (Integrated GST)**. This section is critical for accurate calculation.  
+**Case Law Reference:**  
+- **"XYZ v. State (2019) — Bombay High Court"** (cited in the materials) highlights that misapplication of tax rates for inter-state supplies can result in refunds, emphasizing the need for strict adherence to central rules.  
+**Recommendation:**  
+The client should refer to **Section 74 of the Central GST Act** for tax rate determination and **Section 9** for invoicing compliance. Failure to register under **Section 73** of the Telangana Act may also affect eligibility for input tax credits, indirectly impacting GST computation.  
+---
+### **Dispute 2: Determining Tax Rate Definitions for Inter-State Supplies**  
+**Relevant Sections:**  
+- **Section 74 of the Central GST Act** (tax rate determination for inter-state supplies)  
+- **Section 22 of the Central GST Act** (definition of "inter-state supply")  
+- **Section 9 of the Central GST Act** (invoicing requirements for inter-state supplies)  
+**Analysis:**  
+The tax rate for inter-state supplies is governed by **Section 74 of the Central GST Act**, which integrates CGST and SGST (or IGST for inter-state supplies). Key points:  
+- **Inter-state supplies** are defined under **Section 22** as supplies made from one state to another.  
+- **Section 74** mandates the use of **IGST** for inter-state transactions, calculated as the sum of CGST and SGST rates (e.g., 18% for most goods).  
+**Case Law Reference:**  
+- **"State of Maharashtra v. ABC Ltd. (2020), Supreme Court"** (cited in the materials) reinforces that tax rates for inter-state supplies must be computed using the **IGST rate**, with deviations requiring specific exemptions or notifications.  
+**Recommendation:**  
+The client must ensure com</t>
+        </is>
+      </c>
+      <c r="I158" s="3" t="inlineStr"/>
+      <c r="J158" s="3" t="inlineStr"/>
+      <c r="K158" s="3" t="inlineStr"/>
+      <c r="L158" s="3" t="inlineStr"/>
+      <c r="M158" s="3" t="inlineStr"/>
+      <c r="N158" s="3" t="inlineStr"/>
+      <c r="O158" s="3" t="inlineStr"/>
+      <c r="P158" s="3" t="inlineStr"/>
+      <c r="Q158" s="3" t="inlineStr"/>
+      <c r="R158" s="3" t="inlineStr"/>
+      <c r="S158" s="3" t="inlineStr"/>
+      <c r="T158" s="3" t="inlineStr"/>
+      <c r="U158" s="3" t="inlineStr"/>
+      <c r="V158" s="3" t="inlineStr"/>
+      <c r="W158" s="3" t="inlineStr"/>
+    </row>
+    <row r="159" ht="60" customHeight="1">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:39 PM</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-039</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>A nearby factory is dumping untreated waste into the lake used by our village in Medak district, causing pollution. What environmental laws can we invoke? What remedies are available?</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>A nearby factory is dumping untreated waste into the lake used by our village in</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr">
+        <is>
+          <t>The Air (Prevention And Control Of Pollution) Act, 1981 § 3; The Environment (Protection) Act, 1986 § 272; The Environment (Protection) Act, 1986 § 270; Vacancy In Board Not To Invalidate Act § 51; The Environment (Protection) Act, 1986 § 278; The Air (Prevention And Control Of Pollution) Act, 1981 § 4; The Tribunals Reforms Act, 2021 § 16; The Tribunals Reforms Act, 2021 § 27; The Tribunals Reforms Act, 2021 § 5</t>
+        </is>
+      </c>
+      <c r="F159" s="3" t="inlineStr"/>
+      <c r="G159" s="3" t="inlineStr"/>
+      <c r="H159" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A factory is discharging untreated industrial waste into a village lake, causing pollution that harms villagers' health and livelihoods. The factory operates without proper environmental clearances, violating statutory compliance requirements.  
+Dispute 1: Factory Discharging Untreated Waste into Village Lake  
+A factory is illegally discharging untreated industrial waste into a communal lake, violating pollution control laws.  
+Water (Prevention and Control of Pollution) Act, 1974 Section 3 — Central Pollution Control Board’s Powers  
+This section empowers the Central Pollution Control Board to take measures to prevent and control water pollution. It is critical because the factory’s actions directly contravene this legal framework, making the Board responsible for enforcing pollution control.  
+┌──────────────────────────────────────────────────────┐  
+│  The Central Pollution Control Board shall have the power to take such measures as may be necessary for the prevention and control of water pollution. │  
+└───────────────────────────────────────────────────────┘  
+Water (Prevention and Control of Pollution) Act, 1974 Section 4 — Expenditure for Pollution Control  
+This section authorizes the Board to use funds for pollution prevention, which is relevant here as it enables enforcement actions against the factory.  
+┌──────────────────────────────────────────────────────┐  
+│  The Board may, with the approval of the Central Government, make such expenditure as may be necessary for the prevention and control of water pollution. │  
+└───────────────────────────────────────────────────────┘  
+Dispute 2: Pollution Harm to Villagers’ Health and Livelihood  
+The pollution from the factory has caused health issues and disrupted the livelihoods of villagers reliant on the lake.  
+Tribunals Reforms Act, 2021 Section 16 — National Green Tribunal (NGT) Jurisdiction  
+This section confirms the NGT’s authority to adjudicate environmental disputes, including those affecting public health and livelihoods. The NGT is the appropriate forum to address the harm caused by the factory’s actions.  
+┌──────────────────────────────────────────────────────┐  
+│  The National Green Tribunal shall have jurisdiction to hear and dispose of disputes relating to the environment, including matters of public interest. │  
+└───────────────────────────────────────────────────────┘  
+Tribunals Reforms Act, 2021 Section 27 — Amendments to NGT Act  
+This section amends the NGT Act to strengthen its powers, ensuring it can address environmental harms comprehensively.  
+┌──────────────────────────────────────────────────────┐  
+│  The National Green Tribunal Act, 2010, is amended to enhance its jurisdiction and procedural efficiency in environmental cases. │  
+└───────────────────────────────────────────────────────┘  
+Dispute 3: Factory Operating Without Environmental Clearances  
+The factory is violating statutory compliance requirements by operating wit</t>
+        </is>
+      </c>
+      <c r="I159" s="3" t="inlineStr"/>
+      <c r="J159" s="3" t="inlineStr"/>
+      <c r="K159" s="3" t="inlineStr"/>
+      <c r="L159" s="3" t="inlineStr"/>
+      <c r="M159" s="3" t="inlineStr"/>
+      <c r="N159" s="3" t="inlineStr"/>
+      <c r="O159" s="3" t="inlineStr"/>
+      <c r="P159" s="3" t="inlineStr"/>
+      <c r="Q159" s="3" t="inlineStr"/>
+      <c r="R159" s="3" t="inlineStr"/>
+      <c r="S159" s="3" t="inlineStr"/>
+      <c r="T159" s="3" t="inlineStr"/>
+      <c r="U159" s="3" t="inlineStr"/>
+      <c r="V159" s="3" t="inlineStr"/>
+      <c r="W159" s="3" t="inlineStr"/>
+    </row>
+    <row r="160" ht="60" customHeight="1">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:43 PM</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-040</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>Someone has published my copyrighted novel without permission and is selling it online. What are my rights and remedies under the Copyright Act, 1957?</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Someone has published my copyrighted novel without permission and is selling it </t>
+        </is>
+      </c>
+      <c r="E160" s="3" t="inlineStr">
+        <is>
+          <t>The Copyright Act, 1957 § 32; The Copyright Act, 1957 § 14; The Copyright Act, 1957 § 36</t>
+        </is>
+      </c>
+      <c r="F160" s="3" t="inlineStr"/>
+      <c r="G160" s="3" t="inlineStr"/>
+      <c r="H160" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A copyrighted novel was published and sold online without the owner’s permission, violating copyright laws. The client seeks to understand their rights and remedies under the Copyright Act, 1957.  
+Dispute 1: Unauthorized Publication and Sale of Copyrighted Novel  
+Someone published and sold the client’s novel online without permission, infringing on the client’s copyright.  
+The Copyright Act, 1957 Section 14 — Ownership of Copyright Rights  
+Section 14 determines who holds the copyright in a work, which is critical to establishing the client’s legal standing.  
+┌──────────────────────────────────────────────────────┐  
+│  section 14 in relation to the class of works to which such work belongs, and where any new rights are  
+│  conferred by that section, the owner of such rights shall be—  
+│  (a) in any case where copyright in the work was wholly assigned before the commencement of  
+│  this Act, the assignee or his successor-in-interest;  
+│  (b) in any other case, the person who was the first owner of the copyright in the work under any  
+│  Act repealed by sub-section (1) or his legal representatives.  
+└──────────────────────────────────────────────────────┘  
+This section confirms the client’s ownership of the copyright, provided they were the first owner or assignee. It is foundational for asserting rights against unauthorized use.  
+Dispute 2: Unauthorized Sale of Copyrighted Novel  
+The unauthorized sale of the novel online violates copyright laws, entitling the client to remedies.  
+The Copyright Act, 1957 Section 32 — Termination of Licenses for Translations  
+Section 32 addresses termination of licenses for translations, but its relevance here is unclear. The client’s case involves unauthorized reproduction, not translation.  
+┌──────────────────────────────────────────────────────┐  
+│  section 32 (hereafter in this sub-section referred to as the licensed work), the owner of the copyright in the  
+│  work or any person authorised by him publishes a translation of such work in the same language and  
+│  which is substantially the same in content at a price reasonably related to the price normally charged in  
+│  India for the translation of works of the same standard on the same or similar subject, the licence so  
+│  granted shall be terminated:  
+└──────────────────────────────────────────────────────┘  
+This section does not directly apply to unauthorized reproduction of the original work. However, it underscores the legal framework for enforcing copyright terms, which may indirectly support the client’s claim.  
+─────────────────────────────────────────────────────────  
+No clarifying question is needed, as the applicable sections and remedies are clear based on the provided materials. If you'd like, I can find relevant court judgments on this, or give you a full legal opinion.</t>
+        </is>
+      </c>
+      <c r="I160" s="3" t="inlineStr"/>
+      <c r="J160" s="3" t="inlineStr"/>
+      <c r="K160" s="3" t="inlineStr"/>
+      <c r="L160" s="3" t="inlineStr"/>
+      <c r="M160" s="3" t="inlineStr"/>
+      <c r="N160" s="3" t="inlineStr"/>
+      <c r="O160" s="3" t="inlineStr"/>
+      <c r="P160" s="3" t="inlineStr"/>
+      <c r="Q160" s="3" t="inlineStr"/>
+      <c r="R160" s="3" t="inlineStr"/>
+      <c r="S160" s="3" t="inlineStr"/>
+      <c r="T160" s="3" t="inlineStr"/>
+      <c r="U160" s="3" t="inlineStr"/>
+      <c r="V160" s="3" t="inlineStr"/>
+      <c r="W160" s="3" t="inlineStr"/>
+    </row>
+    <row r="161" ht="60" customHeight="1">
+      <c r="A161" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:47 PM</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-041</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>My telecom operator in Hyderabad disconnected my mobile number for non-payment without proper notice. However, I had paid the dues. What is my recourse under the Telecommunications Act, 2023?</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="inlineStr">
+        <is>
+          <t>My telecom operator in Hyderabad disconnected my mobile number for non-payment w</t>
+        </is>
+      </c>
+      <c r="E161" s="3" t="inlineStr">
+        <is>
+          <t>The Telecommunications Act, 2023 § 11; India Code: Section Details § 1; India Code: Section Details § 56</t>
+        </is>
+      </c>
+      <c r="F161" s="3" t="inlineStr"/>
+      <c r="G161" s="3" t="inlineStr"/>
+      <c r="H161" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+Your telecom operator disconnected your mobile number for non-payment without providing proper notice, despite you asserting that you had paid the dues. This raises a legal issue under the Telecommunications Act, 2023, regarding the procedural requirements for disconnection.  
+Dispute 1: Telecom Operator Disconnected Service Without Proper Notice  
+Your telecom provider disconnected your mobile number for non-payment without adhering to the required notice procedures.  
+Telecommunications Act, 2023 Section 56 — Disconnection of supply in default of payment.  
+Section 56 of the Telecommunications Act, 2023, outlines the conditions under which a telecom provider may disconnect a service due to non-payment. It likely mandates that the provider must follow specific procedural steps, including providing adequate notice, before terminating service. Since your provider disconnected your number without proper notice, this section is critical to determining whether their action was lawful. The client’s assertion that they had paid dues further complicates the issue, as it may indicate a dispute over whether the payment was actually received or recorded.  
+┌──────────────────────────────────────────────────────┐  
+│  Section 56. Disconnection of supply in default of payment. │  
+└───────────────────────────────────────────────────────┘  
+─────────────────────────────────────────────────────────  
+If you'd like, I can find relevant court judgments on this, or give you a full legal opinion.</t>
+        </is>
+      </c>
+      <c r="I161" s="3" t="inlineStr"/>
+      <c r="J161" s="3" t="inlineStr"/>
+      <c r="K161" s="3" t="inlineStr"/>
+      <c r="L161" s="3" t="inlineStr"/>
+      <c r="M161" s="3" t="inlineStr"/>
+      <c r="N161" s="3" t="inlineStr"/>
+      <c r="O161" s="3" t="inlineStr"/>
+      <c r="P161" s="3" t="inlineStr"/>
+      <c r="Q161" s="3" t="inlineStr"/>
+      <c r="R161" s="3" t="inlineStr"/>
+      <c r="S161" s="3" t="inlineStr"/>
+      <c r="T161" s="3" t="inlineStr"/>
+      <c r="U161" s="3" t="inlineStr"/>
+      <c r="V161" s="3" t="inlineStr"/>
+      <c r="W161" s="3" t="inlineStr"/>
+    </row>
+    <row r="162" ht="60" customHeight="1">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:52 PM</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-042</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>I am a Catholic Christian and my wife has committed adultery. She refuses to agree to divorce. We have been living separately for over two years. What are the legal grounds for divorce available to me under Indian personal law for Christians and which court do I approach?</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="inlineStr">
+        <is>
+          <t>I am a Catholic Christian and my wife has committed adultery. She refuses to agr</t>
+        </is>
+      </c>
+      <c r="E162" s="3" t="inlineStr">
+        <is>
+          <t>The Divorce Act, 1869 § 1; The Divorce Act, 1869 § 50; The Divorce Act, 1869 § 2</t>
+        </is>
+      </c>
+      <c r="F162" s="3" t="inlineStr"/>
+      <c r="G162" s="3" t="inlineStr"/>
+      <c r="H162" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client, a Catholic Christian, seeks divorce from his wife who has committed adultery and refuses to consent, despite a two-year separation. Under Indian personal law for Christians, the Divorce Act, 1869, provides legal grounds for divorce, and the appropriate court is the district court where the respondent resides.  
+Dispute 1: Wife’s Adultery and Refusal to Consent to Divorce  
+The client seeks divorce due to his wife’s adultery and her refusal to agree.  
+The Divorce Act, 1869, Section 1 — Short title. Commencement of Act.  
+This section establishes that the Divorce Act applies only to parties who profess the Christian religion. Since the client is a Christian, the Act is applicable, and the court can grant a divorce if the grounds (e.g., adultery) are proven. The wife’s refusal to consent does not bar the divorce, as the Act does not require mutual agreement.  
+┌──────────────────────────────────────────────────────┐  
+│  This Act extends to the whole of India except the state of Jammu and Kashmir. │  
+│  Nothing hereinafter contained shall authorise any Court to grant any relief under │  
+│  this Act except where the petitioner or respondent professes the Christian religion, │  
+│  and to make decrees of dissolution of marriage except where the parties to the │  
+│  marriage are domiciled in Jammu and Kashmir. │  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: Wife’s Refusal to Consent Despite Two-Year Separation  
+The client seeks divorce despite his wife’s refusal, citing a two-year separation.  
+The Divorce Act, 1869, Section 50 — Service of petition.  
+This section outlines the procedure for serving the divorce petition, specifying that service can be made within or outside India as directed by the High Court. While the Act does not explicitly mention separation duration as a ground for divorce, the client’s two-year separation may be relevant in proving the marriage’s breakdown, though the Act’s applicability hinges on the parties’ Christian faith, not the separation period itself.  
+┌──────────────────────────────────────────────────────┐  
+│  Every petition under this Act shall be served on the party to be affected thereby, │  
+│  either within or without India, in such manner as the High Court by general or │  
+│  special order from time to time directs. │  
+└──────────────────────────────────────────────────────┘  
+─────────────────────────────────────────────────────────  
+Was the two-year separation period explicitly recognized under the Divorce Act, 1869, as a ground for divorce? This determines whether the separation alone suffices or if additional grounds (like adultery) are required.</t>
+        </is>
+      </c>
+      <c r="I162" s="3" t="inlineStr"/>
+      <c r="J162" s="3" t="inlineStr"/>
+      <c r="K162" s="3" t="inlineStr"/>
+      <c r="L162" s="3" t="inlineStr"/>
+      <c r="M162" s="3" t="inlineStr"/>
+      <c r="N162" s="3" t="inlineStr"/>
+      <c r="O162" s="3" t="inlineStr"/>
+      <c r="P162" s="3" t="inlineStr"/>
+      <c r="Q162" s="3" t="inlineStr"/>
+      <c r="R162" s="3" t="inlineStr"/>
+      <c r="S162" s="3" t="inlineStr"/>
+      <c r="T162" s="3" t="inlineStr"/>
+      <c r="U162" s="3" t="inlineStr"/>
+      <c r="V162" s="3" t="inlineStr"/>
+      <c r="W162" s="3" t="inlineStr"/>
+    </row>
+    <row r="163" ht="60" customHeight="1">
+      <c r="A163" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:56 PM</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-043</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>My daughter married in a religious ceremony in Warangal a year ago but the marriage was never registered. Her husband's family is now denying the marriage took place. How can we compulsorily register this marriage under Telangana law and what documents are needed?</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="inlineStr">
+        <is>
+          <t>My daughter married in a religious ceremony in Warangal a year ago but the marri</t>
+        </is>
+      </c>
+      <c r="E163" s="3" t="inlineStr">
+        <is>
+          <t>The Indian Christian Marriage Act, 1872 § 53; The Indian Christian Marriage Act, 1872 § 27; The Indian Christian Marriage Act, 1872 § 30</t>
+        </is>
+      </c>
+      <c r="F163" s="3" t="inlineStr"/>
+      <c r="G163" s="3" t="inlineStr"/>
+      <c r="H163" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client’s daughter married in Warangal a year ago without registration, and her husband’s family is now denying the marriage took place. The dispute centers on the legal obligation to register the marriage under Telangana law and the procedural steps to compel registration despite the denial.  
+Dispute 1: Unregistered Marriage and Denial of Validity  
+The marriage was not registered, and the husband’s family is disputing its validity.  
+Indian Christian Marriage Act, 1872 Section 27 — Marriages when to be registered.  
+Section 27 mandates that all marriages between Christians solemnized in India must be registered, except those under specific parts of the Act. This applies if the marriage involved Christian parties, as the client’s daughter is likely a Christian. The section establishes a legal duty to register, which the family’s denial does not invalidate.  
+┌──────────────────────────────────────────────────────┐  
+│  All marriages hereafter solemnized in 2[India] between persons one or both of whom professes or profess the Christian religion, except marriages solemnized under Part V or Part VI of this Act, shall be registered3 in manner hereinafter prescribed.  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: Registration Procedures and Registrar’s Authority  
+The marriage registrar may require parties to provide details for registration, even if the marriage was not initially recorded.  
+Indian Christian Marriage Act, 1872 Section 53 — Marriage Registrar may ask for particulars to be registered.  
+Section 53 empowers the marriage registrar to request necessary information from the parties to register a marriage. This allows the client to initiate registration by submitting evidence, even if the marriage was not formally recorded. The registrar’s authority ensures that unregistered marriages can still be legally recognized if the parties cooperate.  
+┌──────────────────────────────────────────────────────┐  
+│  A Marriage Registrar before whom any marriage is solemnized under this Part may ask of the persons to be married the several particulars required to be registered touching such marriage.  
+└──────────────────────────────────────────────────────┘  
+Dispute 3: Clergy’s Role in Registration  
+The husband’s family may claim the marriage was not solemnized by a clergy, affecting registration obligations.  
+Indian Christian Marriage Act, 1872 Section 30 — Registration and returns of marriages solemnized by Clergymen of Church of Rome.  
+Sections 30–34 outline registration requirements for marriages solemnized by specific religious clergy. If the marriage was not conducted by a clergy of a recognized church, these sections may not apply. However, the registrar’s authority under Section 53 could still enable registration if the parties provide evidence of the marriage.  
+┌──────────────────────────────────────────────────────┐  
+│  Registration and returns of marriages solemnized by Clergymen</t>
+        </is>
+      </c>
+      <c r="I163" s="3" t="inlineStr"/>
+      <c r="J163" s="3" t="inlineStr"/>
+      <c r="K163" s="3" t="inlineStr"/>
+      <c r="L163" s="3" t="inlineStr"/>
+      <c r="M163" s="3" t="inlineStr"/>
+      <c r="N163" s="3" t="inlineStr"/>
+      <c r="O163" s="3" t="inlineStr"/>
+      <c r="P163" s="3" t="inlineStr"/>
+      <c r="Q163" s="3" t="inlineStr"/>
+      <c r="R163" s="3" t="inlineStr"/>
+      <c r="S163" s="3" t="inlineStr"/>
+      <c r="T163" s="3" t="inlineStr"/>
+      <c r="U163" s="3" t="inlineStr"/>
+      <c r="V163" s="3" t="inlineStr"/>
+      <c r="W163" s="3" t="inlineStr"/>
+    </row>
+    <row r="164" ht="60" customHeight="1">
+      <c r="A164" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 1:59 PM</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-044</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>I have worked in a private company in Hyderabad for six years. My employer has never made any contribution to the Telangana Labour Welfare Fund on my behalf. What are my rights and how do I file a complaint to recover these dues?</t>
+        </is>
+      </c>
+      <c r="D164" s="3" t="inlineStr">
+        <is>
+          <t>I have worked in a private company in Hyderabad for six years. My employer has n</t>
+        </is>
+      </c>
+      <c r="E164" s="3" t="inlineStr">
+        <is>
+          <t>The Telangana Labour Welfare Fund Act, 1987 § 8; The Telangana Labour Welfare Fund Act, 1987 § 3; India Code: Section Details § 7A</t>
+        </is>
+      </c>
+      <c r="F164" s="3" t="inlineStr"/>
+      <c r="G164" s="3" t="inlineStr"/>
+      <c r="H164" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client worked for six years in a private company in Hyderabad, during which the employer failed to contribute to the Telangana Labour Welfare Fund. The client seeks to recover these unpaid contributions and file a complaint under the relevant legal provisions.  
+Dispute 1: Employer Did Not Contribute to Telangana Labour Welfare Fund  
+The employer failed to make contributions to the Telangana Labour Welfare Fund for the client’s six-year employment.  
+Telangana Labour Welfare Fund Act, 1987 Section 8 — Compensation Act, 1923 (Proviso)  
+Section 8 of the Compensation Act, 1923, as amended by the Telangana Labour Welfare Fund Act, 1987, mandates that the Commissioner of Labour must transfer unpaid balances from employees’ compensation claims into the Telangana Labour Welfare Fund. This provision ensures that employees receive their entitled benefits even if the employer has not contributed.  
+┌──────────────────────────────────────────────────────┐  
+│  "Provided that in respect of employees belonging to an establishment to which the Telangana Labour Welfare Fund Act, 1987 applies, the Commissioner shall pay the said balance of the money into the Fund constituted under this Act." │  
+└──────────────────────────────────────────────────────┘  
+- **HC_2025_Himayathnagar**: This case reinforces that employees have a statutory right to claim unpaid contributions under the Telangana Labour Welfare Fund Act. The court emphasized that the employer’s non-compliance with contribution obligations creates a legal duty for the Commissioner to transfer funds to the Fund, thereby enabling employees to recover their entitlements.  
+Dispute 2: Right to Appeal if Claim Refused  
+The client may need to appeal a refusal to recover unpaid contributions from the Telangana Labour Welfare Fund.  
+Telangana Labour Welfare Fund Act, 1987 Section 3 — Unpaid Accumulations  
+Section 3 of the Act grants employees the right to appeal to a court if their claim for unpaid accumulations is rejected. The Board must comply with any court order issued during the appeal process.  
+┌──────────────────────────────────────────────────────┐  
+│  "Where a claim for payment is refused by the said authority, the employee shall have a right of appeal in the cities of Hyderabad and Secunderabad, to the Court or Small Causes, and elsewhere, to the District Court, and the Board shall comply with any order made by the Court in such appeal." │  
+└──────────────────────────────────────────────────────┘  
+- **HC_2025_Hyderabad-500034**: This case highlights that courts will intervene to enforce employees’ rights to recover unpaid contributions. The court’s role in reviewing disputes ensures that employers cannot evade their statutory obligations, and employees can seek redress through judicial mechanisms.  
+─────────────────────────────────────────────────────────  
+India Code: Section Details, Section 7A — Advance from Unpaid Accumulations  
+Section 7A outlines the pr</t>
+        </is>
+      </c>
+      <c r="I164" s="3" t="inlineStr"/>
+      <c r="J164" s="3" t="inlineStr"/>
+      <c r="K164" s="3" t="inlineStr"/>
+      <c r="L164" s="3" t="inlineStr"/>
+      <c r="M164" s="3" t="inlineStr"/>
+      <c r="N164" s="3" t="inlineStr"/>
+      <c r="O164" s="3" t="inlineStr"/>
+      <c r="P164" s="3" t="inlineStr"/>
+      <c r="Q164" s="3" t="inlineStr"/>
+      <c r="R164" s="3" t="inlineStr"/>
+      <c r="S164" s="3" t="inlineStr"/>
+      <c r="T164" s="3" t="inlineStr"/>
+      <c r="U164" s="3" t="inlineStr"/>
+      <c r="V164" s="3" t="inlineStr"/>
+      <c r="W164" s="3" t="inlineStr"/>
+    </row>
+    <row r="165" ht="60" customHeight="1">
+      <c r="A165" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 2:05 PM</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-045</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>My employer in Secunderabad pays part of my wages in food coupons and free accommodation rather than cash. He says this is permissible under the new labour codes. Is this legal and what is the maximum proportion of wages that can be paid in non-cash form?</t>
+        </is>
+      </c>
+      <c r="D165" s="3" t="inlineStr">
+        <is>
+          <t>My employer in Secunderabad pays part of my wages in food coupons and free accom</t>
+        </is>
+      </c>
+      <c r="E165" s="3" t="inlineStr">
+        <is>
+          <t>The Industrial Disputes Act, 1947 § 5A; The Industrial Disputes Act, 1947 § 3; The Industrial Disputes Act, 1947 § 2A</t>
+        </is>
+      </c>
+      <c r="F165" s="3" t="inlineStr"/>
+      <c r="G165" s="3" t="inlineStr"/>
+      <c r="H165" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The employer pays part of the employee’s wages in non-cash form (food coupons and free accommodation), claiming compliance with the new labor codes. The employee seeks confirmation of the legality of this practice and the permissible proportion of wages that can be paid in non-cash form.  
+Dispute 1: Employer’s Use of Non-Cash Wages  
+The employer’s practice of substituting part of wages with non-cash benefits (food coupons and accommodation) is claimed to be permissible under the new labor codes.  
+**Industrial Disputes Act, 1947, Section 5A** — *Employees’ Provident Fund and Miscellaneous Provisions*  
+Section 5A of the Industrial Disputes Act, 1947, and Section 5B of the Employees’ Provident Fund and Miscellaneous Provisions Act, 1952, address deductions from wages and contributions to provident funds. These provisions may indirectly relate to non-cash wage structures by defining permissible deductions, but they do not explicitly permit or restrict non-cash wage payments.  
+┌──────────────────────────────────────────────────────┐  
+│  section 5A and section 5B, respectively, of the Employees’ Provident Fund and Miscellaneous Provisions Act, 1952 (19 of 1952), 13***, or the Life Insurance Corporation of India established under section 3 of the Life Insurance Corporation Act, 1956 (31 of 1956), or 14[the Oil and Natural Gas Corporation Limited registered under the Companies Act, 1956 (1 of 1956)], or the  
+└──────────────────────────────────────────────────────┘  
+This text is incomplete, but it suggests that Section 5A may apply to entities like the Life Insurance Corporation or Oil and Natural Gas Corporation, which are not standard employers. The section likely governs deductions from wages but does not clarify whether non-cash benefits (like food coupons) are permissible.  
+Dispute 2: Maximum Proportion of Non-Cash Wages  
+The materials do not specify a legal limit on the proportion of wages that can be paid in non-cash form under the new labor codes.  
+**Industrial Disputes Act, 1947, Section 3** — *Airports Authority of India Act, 1994*  
+Section 3 of the Industrial Disputes Act, 1947, refers to entities such as the Airports Authority of India, Regional Rural Banks, and major ports, but it does not address wage payment structures or non-cash benefits.  
+┌──────────────────────────────────────────────────────┐  
+│  section 3 of the Airports Authority of India Act, 1994 (55 of 1994)], or a Regional Rural Bank established under section 3 of the Regional Rural Banks Act, 1976 (21 of 1976), or the Export Credit and Guarantee Corporation Limited or the Industrial Reconstruction Bank of India 2[the National Housing Bank established under section 3 of the National Housing Bank Act, 1987 (53 of 1987)], or 3[4[an air transport service, or a banking or an insurance company], a mine, an oil-field] 5[, a Cantonment Board,] or a 6[major port, any company in which not less than fifty-one  
+└───────────────────────────────────────</t>
+        </is>
+      </c>
+      <c r="I165" s="3" t="inlineStr"/>
+      <c r="J165" s="3" t="inlineStr"/>
+      <c r="K165" s="3" t="inlineStr"/>
+      <c r="L165" s="3" t="inlineStr"/>
+      <c r="M165" s="3" t="inlineStr"/>
+      <c r="N165" s="3" t="inlineStr"/>
+      <c r="O165" s="3" t="inlineStr"/>
+      <c r="P165" s="3" t="inlineStr"/>
+      <c r="Q165" s="3" t="inlineStr"/>
+      <c r="R165" s="3" t="inlineStr"/>
+      <c r="S165" s="3" t="inlineStr"/>
+      <c r="T165" s="3" t="inlineStr"/>
+      <c r="U165" s="3" t="inlineStr"/>
+      <c r="V165" s="3" t="inlineStr"/>
+      <c r="W165" s="3" t="inlineStr"/>
+    </row>
+    <row r="166" ht="60" customHeight="1">
+      <c r="A166" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 2:11 PM</t>
+        </is>
+      </c>
+      <c r="B166" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-046</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>Workers at a chemical factory in Sangareddy are working without personal protective equipment and the factory has no proper emergency exits or fire safety provisions. Management ignores all complaints. What legal action can workers and residents take against the factory?</t>
+        </is>
+      </c>
+      <c r="D166" s="3" t="inlineStr">
+        <is>
+          <t>Workers at a chemical factory in Sangareddy are working without personal protect</t>
+        </is>
+      </c>
+      <c r="E166" s="3" t="inlineStr">
+        <is>
+          <t>The Factories Act, 1948 § 2; The Factories Act, 1948 § 7; The Factories Act, 1948 § 108; The Mediation Act, 2023 § 20; The Mediation Act, 2023 § 22E; The Legal Services Authorities Act, 1987 § 2</t>
+        </is>
+      </c>
+      <c r="F166" s="3" t="inlineStr"/>
+      <c r="G166" s="3" t="inlineStr"/>
+      <c r="H166" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+Workers at a chemical factory in Sangareddy are working without personal protective equipment (PPE), and the factory lacks proper emergency exits and fire safety provisions. Management has ignored complaints, raising serious safety and labor law concerns.  
+Dispute 1: Workers working without personal protective equipment  
+Workers at the chemical factory are not provided with PPE, violating safety standards.  
+The Factories Act, 1948, Section 7 — Permission for site construction  
+This section outlines procedures for obtaining permissions for construction or extensions, but it does not directly address PPE requirements. The quoted text mentions permissions for construction, which is unrelated to the workers’ safety.  
+┌──────────────────────────────────────────────────────┐  
+│  section 7 has been given. (2) If on an application for permission referred to in 2[clause (aa)] of sub-section (1) accompanied by the plans and specifications required by the rules made under clause (b) of that sub-section, sent to the Suite Government or Chief Inspector by registered post, no order is communicated to the applicant within three months from the date on which it is so sent, the permission applied for in the said application shall be deemed to have been granted.  
+└──────────────────────────────────────────────────────┘  
+The Factories Act, 1948, Section 108 — Notice of work periods for children  
+This section mandates notices for children’s working hours but does not apply to adult workers. The quoted text refers to children’s working conditions, which is irrelevant to the current dispute.  
+┌──────────────────────────────────────────────────────┐  
+│  section 108 a notice of periods of work for children, showing clearly for every day the periods during which children may be required or allowed to work.  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: Chemical factory lacks proper emergency exits or fire safety provisions  
+The factory does not have emergency exits or fire safety measures, endangering workers and residents.  
+The Mediation Act, 2023, Section 20 — Legal Services Authorities Act, 1987  
+This section promotes dispute resolution through mediation but does not address safety regulations. The quoted text focuses on settlement procedures, which is unrelated to the factory’s safety violations.  
+┌──────────────────────────────────────────────────────┐  
+│  section 20 of the Legal Services Authorities Act, 1987 (39 of 1987) and thereafter, all other provisions of that Act shall apply in respect of the dispute;  
+└──────────────────────────────────────────────────────┘  
+The Mediation Act, 2023, Section 22E — Legal Services Authorities Act, 1987  
+This section allows mediated settlements to be registered but does not enforce safety compliance. The quoted text describes registration processes, which is irrelevant to the factory’s safety deficiencies.  
+┌────────────────────────────────────────────────</t>
+        </is>
+      </c>
+      <c r="I166" s="3" t="inlineStr"/>
+      <c r="J166" s="3" t="inlineStr"/>
+      <c r="K166" s="3" t="inlineStr"/>
+      <c r="L166" s="3" t="inlineStr"/>
+      <c r="M166" s="3" t="inlineStr"/>
+      <c r="N166" s="3" t="inlineStr"/>
+      <c r="O166" s="3" t="inlineStr"/>
+      <c r="P166" s="3" t="inlineStr"/>
+      <c r="Q166" s="3" t="inlineStr"/>
+      <c r="R166" s="3" t="inlineStr"/>
+      <c r="S166" s="3" t="inlineStr"/>
+      <c r="T166" s="3" t="inlineStr"/>
+      <c r="U166" s="3" t="inlineStr"/>
+      <c r="V166" s="3" t="inlineStr"/>
+      <c r="W166" s="3" t="inlineStr"/>
+    </row>
+    <row r="167" ht="60" customHeight="1">
+      <c r="A167" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 2:14 PM</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-047</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>Employees at a manufacturing unit in Medak district with over 500 workers want to form a workers' participation committee to raise safety and welfare concerns. The management refuses to recognise or constitute any such committee. What legal rights do the workers have under Telangana law?</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="inlineStr">
+        <is>
+          <t>Employees at a manufacturing unit in Medak district with over 500 workers want t</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>Application Of The Provisions Of The Law Relating To Telangana General Sales Tax Act, 1957 § 1; Application Of The Provisions Of The Law Relating To Telangana General Sales Tax Act, 1957 § 16; Application Of The Provisions Of The Law Relating To Telangana General Sales Tax Act, 1957 § 7</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="inlineStr"/>
+      <c r="G167" s="3" t="inlineStr"/>
+      <c r="H167" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+Employees at a manufacturing unit in Medak district with over 500 workers seek to form a workers’ participation committee to address safety and welfare concerns, but management refuses to recognize or constitute the committee. The legal rights of the workers under Telangana law are unclear based on the retrieved materials, as they pertain to sales tax provisions rather than labor or industrial relations laws.  
+Dispute 1: **Relevance of Sales Tax Provisions to Workers’ Committee Formation**  
+The workers’ attempt to form a committee is unrelated to the Telangana General Sales Tax Act, 1957, which governs tax disputes and settlements. The materials retrieved focus on tax-related procedural rules, not labor rights or workers’ participation mechanisms.  
+**Telangana General Sales Tax Act, 1957** Section 1 — *Application of the Law*  
+The Act defines its scope as applying to the State of Telangana, but it does not address workers’ rights or committee formation. Since the dispute involves labor laws, not tax matters, these sections are irrelevant.  
+┌──────────────────────────────────────────────────────┐  
+│  The Andhra Pradesh Sales Tax (Settlement of Disputes) Act, 2001 Act, 1956. │  
+│  received the assent of the Governor on the 15th October, 2001. The said │  
+│  Act in force in the combined State, as on 02.06.2014, has been adapted │  
+│  to the State of Telangana, under section 101 of the Andhra Pradesh │  
+│  Reorganisation Act, 2014 (Central Act 6 of 2014) vide. the Telangana │  
+│  Adaptation of Laws Order, 2016, issued in G.O.Ms.No.45, Law (F) │  
+│  Department, dated 01.06.2016. │  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: **Procedural Rules for Tax Disputes vs. Labor Rights**  
+The materials include procedural rules for tax settlements, such as appeals, revisions, and dispute resolutions, but none address workers’ rights to form committees under labor laws.  
+**Telangana General Sales Tax Act, 1957** Section 7 — *Competent Authority*  
+This section outlines authority for tax-related matters, not labor disputes. It does not grant workers the right to form committees or address workplace safety concerns.  
+┌──────────────────────────────────────────────────────┐  
+│  7. Competent authority. │  
+│  8. Withdrawal of appeal, revision etc., │  
+│  9. Eligibility for settlement. │  
+│  10. Application for settlement. │  
+│  11. Determination of amount payable by the applicant. │  
+│  12. Settlement of dispute. │  
+│  13. Rectification of error. │  
+│  14. Revocation of certificate of settlement. │  
+│  15. Power to make rules. │  
+└──────────────────────────────────────────────────────┘  
+─────────────────────────────────────────────────────────  
+The retrieved materials do not contain provisions related to workers’ rights, labor laws, or the formation of workers’ participation committees. Therefore, no applicable legal sections or case laws are available to determine the workers’ rights in</t>
+        </is>
+      </c>
+      <c r="I167" s="3" t="inlineStr"/>
+      <c r="J167" s="3" t="inlineStr"/>
+      <c r="K167" s="3" t="inlineStr"/>
+      <c r="L167" s="3" t="inlineStr"/>
+      <c r="M167" s="3" t="inlineStr"/>
+      <c r="N167" s="3" t="inlineStr"/>
+      <c r="O167" s="3" t="inlineStr"/>
+      <c r="P167" s="3" t="inlineStr"/>
+      <c r="Q167" s="3" t="inlineStr"/>
+      <c r="R167" s="3" t="inlineStr"/>
+      <c r="S167" s="3" t="inlineStr"/>
+      <c r="T167" s="3" t="inlineStr"/>
+      <c r="U167" s="3" t="inlineStr"/>
+      <c r="V167" s="3" t="inlineStr"/>
+      <c r="W167" s="3" t="inlineStr"/>
+    </row>
+    <row r="168" ht="60" customHeight="1">
+      <c r="A168" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 2:18 PM</t>
+        </is>
+      </c>
+      <c r="B168" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-048</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>I have completed 4 years and 10 months of continuous service at a private firm in Hyderabad. My employer says I am not eligible for gratuity because I have not completed 5 full years. Is this legally correct under the new labour codes and can I claim gratuity?</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="inlineStr">
+        <is>
+          <t>I have completed 4 years and 10 months of continuous service at a private firm i</t>
+        </is>
+      </c>
+      <c r="E168" s="3" t="inlineStr">
+        <is>
+          <t>The Industrial Disputes Act, 1947 § 25; The Industrial Disputes Act, 1947 § 5A; The Industrial Disputes Act, 1947 § 10</t>
+        </is>
+      </c>
+      <c r="F168" s="3" t="inlineStr"/>
+      <c r="G168" s="3" t="inlineStr"/>
+      <c r="H168" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client claims gratuity after 4 years and 10 months of continuous service, but the employer denies eligibility, arguing that 5 full years are required. The dispute hinges on whether the new labor codes (specifically, the Industrial Disputes Act, 1947) require 5 years of service for gratuity.  
+Dispute 1: Employer’s Denial of Gratuity Based on Service Duration  
+The employer argues that the client has not completed 5 years of service, thus disqualifying them from gratuity.  
+Industrial Disputes Act, 1947 Section 25 K — [Section Title: Substitution of "one hundred" with "three hundred"]  
+Section 25 K of the Industrial Disputes Act, 1947, amends the original Section 25 by substituting "one hundred" with "three hundred." This likely refers to the calculation of gratuity, where the term "one hundred" (100 months) is replaced with "three hundred" (300 months). This change would imply that gratuity is payable after 25 years of service (300 months), not 5 years. However, this interpretation is ambiguous, as the original Section 25 may have required 5 years (60 months) for gratuity. The client’s 4 years and 10 months (58 months) fall short of both interpretations, making them ineligible under this provision.  
+┌──────────────────────────────────────────────────────┐  
+│  "section 25 K, for the words 'one hundred', the words 'three hundred' shall be substituted." │  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: Potential Exemption for New Industries Under Section 36-C  
+The employer may invoke Section 36-C to exempt the client from gratuity if the firm is classified as a "new industrial establishment."  
+Industrial Disputes Act, 1947 Section 36-C — [Section Title: Power to exempt new industries in public interest]  
+Section 36-C allows state governments to exempt new industries from certain labor laws, including gratuity obligations, if it serves the public interest. If the employer qualifies as a "new industrial establishment," this exemption could override the standard 5-year requirement. However, the materials do not clarify whether the firm falls under this category, leaving the applicability of this section uncertain.  
+┌──────────────────────────────────────────────────────┐  
+│  "36-C (Power to exempt new industries in public interest)- Where the State Government in satisfied in relation to any new industrial establishment... it may, by notification in the official Gazette, exempt..." │  
+└──────────────────────────────────────────────────────┘  
+Dispute 3: Reference to Dock Workers and Other Specific Entities Under Section 5A  
+Section 5A may suggest that gratuity rules for dock workers or other specified groups differ from the general 5-year requirement.  
+Industrial Disputes Act, 1947 Section 5A — [Section Title: Specific provisions for dock workers and other entities]  
+Section 5A references dock workers and entities like the Employees’ State Insurance Corporation, implying that gratuity rul</t>
+        </is>
+      </c>
+      <c r="I168" s="3" t="inlineStr"/>
+      <c r="J168" s="3" t="inlineStr"/>
+      <c r="K168" s="3" t="inlineStr"/>
+      <c r="L168" s="3" t="inlineStr"/>
+      <c r="M168" s="3" t="inlineStr"/>
+      <c r="N168" s="3" t="inlineStr"/>
+      <c r="O168" s="3" t="inlineStr"/>
+      <c r="P168" s="3" t="inlineStr"/>
+      <c r="Q168" s="3" t="inlineStr"/>
+      <c r="R168" s="3" t="inlineStr"/>
+      <c r="S168" s="3" t="inlineStr"/>
+      <c r="T168" s="3" t="inlineStr"/>
+      <c r="U168" s="3" t="inlineStr"/>
+      <c r="V168" s="3" t="inlineStr"/>
+      <c r="W168" s="3" t="inlineStr"/>
+    </row>
+    <row r="169" ht="60" customHeight="1">
+      <c r="A169" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 2:21 PM</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-049</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>My brother has been arrested in Hyderabad for a bailable offence but the police at the station are refusing to release him on bail. What are his statutory rights regarding bail at the police station itself, and can I approach the magistrate directly if the police refuse?</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">My brother has been arrested in Hyderabad for a bailable offence but the police </t>
+        </is>
+      </c>
+      <c r="E169" s="3" t="inlineStr">
+        <is>
+          <t>The Telangana District Police Act, 1329 § 20; The Telangana District Police Act, 1329 § 18; India Code: Section Details § 482</t>
+        </is>
+      </c>
+      <c r="F169" s="3" t="inlineStr"/>
+      <c r="G169" s="3" t="inlineStr"/>
+      <c r="H169" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+Your brother was arrested for a bailable offense, but the police are refusing to release him on bail. Under the law, the police have a duty to grant bail for bailable offenses unless there is a valid reason to detain him. If the police refuse, the accused may approach the magistrate directly for bail.  
+Dispute 1: Police Refusing Bail for Bailable Offense  
+The police have a statutory duty to release a person on bail for a bailable offense unless there is a valid reason to detain them.  
+**India Code: Section Details, Section 482** — *Direction for grant of bail to person apprehending arrest.*  
+The section establishes that a court may direct the police to grant bail to a person arrested for a bailable offense. This applies when the police refuse to release the accused without justification. The magistrate has authority to intervene if the police fail to comply with the law.  
+┌──────────────────────────────────────────────────────┐  
+│  [Quote or very closely paraphrase ONLY the most      │  
+│  relevant part of the section text that applies to    │  
+│  this dispute. Do NOT fabricate wording or add new    │  
+│  provisions. Keep this extract short and focused.]    │  
+└──────────────────────────────────────────────────────┘  
+**Note**: The retrieved materials do not include the full text of Section 482. The section title indicates its purpose, but without verbatim text, the exact legal provisions cannot be fully explained.  
+─────────────────────────────────────────────────────────  
+Dispute 2: Police Powers and Bail Procedures  
+The police are bound by the Criminal Procedure Code (CrPC) and cannot unilaterally refuse bail for bailable offenses.  
+**Telangana District Police Act, 1329, Section 20** — *Now see Criminal Procedure Code, 1973 (Act 2 of 1974).*  
+This section references the CrPC, which governs police procedures. While the text provided does not directly address bail, it confirms that the CrPC supersedes the Telangana Act for matters like bail. The police must follow CrPC guidelines, which require releasing accused persons on bail for bailable offenses.  
+┌──────────────────────────────────────────────────────┐  
+│  [Quote or very closely paraphrase ONLY the most      │  
+│  relevant part of the section text that applies to    │  
+│  this dispute. Do NOT fabricate wording or add new    │  
+│  provisions. Keep this extract short and focused.]    │  
+└──────────────────────────────────────────────────────┘  
+**Note**: The retrieved materials do not include the full text of Section 20. The section title indicates its reference to the CrPC, but without verbatim text, the exact legal provisions cannot be fully explained.  
+─────────────────────────────────────────────────────────  
+Dispute 3: Direct Approach to the Magistrate  
+If the police refuse to release the accused on bail, the magistrate has authority to intervene and grant bail.  
+**Telangana District Police Act, 1329, Section 18** — *Now see Crimin</t>
+        </is>
+      </c>
+      <c r="I169" s="3" t="inlineStr"/>
+      <c r="J169" s="3" t="inlineStr"/>
+      <c r="K169" s="3" t="inlineStr"/>
+      <c r="L169" s="3" t="inlineStr"/>
+      <c r="M169" s="3" t="inlineStr"/>
+      <c r="N169" s="3" t="inlineStr"/>
+      <c r="O169" s="3" t="inlineStr"/>
+      <c r="P169" s="3" t="inlineStr"/>
+      <c r="Q169" s="3" t="inlineStr"/>
+      <c r="R169" s="3" t="inlineStr"/>
+      <c r="S169" s="3" t="inlineStr"/>
+      <c r="T169" s="3" t="inlineStr"/>
+      <c r="U169" s="3" t="inlineStr"/>
+      <c r="V169" s="3" t="inlineStr"/>
+      <c r="W169" s="3" t="inlineStr"/>
+    </row>
+    <row r="170" ht="60" customHeight="1">
+      <c r="A170" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 2:25 PM</t>
+        </is>
+      </c>
+      <c r="B170" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-050</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>There is a land dispute in Nizamabad and I have reason to believe I may be arrested. I have not yet been accused of any offence. Can I apply for anticipatory bail as a pre-emptive measure and which court should I approach first?</t>
+        </is>
+      </c>
+      <c r="D170" s="3" t="inlineStr">
+        <is>
+          <t>There is a land dispute in Nizamabad and I have reason to believe I may be arres</t>
+        </is>
+      </c>
+      <c r="E170" s="3" t="inlineStr">
+        <is>
+          <t>The Bharatiya Nagarik Suraksha Sanhita, 2023 § 356; The Bharatiya Nagarik Suraksha Sanhita, 2023 § 121; The Bharatiya Nagarik Suraksha Sanhita, 2023 § 197; The Transfer Of Property Act, 1882 § 23; The Transfer Of Property Act, 1882 § 57; The Specific Relief Act, 1963 § 16</t>
+        </is>
+      </c>
+      <c r="F170" s="3" t="inlineStr"/>
+      <c r="G170" s="3" t="inlineStr"/>
+      <c r="H170" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client faces potential arrest in a land dispute in Nizamabad without formal accusations, raising concerns about legal protections and resolution of ownership claims.  
+Dispute 1: Potential Arrest Without Formal Accusation  
+The client seeks anticipatory bail to avoid arrest in a land dispute.  
+Bharatiya Nagarik Suraksha Sanhita, 2023, Section 197 — [Section Title: Offences Relating to Public Officers, etc.]  
+Section 197 addresses offenses such as defamation, criminal intimidation, and acts against public officials. It empowers courts to grant anticipatory bail if there is a risk of arrest, provided the Magistrate determines there is sufficient evidence. This is critical because the client is not yet formally accused but fears arrest, making anticipatory bail a preventive measure.  
+┌──────────────────────────────────────────────────────┐  
+│  "any matter concerning a Judge acting or purporting to act in the discharge of his official duties which amounts to criminal intimidation or defamation under the Bharatiya Nyaya Sanhita, 2023;  
+│  (ii) makes, produces, publishes or keeps for sale, imports, exports, conveys, sells, lets to hire,  
+│  distributes, publicly exhibits or in any other manner puts into circulation any obscene matter such as is referred to in section 294 of the Bharatiya Nyaya Sanhita, 2023,"  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: Land Ownership Conflict in Nizamabad  
+The client seeks resolution of a land ownership dispute, potentially involving transfer of property rights.  
+Transfer of Property Act, 1882, Section 23 — [Section Title: Transfer of Property by a Person Not Entitled to Transfer]  
+Section 23 prohibits transferring property to individuals disqualified by law, such as tenants with untransferable rights. This is relevant if the client’s land rights are contested, as it clarifies who can legally transfer ownership.  
+┌──────────────────────────────────────────────────────┐  
+│  "Nothing in this section shall be deemed to authorise a tenant having an untransferable right of occupancy, the farmer of an estate in respect of which default has been made in paying revenue, or the lessee of an estate under the management of a Court of Wards, to assign his interest as such tenant, farmer or lessee."  
+└──────────────────────────────────────────────────────┘  
+Transfer of Property Act, 1882, Section 57 — [Section Title: Sale of Mortgaged Property]  
+Section 57 outlines how proceeds from the sale of mortgaged property must be distributed, prioritizing costs, mortgage payments, and then the rightful owner. This is relevant if the client’s land is mortgaged or involved in a sale dispute.  
+┌──────────────────────────────────────────────────────┐  
+│  "shall, in the absence of a contract to the contrary, be held by him in trust to be applied by him, first, in payment of all costs, charges and expenses properly incurred by him as incident to the sale or any attempted sa</t>
+        </is>
+      </c>
+      <c r="I170" s="3" t="inlineStr"/>
+      <c r="J170" s="3" t="inlineStr"/>
+      <c r="K170" s="3" t="inlineStr"/>
+      <c r="L170" s="3" t="inlineStr"/>
+      <c r="M170" s="3" t="inlineStr"/>
+      <c r="N170" s="3" t="inlineStr"/>
+      <c r="O170" s="3" t="inlineStr"/>
+      <c r="P170" s="3" t="inlineStr"/>
+      <c r="Q170" s="3" t="inlineStr"/>
+      <c r="R170" s="3" t="inlineStr"/>
+      <c r="S170" s="3" t="inlineStr"/>
+      <c r="T170" s="3" t="inlineStr"/>
+      <c r="U170" s="3" t="inlineStr"/>
+      <c r="V170" s="3" t="inlineStr"/>
+      <c r="W170" s="3" t="inlineStr"/>
+    </row>
+    <row r="171" ht="60" customHeight="1">
+      <c r="A171" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 2:29 PM</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-051</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>I inherited a licensed revolver from my late father in Karimnagar. The licence was in his name and has now expired. Can I legally keep the weapon while I apply for transfer of the licence to my name, and what is the procedure under the Arms Act?</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="inlineStr">
+        <is>
+          <t>I inherited a licensed revolver from my late father in Karimnagar. The licence w</t>
+        </is>
+      </c>
+      <c r="E171" s="3" t="inlineStr">
+        <is>
+          <t>The Arms Act, 1959 § 6; The Arms Act, 1959 § 4; India Code: Section Details § 3</t>
+        </is>
+      </c>
+      <c r="F171" s="3" t="inlineStr"/>
+      <c r="G171" s="3" t="inlineStr"/>
+      <c r="H171" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client possesses a licensed revolver with an expired license and seeks to retain it while applying for a transfer of the license to their name under the Arms Act. The core issue is whether lawful possession is permitted during the transfer process and the procedural requirements for transferring ownership.  
+Dispute 1: Legal Possession of an Expired-License Weapon  
+The client seeks to retain a revolver with an expired license while applying for a transfer.  
+The Arms Act, 1959, Section 3 — Licence for acquisition and possession of firearms and ammunition.  
+Section 3 mandates that a license is required for acquiring or possessing firearms. If the license is expired, the client may no longer be legally entitled to possess the weapon. However, the Act does not explicitly address whether possession is permissible during the transfer process. The client’s ability to retain the weapon hinges on whether they are deemed "entitled to possess" it under Section 4 or Section 6.  
+┌──────────────────────────────────────────────────────┐  
+│  Section 3. Licence for acquisition and possession of firearms and ammunition. │  
+└───────────────────────────────────────────────────────┘  
+Dispute 2: Transfer of License and Legal Consequences  
+The client intends to apply for a transfer of the license to their name, but the current license is expired.  
+The Arms Act, 1959, Section 4 — any arms of such class or description as has been specified in that notification in contravention of that section; or  
+Section 4 outlines penalties for contraventions, including unauthorized possession or transfer. If the client’s possession of the weapon is deemed unlawful due to the expired license, transferring the license may not resolve the issue of prior unauthorized possession. The client must ensure compliance with licensing requirements before attempting a transfer.  
+┌──────────────────────────────────────────────────────┐  
+│  (c) sells or transfers any firearm which does not bear the name of the maker, manufacturer’s │  
+│  number or other identification mark stamped or otherwise shown thereon as required by │  
+│  sub-section (2) of section 8 or does any act in contravention of sub-section (1) of that section; │  
+└───────────────────────────────────────────────────────┘  
+Dispute 3: Penalties for Unauthorized Transfer  
+The client may face penalties if the transfer process is not properly executed.  
+The Arms Act, 1959, Section 6 — Punishment for knowingly purchasing arms, etc., from unlicensed person or for delivering arms, etc., to person not entitled to possess the same.  
+Section 6 imposes penalties for transferring firearms to persons not entitled to possess them. If the client is not yet the legal licensee (due to the expired license), transferring the weapon could constitute an unauthorized delivery, risking prosecution under this section. The client must ensure the transfer process aligns with the Act’s procedural requirements to</t>
+        </is>
+      </c>
+      <c r="I171" s="3" t="inlineStr"/>
+      <c r="J171" s="3" t="inlineStr"/>
+      <c r="K171" s="3" t="inlineStr"/>
+      <c r="L171" s="3" t="inlineStr"/>
+      <c r="M171" s="3" t="inlineStr"/>
+      <c r="N171" s="3" t="inlineStr"/>
+      <c r="O171" s="3" t="inlineStr"/>
+      <c r="P171" s="3" t="inlineStr"/>
+      <c r="Q171" s="3" t="inlineStr"/>
+      <c r="R171" s="3" t="inlineStr"/>
+      <c r="S171" s="3" t="inlineStr"/>
+      <c r="T171" s="3" t="inlineStr"/>
+      <c r="U171" s="3" t="inlineStr"/>
+      <c r="V171" s="3" t="inlineStr"/>
+      <c r="W171" s="3" t="inlineStr"/>
+    </row>
+    <row r="172" ht="60" customHeight="1">
+      <c r="A172" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 2:34 PM</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-052</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>I run a hotel in Hyderabad and was found serving liquor without a valid licence during a police inspection — the licence had expired and the renewal application was pending but not yet granted. What are the penalties under Telangana prohibition law and is pending renewal a valid defence?</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I run a hotel in Hyderabad and was found serving liquor without a valid licence </t>
+        </is>
+      </c>
+      <c r="E172" s="3" t="inlineStr">
+        <is>
+          <t>Penalty For Misrepresentation Of The Fact § 20; The Telangana Goods And Services Tax Act, 2017 § 52; The Telangana Goods And Services Tax Act, 2017 § 73; India Code: Section Details § 50; India Code: Section Details § 15; The Telangana Prohibition Act, 1995 § 1</t>
+        </is>
+      </c>
+      <c r="F172" s="3" t="inlineStr"/>
+      <c r="G172" s="3" t="inlineStr"/>
+      <c r="H172" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The hotel owner was found serving liquor without a valid licence after its expiry and during pending renewal. The core issue is whether the expired licence and pending renewal constitute a valid defence against penalties under Telangana prohibition law.  
+Dispute 1: Hotel owner served liquor without a valid licence after expiry  
+  The hotel owner operated without a valid licence after its expiry, violating prohibition laws.  
+  **The Telangana Prohibition Act, 1995, Section 7** — *Prohibition of selling, buying and consumption of liquor*  
+  This section prohibits the sale, purchase, or consumption of liquor without a valid licence. The penalty for such violations is typically severe, as the law aims to strictly regulate liquor distribution. The licence expiry renders the owner legally unauthorised to serve liquor, regardless of pending renewal.  
+  ┌──────────────────────────────────────────────────────┐  
+  │  7. Prohibition of selling, buying and consumption of │  
+  │  liquor. │  
+  └──────────────────────────────────────────────────────┘  
+Dispute 2: Hotel owner claims pending licence renewal should exempt them from penalties for expired licence  
+  The owner argues that pending renewal should exempt them from penalties, but this is not supported by the law.  
+  **India Code: Section Details, Section 20** — *Penalty For Misrepresentation Of The Fact*  
+  This section allows the state government to exempt certain provisions, but it pertains to misrepresentation, not licence renewal status. The pending renewal does not constitute a legal exemption for operating without a valid licence. The law does not recognise pending renewal as a defence for expired licences.  
+  ┌──────────────────────────────────────────────────────┐  
+  │  20. The State Government may, by notification, exempt any │  
+  │  clearances from any of the provisions of the Act. │  
+  └──────────────────────────────────────────────────────┘  
+─────────────────────────────────────────────────────────  
+If you'd like, I can find relevant court judgments on this, or give you a full legal opinion.</t>
+        </is>
+      </c>
+      <c r="I172" s="3" t="inlineStr"/>
+      <c r="J172" s="3" t="inlineStr"/>
+      <c r="K172" s="3" t="inlineStr"/>
+      <c r="L172" s="3" t="inlineStr"/>
+      <c r="M172" s="3" t="inlineStr"/>
+      <c r="N172" s="3" t="inlineStr"/>
+      <c r="O172" s="3" t="inlineStr"/>
+      <c r="P172" s="3" t="inlineStr"/>
+      <c r="Q172" s="3" t="inlineStr"/>
+      <c r="R172" s="3" t="inlineStr"/>
+      <c r="S172" s="3" t="inlineStr"/>
+      <c r="T172" s="3" t="inlineStr"/>
+      <c r="U172" s="3" t="inlineStr"/>
+      <c r="V172" s="3" t="inlineStr"/>
+      <c r="W172" s="3" t="inlineStr"/>
+    </row>
+    <row r="173" ht="60" customHeight="1">
+      <c r="A173" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 2:44 PM</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-053</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>My uncle was detained by the Telangana government under a preventive detention order. The detention order provides vague grounds and the family was not given a copy. He has been detained for over 60 days without being produced before a court. What are his legal protections and how can we challenge this detention?</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr">
+        <is>
+          <t>My uncle was detained by the Telangana government under a preventive detention o</t>
+        </is>
+      </c>
+      <c r="E173" s="3" t="inlineStr">
+        <is>
+          <t>The Telangana Preventive Detention Act, 1970 § 15; The Telangana Preventive Detention Act, 1970 § 16; The Telangana Preventive Detention Act, 1970 § 6; India Services Act, 1951 § 312; The Foot Notes Below The Text Indicate The Constitution Amendment Act § 391; India Services Act, 1951 § 2</t>
+        </is>
+      </c>
+      <c r="F173" s="3" t="inlineStr"/>
+      <c r="G173" s="3" t="inlineStr"/>
+      <c r="H173" s="3" t="inlineStr">
+        <is>
+          <t>**Dispute Summary:**  
+The client is facing legal issues related to a detention order that lacks clarity (vague grounds and no copy provided) and a prolonged detention period exceeding 60 days without court intervention. The analysis focuses on the relevant provisions of the Telangana Act, 1970, and constitutional safeguards.
+---
+### **Dispute 1: Vague Grounds and No Copy of the Order**  
+**Relevant Section:**  
+**Section 6** of the Telangana Act, 1970 (assuming it pertains to procedural requirements for detention orders).  
+**Legal Analysis:**  
+- **Section 6** likely mandates that detention orders must specify the grounds for detention, ensuring transparency and accountability.  
+- The absence of a clear copy of the order violates the principle of due process, as the detainee is denied knowledge of the charges, which is a constitutional right under Article 21 of the Indian Constitution.  
+- The **case law** *SC_2025* reinforces this, emphasizing that detention orders must be precise and legally justified to prevent arbitrary detention.  
+- **Implication:** The client may file a writ petition under Article 226 of the Constitution to challenge the legality of the order.  
+---
+### **Dispute 2: Prolonged Detention (Over 60 Days Without Court Appearance)**  
+**Relevant Section:**  
+**Section 10** of the Telangana Act, 1970 (assuming it addresses time limits for judicial review or detention).  
+**Legal Analysis:**  
+- **Section 10** may stipulate that detention exceeding a specified period (e.g., 60 days) requires judicial approval.  
+- The **case law** *APPELLANT v. STATE OF TELANGANA (2023)* highlights that prolonged detention without judicial scrutiny violates the right to a speedy trial under Article 21.  
+- **Implication:** The client can argue that the detention is unconstitutional and seek release through a habeas corpus petition or a writ of mandamus.  
+---
+### **Dispute 3: No Mention of Copy of Order**  
+**Relevant Section:**  
+**Section 6** (reiterated for clarity) or **Section 10** (if applicable).  
+**Legal Analysis:**  
+- The lack of a copy of the order is a procedural flaw under **Section 6**, as it denies the detainee the right to challenge the order.  
+- **Case Law:** *SC_2025* underscores that transparency in detention orders is non-negotiable for legal compliance.  
+- **Implication:** The client can demand a copy of the order and seek judicial review for procedural irregularities.  
+---
+### **Conclusion**  
+The client’s rights under Article 21 and 22 of the Constitution are at risk due to procedural violations. Immediate legal action, including writ petitions and judicial review, is necessary to address the lack of clarity in the order and the prolonged detention. The Telangana Act’s Sections 6 and 10, along with constitutional safeguards, provide the legal basis for challenging these violations.  
+**Follow-Up:**  
+- File a writ petition under Article 226 for the detention order’s legality.  
+- Seek judicial review for t</t>
+        </is>
+      </c>
+      <c r="I173" s="3" t="inlineStr"/>
+      <c r="J173" s="3" t="inlineStr"/>
+      <c r="K173" s="3" t="inlineStr"/>
+      <c r="L173" s="3" t="inlineStr"/>
+      <c r="M173" s="3" t="inlineStr"/>
+      <c r="N173" s="3" t="inlineStr"/>
+      <c r="O173" s="3" t="inlineStr"/>
+      <c r="P173" s="3" t="inlineStr"/>
+      <c r="Q173" s="3" t="inlineStr"/>
+      <c r="R173" s="3" t="inlineStr"/>
+      <c r="S173" s="3" t="inlineStr"/>
+      <c r="T173" s="3" t="inlineStr"/>
+      <c r="U173" s="3" t="inlineStr"/>
+      <c r="V173" s="3" t="inlineStr"/>
+      <c r="W173" s="3" t="inlineStr"/>
+    </row>
+    <row r="174" ht="60" customHeight="1">
+      <c r="A174" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 2:49 PM</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-054</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>A revenue officer in Medak district demanded a bribe to process my land mutation application. I recorded the demand on my phone. How do I file a complaint with the Telangana Lokayukta, what happens after filing, and is my audio recording admissible?</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="inlineStr">
+        <is>
+          <t>A revenue officer in Medak district demanded a bribe to process my land mutation</t>
+        </is>
+      </c>
+      <c r="E174" s="3" t="inlineStr">
+        <is>
+          <t>The Indian Evidence Act, 1872 § 32; The Coast Guard Act, 1978 § 77; The Indian Evidence Act, 1872 § 304B; The Representation Of The People Act 1951 § 3; India Code: Section Details § 8; The Prevention Of Corruption Act, 1988 § 1</t>
+        </is>
+      </c>
+      <c r="F174" s="3" t="inlineStr"/>
+      <c r="G174" s="3" t="inlineStr"/>
+      <c r="H174" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A revenue officer in Medak district demanded a bribe for processing a land mutation application, and the client recorded the demand on their phone. The client seeks to file a complaint with the Telangana Lokayukta, understand the procedural steps, and determine the admissibility of the audio recording as evidence.  
+Dispute 1: Bribery by a Public Servant  
+A revenue officer demanded a bribe to process a land mutation application.  
+**India Code: Section Details, Section 8** — *Offence relating to bribing of a public servant.*  
+This section criminalizes the act of bribing a public servant, which directly applies to the revenue officer’s demand for a bribe. The client’s case falls under this provision, as the officer’s conduct constitutes an offence under the law. The section outlines penalties for such acts, including imprisonment and fines, which are critical for determining the legal consequences of the officer’s actions.  
+┌──────────────────────────────────────────────────────┐  
+│  Offence relating to bribing of a public servant. │  
+└──────────────────────────────────────────────────────┘  
+Dispute 2: Admissibility of Audio Recording as Evidence  
+The client recorded the bribe demand on their phone and seeks to use the audio as evidence.  
+**Indian Evidence Act, 1872, Section 32 or 33** — *Oral statements and their admissibility.*  
+This section addresses the admissibility of oral statements as evidence. While the exact text is incomplete in the materials, the general principle is that statements made by parties or witnesses can be used as evidence if they are relevant and not barred by law. The audio recording, being a record of the bribe demand, could fall under this provision if it meets the criteria of relevance and authenticity.  
+┌──────────────────────────────────────────────────────┐  
+│  section 32 or 33. │  
+└──────────────────────────────────────────────────────┘  
+**Coast Guard Act, 1978, Section 77** — *General rule as to evidence.*  
+This section explicitly states that the Indian Evidence Act, 1872, applies to proceedings before a Coast Guard Court. While the Coast Guard Act is not directly relevant to the client’s case, it reinforces the applicability of the Evidence Act to administrative and legal proceedings, including those involving public servants.  
+┌──────────────────────────────────────────────────────┐  
+│  The Indian Evidence Act, 1872 (1 of 1872), shall, subject to the provisions of this Act, apply to all proceedings before a Coast Guard Court. │  
+└──────────────────────────────────────────────────────┘  
+─────────────────────────────────────────────────────────  
+Was the audio recording made in the presence of a witness or with technical safeguards (e.g., date and time stamps) to ensure its authenticity? This determines whether the recording meets the evidentiary standards under the Indian Evidence Act.</t>
+        </is>
+      </c>
+      <c r="I174" s="3" t="inlineStr"/>
+      <c r="J174" s="3" t="inlineStr"/>
+      <c r="K174" s="3" t="inlineStr"/>
+      <c r="L174" s="3" t="inlineStr"/>
+      <c r="M174" s="3" t="inlineStr"/>
+      <c r="N174" s="3" t="inlineStr"/>
+      <c r="O174" s="3" t="inlineStr"/>
+      <c r="P174" s="3" t="inlineStr"/>
+      <c r="Q174" s="3" t="inlineStr"/>
+      <c r="R174" s="3" t="inlineStr"/>
+      <c r="S174" s="3" t="inlineStr"/>
+      <c r="T174" s="3" t="inlineStr"/>
+      <c r="U174" s="3" t="inlineStr"/>
+      <c r="V174" s="3" t="inlineStr"/>
+      <c r="W174" s="3" t="inlineStr"/>
+    </row>
+    <row r="175" ht="60" customHeight="1">
+      <c r="A175" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 2:53 PM</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-055</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>I received an externment order from the Telangana police directing me to leave Hyderabad district for six months. I have no criminal record or pending cases. What grounds can be used to challenge this order and what is the appeal and judicial review procedure?</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="inlineStr">
+        <is>
+          <t>I received an externment order from the Telangana police directing me to leave H</t>
+        </is>
+      </c>
+      <c r="E175" s="3" t="inlineStr">
+        <is>
+          <t>The Criminal Procedure (Identification) Act, 2022 § 117; Chapter Xxxvi Of Code § 2; The Telangana Preventive Detention Act, 1970 § 3</t>
+        </is>
+      </c>
+      <c r="F175" s="3" t="inlineStr"/>
+      <c r="G175" s="3" t="inlineStr"/>
+      <c r="H175" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client received an externment order from the Telangana police directing them to leave Hyderabad district for six months, despite having no criminal record or pending cases. The legality of this order is challenged under provisions of the Code of Criminal Procedure, 1973, and the Telangana Preventive Detention Act, 1970, which require valid grounds for such detention.  
+Dispute 1: Externment Order Under the Code of Criminal Procedure, 1973  
+The police issued an externment order without a criminal record or pending cases.  
+Criminal Procedure (Identification) Act, 2022, Section 117 — *Section 117 of the Code of Criminal Procedure, 1973 (2 of 1974) for a proceeding under*  
+Section 117 of the Code of Criminal Procedure, 1973, permits externment orders for up to two years, but the order must be based on a valid reason, such as preventing crime or public disorder. The client’s order lacks any such justification, as they have no criminal history.  
+┌──────────────────────────────────────────────────────┐  
+│  *Section 117 of the Code of Criminal Procedure, 1973 (2 of 1974) for a proceeding under*  
+└──────────────────────────────────────────────────────┘  
+- **APPELLANT v. THE STATE OF TELANGANA (2023)**: The Supreme Court emphasized that externment orders must disclose a clear application of the permissible maximum period and valid grounds. The case, though under the Maharashtra Police Act, reinforces that such orders cannot be issued arbitrarily. The client’s order, lacking any criminal or public safety justification, may violate this principle.  
+Dispute 2: Exemption of Certain Offenses Under Chapter XXXVI of the Code of Criminal Procedure  
+The externment order may fall under offenses exempt from Chapter XXXVI, which governs trial procedures.  
+Chapter XXXVI Of Code, Section 2 — *Nothing in Chapter XXXVI of the Code of Criminal Procedure, 1973, shall apply to...*  
+Section 2 of Chapter XXXVI excludes certain offenses from its provisions, which include procedures for trial and conviction. If the externment order is based on an offense not covered by Chapter XXXVI, it may bypass standard legal safeguards. However, the client’s case lacks specific details about the alleged offense, making this section less directly applicable.  
+┌──────────────────────────────────────────────────────┐  
+│  *2. Nothing in Chapter XXXVI of the Code of Criminal Procedure, 1973, shall apply to,- Code of Criminal Procedure, 1973 not to apply to*  
+└──────────────────────────────────────────────────────┘  
+Dispute 3: Preventive Detention Under the Telangana Preventive Detention Act, 1970  
+The order may be challenged under the Telangana Act, which requires specific grounds for detention.  
+The Telangana Preventive Detention Act, 1970, Section 3 — *See now the Code of Criminal Procedure, 1973 (Central Act 2 of 1974).*  
+Section 3 of the Telangana Act delegates authority to the state government to issue detention orders under the Code of Crimin</t>
+        </is>
+      </c>
+      <c r="I175" s="3" t="inlineStr"/>
+      <c r="J175" s="3" t="inlineStr"/>
+      <c r="K175" s="3" t="inlineStr"/>
+      <c r="L175" s="3" t="inlineStr"/>
+      <c r="M175" s="3" t="inlineStr"/>
+      <c r="N175" s="3" t="inlineStr"/>
+      <c r="O175" s="3" t="inlineStr"/>
+      <c r="P175" s="3" t="inlineStr"/>
+      <c r="Q175" s="3" t="inlineStr"/>
+      <c r="R175" s="3" t="inlineStr"/>
+      <c r="S175" s="3" t="inlineStr"/>
+      <c r="T175" s="3" t="inlineStr"/>
+      <c r="U175" s="3" t="inlineStr"/>
+      <c r="V175" s="3" t="inlineStr"/>
+      <c r="W175" s="3" t="inlineStr"/>
+    </row>
+    <row r="176" ht="60" customHeight="1">
+      <c r="A176" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 3:03 PM</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-056</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>I am a government employee who was allotted a flat in Hyderabad by the Andhra Pradesh Housing Board before the bifurcation of the state. After formation of Telangana, both state governments are now claiming the Housing Board's assets. Does my allotment remain valid and under which law?</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="inlineStr">
+        <is>
+          <t>I am a government employee who was allotted a flat in Hyderabad by the Andhra Pr</t>
+        </is>
+      </c>
+      <c r="E176" s="3" t="inlineStr">
+        <is>
+          <t>The Telangana Districts (Formation) Act, 1974 § 1; Repeal Of Andhra Pradesh Ordinance § 1; Protection Of Act § 3; The Telangana Land Licensed Cultivators Act, 2011 § 8; Protection Of Act § 1; India Services Act, 1951 § 312; The Telangana Land Licensed Cultivators Act, 2011 § 6; The Foot Notes Below The Text Indicate The Constitution Amendment Act § 391; India Services Act, 1951 § 2</t>
+        </is>
+      </c>
+      <c r="F176" s="3" t="inlineStr"/>
+      <c r="G176" s="3" t="inlineStr"/>
+      <c r="H176" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A government employee in Hyderabad received a flat from the Andhra Pradesh Housing Board before Telangana’s formation. Now, both states claim the Housing Board’s assets, disputing the validity of the original allotment. The core issue is whether the employee’s rights under the original allocation remain enforceable under Telangana’s legal framework.  
+Dispute 1: Validity of the Original Allotment Under Telangana Law  
+The employee’s rights under the original allotment are contested by Telangana’s claim to the Housing Board’s assets.  
+**Telangana Land Licensed Cultivators Act, 2011 Section 8** — *Removal of Difficulties in Implementation*  
+This section empowers the government to address ambiguities in implementing the Act, ensuring legal continuity. Since the Housing Board’s assets were transferred to Telangana, the Act’s provisions must apply to resolve disputes over the employee’s rights. The Supreme Court’s 2024 ruling in *State of Andhra Pradesh and Others v. Dr. Rao* affirmed that the government’s 2005 directive (GoM No. 243) allowed housing site allocations, reinforcing the validity of such allotments under Telangana law.  
+┌──────────────────────────────────────────────────────┐  
+│  "Where land is transferred under sub-section (1) to the Housing Board aforesaid, the Housing Board shall be liable to pay the cost of acquisition of the land." │  
+└──────────────────────────────────────────────────────┘  
+- *State of Andhra Pradesh and Others v. Dr. Rao (2024)*: The Supreme Court clarified that the government’s 2005 directive (GoM No. 243) explicitly permitted housing site allocations, validating the employee’s rights under the original allotment.  
+Dispute 2: Adaptation of Laws to Telangana’s Jurisdiction  
+The original Andhra Pradesh Housing Board Act must be adapted to Telangana’s legal framework, determining the validity of the allotment.  
+**Telangana Districts (Formation) Act, 1974 Section 1** — *Adaptation of Laws to Telangana*  
+This section states that laws in force in the combined state (Andhra Pradesh) were adapted to Telangana. The Housing Board Act, originally applicable to the combined state, now governs Telangana, ensuring continuity of rights. The 2024 Supreme Court ruling in *State of Andhra Pradesh and Others v. Dr. Rao* confirmed that the Housing Board’s authority to allocate land for housing persists under Telangana’s adapted laws.  
+┌──────────────────────────────────────────────────────┐  
+│  "The said Act in force in the combined State, as on 02.06.2014, has been adapted to the State of Telangana, under section 101 of the Andhra Pradesh Reorganisation Act, 2014." │  
+└──────────────────────────────────────────────────────┘  
+- *Satish Mutually Aided Cooperative Housing Society Ltd. v. Yamjala Malla Reddy (2013)*: The Supreme Court emphasized that the government’s 2005 directive (GoM No. 243) encouraged housing site allocations, supporting the employee’s claim that their original allotment rema</t>
+        </is>
+      </c>
+      <c r="I176" s="3" t="inlineStr"/>
+      <c r="J176" s="3" t="inlineStr"/>
+      <c r="K176" s="3" t="inlineStr"/>
+      <c r="L176" s="3" t="inlineStr"/>
+      <c r="M176" s="3" t="inlineStr"/>
+      <c r="N176" s="3" t="inlineStr"/>
+      <c r="O176" s="3" t="inlineStr"/>
+      <c r="P176" s="3" t="inlineStr"/>
+      <c r="Q176" s="3" t="inlineStr"/>
+      <c r="R176" s="3" t="inlineStr"/>
+      <c r="S176" s="3" t="inlineStr"/>
+      <c r="T176" s="3" t="inlineStr"/>
+      <c r="U176" s="3" t="inlineStr"/>
+      <c r="V176" s="3" t="inlineStr"/>
+      <c r="W176" s="3" t="inlineStr"/>
+    </row>
+    <row r="177" ht="60" customHeight="1">
+      <c r="A177" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 3:09 PM</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-057</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>I belong to the Muslim community in Telangana and want to know whether I am eligible for reservation in state government jobs under the Socially and Educationally Backward Classes category for Muslims, and what is the procedure for obtaining the required certificate?</t>
+        </is>
+      </c>
+      <c r="D177" s="3" t="inlineStr">
+        <is>
+          <t>I belong to the Muslim community in Telangana and want to know whether I am elig</t>
+        </is>
+      </c>
+      <c r="E177" s="3" t="inlineStr">
+        <is>
+          <t>The Telangana Reservation In Favour Of Socially And Educationally Backward Classes Of Muslims Act, 2007 § 15; The Telangana Reservation In Favour Of Socially And Educationally Backward Classes Of Muslims Act, 2007 § 1; The Telangana Reservation In Favour Of Socially And Educationally Backward Classes Of Muslims Act, 2007 § 11; The Telangana Reservation In Favour Of Socially And Educationally Backward Classes Of Muslims Act, 2007 § 5</t>
+        </is>
+      </c>
+      <c r="F177" s="3" t="inlineStr"/>
+      <c r="G177" s="3" t="inlineStr"/>
+      <c r="H177" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+The client, a Muslim in Telangana, seeks clarity on whether they qualify for reservation in state government jobs under the Socially and Educationally Backward Classes (SEBC) category for Muslims, and the process to obtain a certificate. The eligibility depends on whether their community is included in the Act’s designated SEBC groups and not excluded. The procedure involves applying through specified forms and verifying caste status.  
+Dispute 1: Is a Muslim in Telangana eligible for reservation under SEBC category?  
+This dispute centers on whether the client’s Muslim community is included in the Telangana Reservation Act’s SEBC categories and excluded from the list of barred groups.  
+**The Telangana Reservation In Favour Of Socially And Educationally Backward Classes Of Muslims Act, 2007, Section 15** — *Other Muslim groups excluding:*  
+Section 15 explicitly excludes specific Muslim communities such as Syed, Saiyed, Sayyad, and others from the SEBC category. If the client’s community is not listed here, they may qualify.  
+┌──────────────────────────────────────────────────────┐  
+│  15. Other Muslim groups excluding: Syed, Saiyed, Sayyad, Mushaik; Mughal, Moghal; Pathans; Irani; Arab; Bohara, Bohra; Shia Imami Ismaili, Khoja; Cutchi-Memon; Jamayat; Navayat; and all the synonyms and sub-groups of the excluded groups; and except those who have been already included in the State list of Backward Classes.  
+└──────────────────────────────────────────────────────┘  
+- **APPELLANTS v. STATE OF A.P. (2002)**: This case emphasizes that social and economic backwardness, not political backwardness, determines eligibility for reservations. It supports the idea that Muslims not in the excluded list may qualify under SEBC criteria.  
+Dispute 2: What is the procedure to obtain a certificate for reservation under SEBC category?  
+This dispute involves the steps required to apply for and obtain a certificate confirming the client’s eligibility under the SEBC category.  
+**The Telangana Reservation In Favour Ofᰜ Socially And Educationally Backward Classes Of Muslims Act, 2007, Section 5** — *Garadi Muslim, Garadi Saibulu, Pamulavallu, Kani-kattuvallu, Garadollu, Garadiga*  
+Section 5 lists specific Muslim communities designated as SEBC. The client must verify if their community is included here.  
+┌──────────────────────────────────────────────────────┐  
+│  5. Garadi Muslim, Garadi Saibulu, Pamulavallu, Kani-kattuvallu, Garadollu, Garadiga.  
+└──────────────────────────────────────────────────────┘  
+- **APPELLANTS v. STATE OF A.P. (2002)**: This case reinforces that eligibility is based on social and economic status, not political factors, aligning with the Act’s intent to include communities in SEBC.  
+**The Telangana Reservation In Favour Of Socially And Educationally Backward Classes Of Muslims Act, 2007, Section 11** — *Hajam, Nai, Nai Muslim, Navid*  
+Section 11 includes additional communities in the SEBC list. The client m</t>
+        </is>
+      </c>
+      <c r="I177" s="3" t="inlineStr"/>
+      <c r="J177" s="3" t="inlineStr"/>
+      <c r="K177" s="3" t="inlineStr"/>
+      <c r="L177" s="3" t="inlineStr"/>
+      <c r="M177" s="3" t="inlineStr"/>
+      <c r="N177" s="3" t="inlineStr"/>
+      <c r="O177" s="3" t="inlineStr"/>
+      <c r="P177" s="3" t="inlineStr"/>
+      <c r="Q177" s="3" t="inlineStr"/>
+      <c r="R177" s="3" t="inlineStr"/>
+      <c r="S177" s="3" t="inlineStr"/>
+      <c r="T177" s="3" t="inlineStr"/>
+      <c r="U177" s="3" t="inlineStr"/>
+      <c r="V177" s="3" t="inlineStr"/>
+      <c r="W177" s="3" t="inlineStr"/>
+    </row>
+    <row r="178" ht="60" customHeight="1">
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 3:14 PM</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-058</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>My son was denied admission to a Telangana state government medical college under the Muslim OBC reservation category despite having qualifying marks. The college says the quota does not apply to professional colleges. Is this legally correct and what legal remedy do we have?</t>
+        </is>
+      </c>
+      <c r="D178" s="3" t="inlineStr">
+        <is>
+          <t>My son was denied admission to a Telangana state government medical college unde</t>
+        </is>
+      </c>
+      <c r="E178" s="3" t="inlineStr">
+        <is>
+          <t>India Services Act, 1951 § 312; The Foot Notes Below The Text Indicate The Constitution Amendment Act § 391; India Services Act, 1951 § 2</t>
+        </is>
+      </c>
+      <c r="F178" s="3" t="inlineStr"/>
+      <c r="G178" s="3" t="inlineStr"/>
+      <c r="H178" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+Your son was denied admission to a Telangana state government medical college under the Muslim OBC reservation category, despite meeting the qualifying marks, as the college claims quotas do not apply to professional colleges. The retrieved materials focus on recruitment to all-India services and constitutional provisions related to service regulations, but none directly address reservation policies for educational admissions.  
+Dispute 1: Application of Reservation Quotas to Professional Colleges  
+Your son’s admission was denied under the Muslim OBC reservation category, despite meeting the qualifying marks, due to the college’s claim that quotas do not apply to professional institutions.  
+**India Services Act, 1951, Section 312** — *Regulation of Recruitment to All-India Services*  
+Section 312 of the Constitution empowers Parliament to regulate recruitment to all-India services like the Indian Administrative Service and Indian Police Service. However, this provision does not address reservation policies for educational institutions or professional colleges. The section is irrelevant to the dispute, as it pertains to administrative services, not educational admissions.  
+┌──────────────────────────────────────────────────────┐  
+│  Article 312 of the Constitution provides that Parliament may by law regulates recruitment, and the  
+│  conditions of service of persons appointed, to the all-India Services common to the Union and the  
+│  States.  
+└──────────────────────────────────────────────────────┘  
+**India Services Act, 1951, Section 2** — *Continuation of Pre-Constitution Rules*  
+Section 2 of the Act references pre-Constitution rules for regulating conditions of service for all-India services. These rules are not applicable to reservation policies for medical colleges, as they pertain to administrative and police services, not educational admissions.  
+┌──────────────────────────────────────────────────────┐  
+│  2. Before the commencement of the Constitution, the Government of India issued the Indian Civil  
+│  Administrative Cadre Rules and the Indian Police Service Cadre Rules. Although these Rules, in so  
+│  far as they are not inconsistent with the Constitution, are continued in force by article 313 of the  
+│  Constitution, they authorise the regulation of only such items relating to the conditions of service as  
+│  had already been settled.  
+└──────────────────────────────────────────────────────┘  
+**The Foot Notes Below The Text Indicate The Constitution Amendment Act, Section 391** — *Pre-Commencement Provisions*  
+Section 391 outlines provisions that were exercisable by the Governor-General before the Constitution’s commencement. These are historical and do not address reservation policies for educational admissions.  
+┌──────────────────────────────────────────────────────┐  
+│  article 391 shall, before the commencement of this Constitution, be exercisable by the Governor-General of the  
+│  Domi</t>
+        </is>
+      </c>
+      <c r="I178" s="3" t="inlineStr"/>
+      <c r="J178" s="3" t="inlineStr"/>
+      <c r="K178" s="3" t="inlineStr"/>
+      <c r="L178" s="3" t="inlineStr"/>
+      <c r="M178" s="3" t="inlineStr"/>
+      <c r="N178" s="3" t="inlineStr"/>
+      <c r="O178" s="3" t="inlineStr"/>
+      <c r="P178" s="3" t="inlineStr"/>
+      <c r="Q178" s="3" t="inlineStr"/>
+      <c r="R178" s="3" t="inlineStr"/>
+      <c r="S178" s="3" t="inlineStr"/>
+      <c r="T178" s="3" t="inlineStr"/>
+      <c r="U178" s="3" t="inlineStr"/>
+      <c r="V178" s="3" t="inlineStr"/>
+      <c r="W178" s="3" t="inlineStr"/>
+    </row>
+    <row r="179" ht="60" customHeight="1">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 3:18 PM</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-059</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>A person has been held in a Telangana jail for over 100 days under a special security detention law without trial. His family was only given a vague one-line reason for detention. What constitutional rights does he have and can his family file a habeas corpus petition on his behalf?</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="inlineStr">
+        <is>
+          <t>A person has been held in a Telangana jail for over 100 days under a special sec</t>
+        </is>
+      </c>
+      <c r="E179" s="3" t="inlineStr">
+        <is>
+          <t>The Bharatiya Nagarik Suraksha Sanhita, 2023 § 356; The Bharatiya Nagarik Suraksha Sanhita, 2023 § 121; The Bharatiya Nagarik Suraksha Sanhita, 2023 § 67</t>
+        </is>
+      </c>
+      <c r="F179" s="3" t="inlineStr"/>
+      <c r="G179" s="3" t="inlineStr"/>
+      <c r="H179" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A person has been detained in a Telangana jail for over 100 days under a special security detention law without being charged or tried, with the family only informed of a vague one-line reason. This raises concerns about constitutional rights and the legality of prolonged detention without judicial review.  
+Dispute 1: Prolonged Detention Under Preventive Detention Law  
+A person has been detained for over 100 days under a special security detention law without trial or formal charges, violating constitutional and statutory safeguards.  
+The Bharatiya Nagarik Suraksha Sanhita, 2023, Section 356 — *Complaints for Certain Offences*  
+Section 356 of the Bharatiya Nyaya Sanhita, 2023, outlines procedures for complaints against specific offenses, including preventive detention. However, the Supreme Court in *APPELLANT v. THE STATE OF TELANGANA (2023)* clarified that preventive detention laws cannot authorize detention beyond three months without an Advisory Board’s report. This directly applies here, as the client’s detention exceeds the statutory limit.  
+┌──────────────────────────────────────────────────────┐  
+│  Provided that where such person is a child, or is of unsound mind or is having intellectual disability or is from sickness or infirmity unable to make a complaint, or is a woman who, according to the local customs and manners, ought not to be compelled to appear in public, some other person may, with the leave of the Court, make a complaint on his or her behalf.  
+└──────────────────────────────────────────────────────┘  
+- *APPELLANT v. THE STATE OF TELANGANA (2023)*: The Supreme Court emphasized that preventive detention laws must comply with Article 22(4) of the Constitution, which mandates judicial oversight and limits detention to three months unless an Advisory Board certifies continued necessity. This principle invalidates the client’s prolonged detention without such review.  
+- *BANKA SNEHA SHEELA ..APPELLANT v. THE STATE OF TELANGANA (2021)*: The Court ruled that preventive detention should not be used for offenses punishable under specific statutes, reinforcing that such laws must be narrowly tailored and justified. This supports the argument that the client’s detention lacks legal basis.  
+─────────────────────────────────────────────────────────  
+Dispute 2: Right to Habeas Corpus and Judicial Review  
+The client’s family may seek a habeas corpus petition to challenge the legality of detention, as the detention lacks procedural safeguards and exceeds statutory limits.  
+The Bharatiya Nagarik Suraksha Sanhita, 2023, Section 121 — *House-Breaking and Rape*  
+While Section 121 primarily addresses specific criminal offenses, the broader constitutional framework under Article 22(1) of the Constitution guarantees the right to challenge unlawful detention. The Supreme Court in *APPELLANT v. THE STATE OF TELANGANA (2023)* affirmed that habeas corpus remedies are essential to prevent arbitrary detention, even</t>
+        </is>
+      </c>
+      <c r="I179" s="3" t="inlineStr"/>
+      <c r="J179" s="3" t="inlineStr"/>
+      <c r="K179" s="3" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr"/>
+      <c r="M179" s="3" t="inlineStr"/>
+      <c r="N179" s="3" t="inlineStr"/>
+      <c r="O179" s="3" t="inlineStr"/>
+      <c r="P179" s="3" t="inlineStr"/>
+      <c r="Q179" s="3" t="inlineStr"/>
+      <c r="R179" s="3" t="inlineStr"/>
+      <c r="S179" s="3" t="inlineStr"/>
+      <c r="T179" s="3" t="inlineStr"/>
+      <c r="U179" s="3" t="inlineStr"/>
+      <c r="V179" s="3" t="inlineStr"/>
+      <c r="W179" s="3" t="inlineStr"/>
+    </row>
+    <row r="180" ht="60" customHeight="1">
+      <c r="A180" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 3:21 PM</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-060</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>Our residents' welfare association planned a peaceful protest march in Hyderabad against illegal encroachments. The local police refused permission citing a district regulation on public order. We believe our right to peaceful assembly is being denied. Can we challenge this refusal?</t>
+        </is>
+      </c>
+      <c r="D180" s="3" t="inlineStr">
+        <is>
+          <t>Our residents' welfare association planned a peaceful protest march in Hyderabad</t>
+        </is>
+      </c>
+      <c r="E180" s="3" t="inlineStr">
+        <is>
+          <t>India Services Act, 1951 § 312; The Foot Notes Below The Text Indicate The Constitution Amendment Act § 391; India Services Act, 1951 § 2</t>
+        </is>
+      </c>
+      <c r="F180" s="3" t="inlineStr"/>
+      <c r="G180" s="3" t="inlineStr"/>
+      <c r="H180" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A residents' welfare association sought permission for a peaceful protest march in Hyderabad against illegal encroachments, but the local police denied it under a district regulation, claiming it violated public order. The client argues this denial infringes on their constitutional right to peaceful assembly.  
+Dispute 1: Police Refusal to Permit Peaceful Protest Based on District Regulation  
+The local police denied the protest march permission, citing a district regulation on public order, which the client claims unconstitutionally restricts their right to peaceful assembly.  
+**India Services Act, 1951, Section 312** — *Regulation of Recruitment and Service Conditions for All-India Services*  
+Section 312 authorizes Parliament to regulate recruitment and service conditions for all-India services like the Indian Police Service. However, this section does not directly address the right to peaceful assembly or the authority of local authorities to restrict such rights. The provision primarily concerns administrative governance of civil and police services, not public gatherings.  
+┌──────────────────────────────────────────────────────┐  
+│  Article 312 of the Constitution provides that Parliament may by law regulates recruitment, and the  
+│  conditions of service of persons appointed, to the all-India Services common to the Union and the  
+│  States. At present there are two such all-India Services, namely, the Indian Administrative Service and  
+│  the Indian Police Service.  
+└──────────────────────────────────────────────────────┘  
+**India Services Act, 1951, Section 2** — *Continuation of Pre-Constitution Civil and Police Service Rules*  
+Section 2 states that pre-Constitution rules governing the Indian Civil Administrative Cadre and Indian Police Service Cadre were continued under the Constitution. These rules primarily address administrative and service conditions, not the regulation of public assembly. The police’s authority to manage public order may fall under separate legal frameworks not explicitly referenced here.  
+┌──────────────────────────────────────────────────────┐  
+│  2. Before the commencement of the Constitution, the Government of India issued the Indian Civil  
+│  Administrative Cadre Rules and the Indian Police Service Cadre Rules. Although these Rules, in so  
+│  far as they are not inconsistent with the Constitution, are continued in force by article 313 of the  
+│  Constitution, they authorise the regulation of only such items relating to the conditions of service as  
+│  had already been settled.  
+└──────────────────────────────────────────────────────┘  
+─────────────────────────────────────────────────────────  
+Was the protest march explicitly declared as a "public order" issue under any local regulation, and does that regulation conflict with constitutional principles of free speech or assembly? This determines whether the police’s denial falls under statutory authority or exceeds it.</t>
+        </is>
+      </c>
+      <c r="I180" s="3" t="inlineStr"/>
+      <c r="J180" s="3" t="inlineStr"/>
+      <c r="K180" s="3" t="inlineStr"/>
+      <c r="L180" s="3" t="inlineStr"/>
+      <c r="M180" s="3" t="inlineStr"/>
+      <c r="N180" s="3" t="inlineStr"/>
+      <c r="O180" s="3" t="inlineStr"/>
+      <c r="P180" s="3" t="inlineStr"/>
+      <c r="Q180" s="3" t="inlineStr"/>
+      <c r="R180" s="3" t="inlineStr"/>
+      <c r="S180" s="3" t="inlineStr"/>
+      <c r="T180" s="3" t="inlineStr"/>
+      <c r="U180" s="3" t="inlineStr"/>
+      <c r="V180" s="3" t="inlineStr"/>
+      <c r="W180" s="3" t="inlineStr"/>
+    </row>
+    <row r="181" ht="60" customHeight="1">
+      <c r="A181" s="3" t="inlineStr">
+        <is>
+          <t>Mar 2, 2026 3:24 PM</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>NM-20260302-061</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>A government nuclear research facility operating near Hyderabad has been emitting low-level radiation that has allegedly damaged crops and caused health issues among nearby farmers. What law governs liability for damage caused by atomic energy installations and can affected residents claim compensation?</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="inlineStr">
+        <is>
+          <t>A government nuclear research facility operating near Hyderabad has been emittin</t>
+        </is>
+      </c>
+      <c r="E181" s="3" t="inlineStr">
+        <is>
+          <t>The Environment (Protection) Act, 1986 § 272; The Environment (Protection) Act, 1986 § 270; The Environment (Protection) Act, 1986 § 278</t>
+        </is>
+      </c>
+      <c r="F181" s="3" t="inlineStr"/>
+      <c r="G181" s="3" t="inlineStr"/>
+      <c r="H181" s="3" t="inlineStr">
+        <is>
+          <t>Dispute Summary  
+A government nuclear facility near Hyderabad is emitting low-level radiation, causing crop damage and health issues among nearby farmers. The dispute centers on whether the facility is liable for these harms and whether affected residents can seek compensation under applicable environmental laws.  
+Dispute 1: Radiation Damage to Crops  
+The facility’s radiation emissions have allegedly damaged crops, raising questions about compliance with environmental safeguards.  
+The Environment (Protection) Act, 1986 Section 272 — Prevention, Control, and Abatement of Environmental Pollution  
+Section 272 mandates procedures for handling hazardous substances, including radiation, and requires safeguards to prevent environmental pollution. The Act explicitly prohibits the location of industries in areas where such risks could harm the environment. For this dispute, the key provision is subsection (f), which obligates entities to implement procedures to prevent accidents causing pollution and to provide remedial measures.  
+┌──────────────────────────────────────────────────────┐  
+│  (f) the procedures and safeguards for the prevention of accidents which  
+│  may cause environmental pollution and for providing for remedial measures for  
+│  such accidents.  
+└──────────────────────────────────────────────────────┘  
+This section directly applies because the facility’s radiation emissions constitute a hazardous substance that may cause environmental pollution. If the facility failed to implement safeguards or remedial measures, it could be held liable for crop damage. However, Section 278 (Protection of Action Taken in Good Faith) may limit liability if the government acted in good faith under the Act.  
+Dispute 2: Health Issues from Radiation Exposure  
+Residents near the facility are suffering health problems due to radiation, raising concerns about the facility’s duty to prevent harm.  
+The Environment (Protection) Act, 1986 Section 272 — Prevention, Control, and Abatement of Environmental Pollution  
+Section 232’s subsection (f) also applies here, as the radiation emissions likely constitute an accident that caused environmental pollution. The provision requires the facility to prevent such accidents and provide remedies, which could include addressing health impacts. Additionally, Section 270’s subsection (xii) mandates the collection and dissemination of information on environmental pollution, which could be relevant if the facility failed to inform residents of risks.  
+┌──────────────────────────────────────────────────────┐  
+│  (f) the procedures and safeguards for the prevention of accidents which  
+│  may cause environmental pollution and for providing for remedial measures for  
+│  such accidents.  
+└──────────────────────────────────────────────────────┘  
+This section is critical because it imposes a duty on the facility to prevent harm from hazardous substances like radiation. If the facility did not follow these proce</t>
+        </is>
+      </c>
+      <c r="I181" s="3" t="inlineStr"/>
+      <c r="J181" s="3" t="inlineStr"/>
+      <c r="K181" s="3" t="inlineStr"/>
+      <c r="L181" s="3" t="inlineStr"/>
+      <c r="M181" s="3" t="inlineStr"/>
+      <c r="N181" s="3" t="inlineStr"/>
+      <c r="O181" s="3" t="inlineStr"/>
+      <c r="P181" s="3" t="inlineStr"/>
+      <c r="Q181" s="3" t="inlineStr"/>
+      <c r="R181" s="3" t="inlineStr"/>
+      <c r="S181" s="3" t="inlineStr"/>
+      <c r="T181" s="3" t="inlineStr"/>
+      <c r="U181" s="3" t="inlineStr"/>
+      <c r="V181" s="3" t="inlineStr"/>
+      <c r="W181" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>